<commit_message>
Add late-2025/early-2026 forecast notes for companies still without 2026 figures
Where a ruble number does not exist, the comment column now says so explicitly and records the industry or qualitative outlook (INFOLine, Data Insight, M&A talk) instead of a generic blank. Also fill Globus and Logika moloka H1 facts that were previously missing.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="6" min="1" max="1"/>
@@ -476,17 +476,29 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Пустых «примерно» без источника. Если открытой цифры нет — «н/д». Региональные сети и большинство молочных заводов так и стоят: они отчитаются в 2027-м.</t>
+          <t>Пустых «примерно» без источника. Если открытой цифры нет — «н/д». Региональные сети и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Отраслевой фон (топ-10 сетей +9–11%, пищепром около нуля, e-grocery 1,83 трлн) в персональную ячейку не ставили.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="64" customHeight="1" s="6">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>Были ли прогнозы в конце 2025 / начале 2026</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Свои рублёвые — почти ни у кого из «н/д». X5 ещё в марте держала +12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «проекты начнут окупаться», без суммы. У регионалов вместо прогноза кассы были новости про продажу сети. Глобальные PepsiCo/Nestlé — мировой organic, не Россия.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="64" customHeight="1" s="6">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>Формат файла</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Шрифт Times New Roman 11, шапка и столбец «Компания» — заливка #A2C4C9, как в вашей Google-таблице. Списки те же: сети и производители в том же порядке. Добавлен только этот лист и обновлён «Медиа».</t>
         </is>
@@ -950,7 +962,7 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Отдельной продуктовой выручки Ozon Fresh за 2026 нет. Data Insight: пятёрка e-grocery (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) во 2 кв. вместе 260 млрд ₽ и 214 млн заказов; у Ozon Fresh заказы +65%. Это оборот рынка доставки, не строка МСФО Ozon. https://abn.agency/2026/08/14/oborot-rossijskogo-egrocery-dostig-8942-mlrd-rublej-za-polugodie/</t>
+          <t>Своей продуктовой выручки Ozon Fresh на 2026 нет — ни факта, ни прогноза компании. Что было в начале года: Data Insight в январе 2026 ждал рынок e-grocery 1,8 трлн ₽ за год (+24% к 2025), к марту уточнил до 1,83 трлн (+22%), к маю 1,84 трлн. Это весь рынок доставки, не строка МСФО Ozon. Во 2 кв. пятёрка (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) вместе 260 млрд; у Ozon Fresh заказы +65%. https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
     </row>
@@ -992,7 +1004,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Выручку Лавки отдельно не публикуют. Блок e-com Яндекса (Лавка+Маркет+Еда+Деливери) 1П 247 млрд (+19%) — это не только продукты. Заказы Лавки во 2 кв. +5% (Data Insight). https://www.comnews.ru/content/246667/2026-07-31/2026-w31/1008/ozon-ustremilsya-lidery-sredi-marketpleysov</t>
+          <t>Выручку Лавки отдельно не публикуют и прогноза по ней не было. Блок e-com Яндекса (Лавка+Маркет+Еда+Деливери) 1П 247 млрд (+19%) — это не только продукты. Заказы Лавки во 2 кв. +5% (Data Insight). Рыночный ориентир того же агентства на 2026: весь e-grocery 1,83–1,84 трлн — не цифра Лавки. https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1042,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1" s="6">
+    <row r="15" ht="48" customHeight="1" s="6">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>ТС Победа / Гулливер / Народный амбар (ТК Лето)</t>
@@ -1068,11 +1080,11 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1" s="6">
+          <t>Своего рублёвого прогноза на 2026 не было. В начале 2026 «Гулливер» из того же контура писали как выставленный на продажу. Аналитик Совкомбанка: независимые сети с кассой &gt;100 млрд (Победа, Командор, Ярче, Аникс) в 2–3 года могут сменить собственника — это не цифра выручки. Последнее открытое: 176 млрд за 2025. https://www.kommersant.ru/doc/8364093</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" s="6">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Ярче! (Камелот-А, Томск)</t>
@@ -1110,11 +1122,11 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1" s="6">
+          <t>Прогноза выручки на 2026 нет. В обзорах конца 2025 / 2026 фигурирует как кандидат на M&amp;A, не как эмитент с guidance. Последнее открытое: 168 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" s="6">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Гиперглобус (Globus)</t>
@@ -1125,38 +1137,30 @@
           <t>гипер</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
+      <c r="C17" s="3" t="n">
+        <v>80.59999999999999</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
+          <t>1 пол.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="32" customHeight="1" s="6">
+          <t>INFOLine / «Коммерсантъ»: 1П 80,6 млрд без НДС (+2,7%). Сопоставимые продажи 1П +5,7%, корзина +7,5% (оценка, знакомая с аналитикой сети). Своего прогноза выручки на 2026 нет. План экспансии — гипер в 2027 (&gt;4 млрд капзатрат), не цифра кассы на этот год. Оценка года: 165,6 × 1,027. https://www.kommersant.ru/doc/9005166</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" s="6">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Верный (Союз Святого Иоанна Воина)</t>
@@ -1194,7 +1198,7 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Прогноза кассы на 2026 нет. Октябрь 2025: основатель ищет покупателя, оценка бизнеса 25–35 млрд ₽ (это цена сети, не выручка года). РСБУ 2025 вышел 1 апреля 2026: 154,4 млрд — прошлый год. https://www.kommersant.ru/doc/8158706</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1238,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1" s="6">
+    <row r="20" ht="48" customHeight="1" s="6">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Мария-Ра (Розница К-1)</t>
@@ -1265,18 +1269,16 @@
           <t>н/д</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
+      <c r="G20" s="3" t="n">
+        <v>1303</v>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1" s="6">
+          <t>Прогноза выручки на 2026 нет. Последнее: РСБУ 2025 = 127,5 млрд (+5%). На 1 июля 2026 — 1 303 магазина (штуки, не касса). Летом 2026 писали, что Лента смотрит покупку — сделка не подтверждена и цифры года не даёт. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" s="6">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Ермолино (оценка INFOLine, производство + своя розница)</t>
@@ -1314,11 +1316,11 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1" s="6">
+          <t>Своего прогноза на 2026 нет. INFOLine ставит оценку только по закрытому году. Последнее: ~111 млрд за 2025 (оценка, не МСФО).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1" s="6">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>ГК Командор (Командор, Аллея, Хороший)</t>
@@ -1356,7 +1358,7 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Прогноза выручки на 2026 нет. В списках возможных M&amp;A 2026–2028 (Совкомбанк) — без суммы кассы. Последнее открытое: ~100 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1434,7 @@
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1476,7 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1518,7 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1560,7 @@
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1600,11 +1602,11 @@
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1" s="6">
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1" s="6">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Аникс (ТС Аникс + Прайд-А)</t>
@@ -1642,7 +1644,7 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Прогноза на 2026 нет. Упоминается рядом с Победой / Ярче / Командором как возможный объект консолидации. Последнее: 31,3 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1686,7 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1728,7 @@
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1770,7 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1812,7 @@
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1854,7 @@
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1896,7 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1938,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1980,7 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2022,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2064,7 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2106,7 @@
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Региональные сети обычно публикуют РСБУ только весной следующего года.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1" s="6">
+    <row r="2" ht="48" customHeight="1" s="6">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>PepsiCo Россия (вкл. Вимм-Билль-Данн)</t>
@@ -2213,7 +2215,7 @@
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Российского прогноза в рублях нет (с 2022 глобальная PepsiCo не даёт локальный outlook). Глобально декабрь 2025 / весна 2026: органика +2–4% на 2026 — это мир, не «PepsiCo Россия». https://www.interfax.ru/business/1070847</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2255,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1" s="6">
+    <row r="4" ht="48" customHeight="1" s="6">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ЭФКО</t>
@@ -2291,7 +2293,7 @@
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Цифры на 2026 нет. План на 2025 был 440 млрд — не взяли (факт 344, 0%). Весной 2026 менеджмент: новые проекты начнут окупаться в 2026–2027, ждут рост выручки и прибыли — без суммы. https://abireg.ru/newsitem/113897/</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2337,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1" s="6">
+    <row r="6" ht="48" customHeight="1" s="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>KDV Group</t>
@@ -2373,7 +2375,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Прогноза на 2026 нет. INFOLine прямо ставит KDV в пример замедления: уже 2025 только +1%, в 2026 «динамика лидеров около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
     </row>
@@ -2409,11 +2411,11 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П: 141,6 млрд (+3,5%); скорр. EBITDA 27,2 (+38%). Оценка года: 288,7 × 1,035. https://www.interfax.ru/business/1111410</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="32" customHeight="1" s="6">
+          <t>МСФО 1П: 141,6 млрд (+3,5%). Свой рублёвый прогноз на год компания не давала — только «продолжим увеличивать выручку», капзатраты 2026 снова режут. Независимая оценка smart-lab: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" s="6">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ГАП Ресурс</t>
@@ -2451,11 +2453,11 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="32" customHeight="1" s="6">
+          <t>Рублёвого прогноза на 2026 нет. Июнь 2025 (ПМЭФ): трёхлетка капзатрат &gt;40 млрд, доп. объёмы птицы — в 2027. На 2025 обещали удержать выпуск ~1 070 тыс. т — факт 1 054. Это тонны, не касса 2026. https://www.agroinvestor.ru/investments/news/44400-gap-resurs-vlozhit-40-mlrd-rubley-v-rasshirenie-proizvodstva/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" s="6">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Nestlé Россия</t>
@@ -2493,11 +2495,11 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1" s="6">
+          <t>Выручки и прогноза по России на 2026 нет. Глобальный consensus аналитиков к Nestlé SA: органика ~3,5–3,7% на год — не российская цифра. https://www.nestle.com/sites/default/files/2026-10/nestle-sa-consensus-pre-Q32026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" s="6">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Mars Россия</t>
@@ -2535,11 +2537,11 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1" s="6">
+          <t>Локального прогноза выручки на 2026 не публиковали.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" s="6">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Продимекс (сумма предприятий группы)</t>
@@ -2577,11 +2579,11 @@
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1" s="6">
+          <t>Прогноза выручки на 2026 не было. Открытое — сумма заводов за 2025 (~220–224 млрд по разным периметрам). РСБУ за 2026 выйдет весной 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" s="6">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Агропромкомплектация</t>
@@ -2619,11 +2621,11 @@
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1" s="6">
+          <t>Сводного прогноза группы на 2026 нет. INFOLine за 2025: 204,4 млрд (+15%). Отдельные юрлица (АПК-Курск и др.) отчитываются по РСБУ раз в год.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" s="6">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Логика молока (ex-Danone / Health&amp;Nutrition)</t>
@@ -2634,38 +2636,30 @@
           <t>молочка / детское питание</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
+      <c r="C13" s="3" t="n">
+        <v>84.5</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>н/д</t>
-        </is>
+          <t>1 пол.</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>173</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>13</v>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1" s="6">
+          <t>Сама компания 16.07.2026: 84,5 млрд (+3,5%), молочка 510 тыс. т (+2,7%). Ориентир на год — не рубли, а «преодолеть 1 млн тонн готовой продукции». Инвестплан до 2030: 120 млрд. Оценка рублей на год: 167,1 × 1,035. https://logikamoloka.ru/press-centr/news/logika-moloka-podvodit-rezultaty-i-polugodiya-2026-goda/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" s="6">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Напитки вместе (ex-AB InBev Efes)</t>
@@ -2703,11 +2697,11 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1" s="6">
+          <t>Выручки 2026 нет. Стратегия без суммы: пиво &gt;30% рынка, безалкоголка &gt;8% портфеля в 1П, 700 млн в завод Саранск в 2026. https://napitkivmeste.ru/odin-god-pod-brendom-napitki-vmeste-bolee-30-novyh-produktov-i-rekordnye-vlozheniya-v-zavody/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" s="6">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Балтика (ООО ПК Балтика)</t>
@@ -2745,11 +2739,11 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1" s="6">
+          <t>Прогноза выручки на 2026 нет. По 2025 выпуск пива −16% — компания сама назвала это запланированной модернизацией. https://www.kommersant.ru/doc/8401281</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1" s="6">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Сибагро (совокупность компаний группы)</t>
@@ -2787,11 +2781,11 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1" s="6">
+          <t>Прогноза кассы на 2026 нет. После убытка 2025 (~4,2 млрд) холдинг сам сказал: масштабирование временно снимаем, фокус на рентабельности; точечно ~500 млн в Томскую птицефабрику. https://www.akm.ru/news/gruppa_kompaniy_sibagro_narastila_vyruchku_na_14_odnako_zakonchila_2025_god_s_chistym_ubytkom/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1" s="6">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Объединённые кондитеры (ООО, дистрибуция группы)</t>
@@ -2829,11 +2823,11 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="32" customHeight="1" s="6">
+          <t>Прогноза на 2026 нет. В конце 2025 ходили слухи о продаже холдинга — «Гута» опровергла. Последнее открытое: ~113 млрд за 2025. https://www.kommersant.ru/doc/8339681</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1" s="6">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>АБИ (ABI Product)</t>
@@ -2871,7 +2865,7 @@
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. Последнее: ~88 млрд за 2025 (INFOLine).</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2905,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1" s="6">
+    <row r="20" ht="48" customHeight="1" s="6">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Комос Групп (молочный контур рейтинга)</t>
@@ -2949,11 +2943,11 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1" s="6">
+          <t>Прогноза выручки на 2026 нет. INFOLine отмечает холдинг среди быстрорастущих молочников 2025, без цифры на этот год. Последнее: молочный контур 63,1 млрд за 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1" s="6">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Орими Трейд (Tess, Greenfield, Jardin)</t>
@@ -2991,7 +2985,7 @@
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Локального прогноза на 2026 не публиковали. Последнее: 62,3 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3027,7 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3069,7 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3109,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="32" customHeight="1" s="6">
+    <row r="25" ht="48" customHeight="1" s="6">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Прогресс (ФрутоНяня / Малышам)</t>
@@ -3153,11 +3147,11 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1" s="6">
+          <t>Прогноза на 2026 нет. Март 2026 — это отчёт за 2025: выручка 52,1 (+8%), прибыль 10,2. https://www.kommersant.ru/doc/8552221</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1" s="6">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>ГК Молвест</t>
@@ -3195,11 +3189,11 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1" s="6">
+          <t>Рублёвого прогноза выручки на 2026 нет. Июль 2026: инвестпрограмма ~13 млрд до 2028 (глубокая переработка, ингредиенты) — это капзатраты, не касса года. https://milknews.ru/index/molochnye-produkty/molvest-13-mlrd-investicii.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="48" customHeight="1" s="6">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Эссен Продакшн (Махеевъ)</t>
@@ -3237,7 +3231,7 @@
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Прогноза выручки на 2026 нет. Отраслевой фон кондитеров: дорогое какао и упаковка, без персональной цифры. Последнее: 50,2 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3273,7 @@
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3315,7 @@
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Выручку 2026 не публиковали. 1 кв.: продажи в натуральном выражении +7,5%, бренды «Сады Придонья» +11%, Nemoloko +19% (РБК Компании). https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
+          <t>Выручку 2026 не публиковали. 1 кв.: продажи в натуральном выражении +7,5%, бренды «Сады Придонья» +11%, Nemoloko +19% (РБК Компании). Рублёвого прогноза года нет. https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3357,7 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3405,7 +3399,7 @@
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3447,7 +3441,7 @@
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3483,7 @@
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3563,7 @@
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3605,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3647,7 @@
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3689,7 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3731,7 @@
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3773,7 @@
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3815,7 @@
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3857,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3899,7 @@
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3941,7 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3983,7 @@
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4025,7 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4067,7 @@
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4109,7 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4151,7 @@
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4193,7 @@
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4235,7 @@
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4283,7 +4277,7 @@
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4319,7 @@
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4367,7 +4361,7 @@
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4409,7 +4403,7 @@
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4451,7 +4445,7 @@
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4487,7 @@
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4529,7 @@
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4571,7 @@
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4613,7 @@
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4661,7 +4655,7 @@
       </c>
       <c r="H61" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4697,7 @@
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4745,7 +4739,7 @@
       </c>
       <c r="H63" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4787,7 +4781,7 @@
       </c>
       <c r="H64" s="11" t="inlineStr">
         <is>
-          <t>Открытой выручки / прогноза за 2026 не нашли. Большинство заводов рейтинга INFOLine отчитываются раз в год.</t>
+          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4796,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="6" min="1" max="1"/>
@@ -5083,212 +5077,110 @@
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
+    <row r="14" ht="72" customHeight="1" s="6">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Что было вместо цифры, если её нет</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>По большинству региональных сетей и заводов своего рублёвого прогноза на 2026 не было ни в конце 2025, ни в начале 2026. Что находилось: отраслевой фон (INFOLine: топ-10 сетей за год +9–11%; пищепром «около нуля»), рынок e-grocery 1,83–1,84 трлн (Data Insight, это не Ozon и не Лавка), и качественные фразы вроде «проекты начнут окупаться» у ЭФКО. В ячейку это не ставили — это не выручка компании.</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+        </is>
+      </c>
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
+    <row r="15" ht="72" customHeight="1" s="6">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>INFOLine — сети на весь 2026</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (в 1П десятка уже +11,6%, годом раньше было +17%). Это прогноз десятки, не Мария-Ра и не Командор.</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>https://www.kommersant.ru/doc/8923592</t>
+        </is>
+      </c>
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
+    <row r="16" ht="72" customHeight="1" s="6">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>INFOLine — заводы</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Светлана Силенина, сентябрь 2026: после эмбарго-2014 крупные производители росли на 11–16% в год, в 2025 среднее уже +0,4%, в 2026 динамика лидеров «приблизилась к нулю». KDV как пример: уже 2025 только +1%.</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+        </is>
+      </c>
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
+    <row r="17" ht="72" customHeight="1" s="6">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Data Insight — e-grocery, начало 2026</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>В январе агентство заложило рынок доставки продуктов на 1,8 трлн ₽ за 2026 (+24%). К марту 1,83 трлн (+22%), к маю 1,84 трлн. Это весь рынок с НДС и доставкой, не выручка одной Лавки или Ozon Fresh.</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>https://datainsight.ru/DI_eGrocery_april_2026</t>
+        </is>
+      </c>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="n"/>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
+    <row r="18" ht="72" customHeight="1" s="6">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Региональные сети — не прогноз кассы, а продажа</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Верный с октября 2025 ищут покупателя (оценка 25–35 млрд — цена бизнеса). Гулливер в начале 2026 писали как выставленный на продажу. Про Мария-Ра летом 2026 писали, что смотрит Лента. Цифры выручки на 2026 никто из них не давал.</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>https://www.kommersant.ru/doc/8158706</t>
+        </is>
+      </c>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="n"/>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="n"/>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="n"/>
-      <c r="B30" s="3" t="n"/>
-      <c r="C30" s="3" t="n"/>
-      <c r="D30" s="3" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="n"/>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="n"/>
-      <c r="B32" s="3" t="n"/>
-      <c r="C32" s="3" t="n"/>
-      <c r="D32" s="3" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="n"/>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="n"/>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="n"/>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="n"/>
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5304,6 +5196,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rewrite 2026 comments in plain Russian without industry abbreviations
Spell out periods, reports, and market notes so a reader outside retail can follow the same facts.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -440,7 +440,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Сегодня 19 октября 2026. Финансовый год закроется 31 декабря. Годовые МСФО/РСБУ компании обычно публикуют весной 2027. Поэтому в таблице два разных числа: уже вышедший кусок года и, где можно, оценка полного года.</t>
+          <t>Сегодня 19 октября 2026. Год закроется 31 декабря. Полные годовые отчёты компании обычно публикуют весной 2027. Поэтому в таблице два разных числа: уже вышедший кусок года и, где можно, оценка полного года.</t>
         </is>
       </c>
     </row>
@@ -452,7 +452,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Только опубликованная выручка за 9 месяцев, полугодие или (редко) квартал. X5 — единственная из крупных, у кого на октябрь уже есть 9 месяцев. Магнит, Лента, Fix Price, Русагро, Черкизово — полугодие. Светофор, Mercury, Самокат, Ашан, Metro — оценки INFOLine за полугодие, не их собственный МСФО.</t>
+          <t>Только опубликованная выручка за девять месяцев, полгода или (редко) квартал. X5 — единственная из крупных, у кого на октябрь уже есть девять месяцев. Магнит, Лента, Fix Price, Русагро, Черкизово — полгода. Светофор, Mercury, Самокат, Ашан, Metro — оценки агентства INFOLine за полгода, не их собственный отчёт.</t>
         </is>
       </c>
     </row>
@@ -464,7 +464,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Либо слова самой компании (X5: рост 12–16%; Мираторг: «несколько процентов»), либо простая арифметика: выручка-2025 × темп уже вышедшего куска 2026. Это не отчёт и не гарантия. У агро (Русагро) второе полугодие обычно сильнее первого — поэтому не умножали полугодие на два.</t>
+          <t>Либо слова самой компании (X5: рост 12–16%; Мираторг: «несколько процентов»), либо простая арифметика: выручка 2025, умноженная на рост уже вышедшего куска 2026. Это не отчёт и не гарантия. У «Русагро» осень обычно сильнее весны — поэтому полугодие на два не умножали.</t>
         </is>
       </c>
     </row>
@@ -476,7 +476,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Пустых «примерно» без источника. Если открытой цифры нет — «н/д». Региональные сети и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Отраслевой фон (топ-10 сетей +9–11%, пищепром около нуля, e-grocery 1,83 трлн) в персональную ячейку не ставили.</t>
+          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных» (в таблице «н/д»). Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей +9–11%, производители еды около нуля, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Свои рублёвые — почти ни у кого из «н/д». X5 ещё в марте держала +12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «проекты начнут окупаться», без суммы. У регионалов вместо прогноза кассы были новости про продажу сети. Глобальные PepsiCo/Nestlé — мировой organic, не Россия.</t>
+          <t>Свои в рублях — почти ни у кого из тех, у кого в таблице «нет данных». X5 ещё в марте держала +12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «новые заводы начнут себя окупать», без суммы. У сетей из регионов вместо прогноза продаж были новости про продажу самой сети. Мировые PepsiCo и Nestlé дают прогноз на весь мир, не на Россию.</t>
         </is>
       </c>
     </row>
@@ -546,17 +546,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Период факта</t>
+          <t>За какой кусок года</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>YoY факта, %</t>
+          <t>Рост к тому же куску 2025, %</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Оценка / прогноз года 2026, млрд ₽</t>
+          <t>Оценка / прогноз на весь 2026, млрд ₽</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Откуда цифра / как считали оценку</t>
+          <t>Откуда цифра, простыми словами</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>9 мес.</t>
+          <t>январь–сентябрь</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -602,7 +602,7 @@
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>ПАО, trading update 16.10.2026 (предварительные, без аудита). 9М выручка 3 791,5 млрд (+11,4%); 3 кв. 1 311 млрд (+13,0%). Пятёрочка 9М 2 918 (+9,4%), Перекрёсток 413 (+7,1%), Чижик 391 (+31,4%), X5 Digital 257 (+28,4%). Магазинов 30 981 на 30.09. Прогноз самой компании на год: рост 12–16% от 4 642 → 5 200–5 385. https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
+          <t>Сама компания 16 октября 2026, цифры ещё без проверки аудитора. За январь–сентябрь продали на 3 791,5 млрд рублей — на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь: 1 311 млрд (+13%). Пятёрочка за девять месяцев 2 918 (+9,4%), Перекрёсток 413 (+7,1%), Чижик 391 (+31,4%), доставка X5 — 257 (+28,4%). Магазинов 30 981 на конец сентября. Свой прогноз на весь год компания не снимала: рост 12–16%. От выручки 2025 (4 642) это 5 200–5 385. https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -636,7 +636,7 @@
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П, 28.08.2026: 1 887,2 млрд (+12,8%). Чистая розница 1 871. Магазинов 33 652. Чистый долг ~514,5; убыток по IFRS 16 ≈ −9,5. Оценка года: 3 509 × 1,128, если темп 1П удержится (это не отчёт за год). https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
+          <t>Официальный отчёт 28 августа 2026: за полгода продали на 1 887,2 млрд рублей (+12,8%). Из них магазины 1 871. Точек 33 652. Долги минус деньги на счетах ≈ 514,5 млрд. По прибыли группа всё ещё в минусе (около −9,5) — мешают проценты по кредитам. Оценка всего года, если второе полугодие будет как первое: 3 509 × 1,128. Это не отчёт за год. https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -667,12 +667,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ» 02.09.2026, топ-10 FMCG 1П: 878 млрд (+11,2%). Сводного МСФО холдинга нет. Оценка года: 1 660 × 1,112, если темп 1П удержится. https://www.kommersant.ru/doc/8923592</t>
+          <t>Агентство INFOLine в «Коммерсанте» 2 сентября 2026: за полгода 878 млрд (+11,2%). Своего сводного отчёта всей группы нет. Оценка года, если темп удержится: 1 660 × 1,112. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П: 648,5 млрд (+26,2%); 2 кв. 341,6 (+28,8%). Магазинов 7 456 на 30.06. Супер Лента +30,2%, Монетка +26,1%, гипер +12,9% (INFOLine). В августе закрыла покупку гипермаркетов «О’КЕЙ» — во 2П периметр шире. Оценка года без сделки: 1 104 × 1,262. Стратегия к 2028 — 2,2 трлн. https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
+          <t>Официальный отчёт: за полгода 648,5 млрд (+26,2%); апрель–июнь 341,6 (+28,8%). Магазинов 7 456 на 30 июня. Быстрее всех внутри группы — «Супер Лента» (+30,2%) и «Монетка» (+26,1%), большие магазины +12,9%. В августе купила большие магазины «О’КЕЙ» — с осени в цифрах будут ещё и чужие точки. Оценка года без этой покупки: 1 104 × 1,262. К 2028 сама Лента хочет 2,2 триллиона — это цель на потом, не на 2026. https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -737,12 +737,12 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ»: 189 млрд (−4,5%). Оценка года: 394 × 0,955. https://www.kommersant.ru/doc/8923592</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 189 млрд — на 4,5% меньше, чем годом раньше. Оценка года: 394 × 0,955. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
@@ -762,7 +762,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -773,12 +773,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ»: 191,06 млрд (+7,8%), обогнал Светофор в топ-5. Оценка года: 359 × 1,078. https://www.infoline.spb.ru/news/?news=308855</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 191,06 млрд (+7,8%). Обогнал «Светофор» среди пяти крупнейших. Оценка года: 359 × 1,078. https://www.infoline.spb.ru/news/?news=308855</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -812,7 +812,7 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П, 27.08.2026: 155,3 млрд (+4,8%); 2 кв. 82,2 (+6,9%). Розница 1П 138,2, опт 17,1. Магазинов 8 077. Оценка года: 313 × 1,048. https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
+          <t>Официальный отчёт 27 августа 2026: за полгода 155,3 млрд (+4,8%); апрель–июнь 82,2 (+6,9%). Магазины 138,2, опт 17,1. Точек 8 077. Оценка года: 313 × 1,048. https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -843,12 +843,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Оценка INFOLine / «Коммерсантъ»: 135 млрд (+15,5%). Оценка года: 279 × 1,155. https://www.kommersant.ru/doc/8923592</t>
+          <t>Оценка агентства INFOLine / «Коммерсантъ»: за полгода 135 млрд (+15,5%). Оценка года: 279 × 1,155. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -879,12 +879,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ»: 118,9 млрд (+0,5%). Оценка года: 260 × 1,005. https://www.kommersant.ru/doc/8923610</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 118,9 млрд (+0,5%). Оценка года: 260 × 1,005. https://www.kommersant.ru/doc/8923610</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -915,12 +915,12 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ»: 127 млрд (−2,5%). Оценка года: 250 × 0,975. https://www.kommersant.ru/doc/8923592</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 127 млрд — на 2,5% меньше, чем годом раньше. Оценка года: 250 × 0,975. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
@@ -937,32 +937,32 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Своей продуктовой выручки Ozon Fresh на 2026 нет — ни факта, ни прогноза компании. Что было в начале года: Data Insight в январе 2026 ждал рынок e-grocery 1,8 трлн ₽ за год (+24% к 2025), к марту уточнил до 1,83 трлн (+22%), к маю 1,84 трлн. Это весь рынок доставки, не строка МСФО Ozon. Во 2 кв. пятёрка (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) вместе 260 млрд; у Ozon Fresh заказы +65%. https://datainsight.ru/DI_eGrocery_april_2026</t>
+          <t>Сколько именно продуктов продал Ozon Fresh в 2026, компания не говорит — ни факта, ни своего прогноза. Что было в начале года: агентство Data Insight в январе ждало, что вся доставка продуктов в России за 2026 год будет около 1,8 триллиона рублей (+24% к 2025). К марту уточнили 1,83 триллиона (+22%), к маю 1,84. Это весь рынок доставки, не цифра Ozon. За апрель–июнь пять сервисов (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) вместе сделали 260 млрд; заказы Ozon Fresh +65%. https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
     </row>
@@ -979,32 +979,32 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Выручку Лавки отдельно не публикуют и прогноза по ней не было. Блок e-com Яндекса (Лавка+Маркет+Еда+Деливери) 1П 247 млрд (+19%) — это не только продукты. Заказы Лавки во 2 кв. +5% (Data Insight). Рыночный ориентир того же агентства на 2026: весь e-grocery 1,83–1,84 трлн — не цифра Лавки. https://datainsight.ru/DI_eGrocery_april_2026</t>
+          <t>Выручку Лавки отдельно не публикуют, своего прогноза по ней тоже не было. Весь интернет-блок Яндекса (Лавка + Маркет + Еда + Деливери) за полгода 247 млрд (+19%) — туда входят не только продукты. Заказов у Лавки за апрель–июнь +5%. Прогноз агентства Data Insight на 2026 — вся доставка продуктов в стране 1,83–1,84 триллиона. Это не цифра Лавки. https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>1 пол. «ДА!»</t>
+          <t>январь–июнь, только «ДА!»</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>После продажи гипер в конце 2025 у листинга O’KEY Group остался только «ДА!»: МСФО 1П 43,3 млрд (+10,4%), 236 магазинов. Оценка года контура «ДА!»: 80 × 1,104. Гипер ООО «О’КЕЙ» по РСБУ 1П 68,2 (−5,6%) — уже периметр Ленты, не складывать с «ДА!». https://okeygroup.lu/upload/IFRS%201H2026_RUS_final_.pdf</t>
+          <t>Большие магазины «О’КЕЙ» в конце 2025 продали. У оставшейся компании на бирже теперь только «ДА!»: за полгода 43,3 млрд (+10,4%), 236 магазинов. Оценка года именно «ДА!»: 80 × 1,104. Большие магазины ООО «О’КЕЙ» за полгода 68,2 (−5,6%) — это уже Лента, с «ДА!» не складывать. https://okeygroup.lu/upload/IFRS%201H2026_RUS_final_.pdf</t>
         </is>
       </c>
     </row>
@@ -1055,32 +1055,32 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не было. В начале 2026 «Гулливер» из того же контура писали как выставленный на продажу. Аналитик Совкомбанка: независимые сети с кассой &gt;100 млрд (Победа, Командор, Ярче, Аникс) в 2–3 года могут сменить собственника — это не цифра выручки. Последнее открытое: 176 млрд за 2025. https://www.kommersant.ru/doc/8364093</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не было. В начале 2026 про «Гулливер» из той же группы писали: сеть выставлена на продажу. Аналитик Совкомбанка: независимые сети, которые в 2025 продали больше чем на 100 млрд (Победа, Командор, Ярче, Аникс), в ближайшие 2–3 года могут сменить хозяина. Это не цифра выручки. Последнее открытое: 176 млрд за 2025. https://www.kommersant.ru/doc/8364093</t>
         </is>
       </c>
     </row>
@@ -1097,32 +1097,32 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. В обзорах конца 2025 / 2026 фигурирует как кандидат на M&amp;A, не как эмитент с guidance. Последнее открытое: 168 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+          <t>Прогноза выручки на 2026 нет. В обзорах конца 2025 и 2026 сеть называют как возможную покупку для крупного игрока — не как компанию со своим прогнозом. Последнее открытое: 168 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ»: 1П 80,6 млрд без НДС (+2,7%). Сопоставимые продажи 1П +5,7%, корзина +7,5% (оценка, знакомая с аналитикой сети). Своего прогноза выручки на 2026 нет. План экспансии — гипер в 2027 (&gt;4 млрд капзатрат), не цифра кассы на этот год. Оценка года: 165,6 × 1,027. https://www.kommersant.ru/doc/9005166</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 80,6 млрд без налога (+2,7%). В тех же магазинах, что были год назад, продажи +5,7%, средний чек +7,5%. Своего прогноза выручки на 2026 нет. Новый большой магазин планируют на 2027 (больше 4 млрд на стройку) — это не цифра продаж на этот год. Оценка года: 165,6 × 1,027. https://www.kommersant.ru/doc/9005166</t>
         </is>
       </c>
     </row>
@@ -1173,32 +1173,32 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Прогноза кассы на 2026 нет. Октябрь 2025: основатель ищет покупателя, оценка бизнеса 25–35 млрд ₽ (это цена сети, не выручка года). РСБУ 2025 вышел 1 апреля 2026: 154,4 млрд — прошлый год. https://www.kommersant.ru/doc/8158706</t>
+          <t>Прогноза выручки на 2026 нет. В октябре 2025 основатель искал покупателя: сеть оценивали в 25–35 млрд рублей. Это цена всего бизнеса, если его продадут, а не «сколько продадут за год». Российский отчёт за 2025 вышел 1 апреля 2026: 154,4 млрд — это прошлый год. https://www.kommersant.ru/doc/8158706</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>INFOLine / «Коммерсантъ»: «Спар Миддл Волга, Smart» 103,57 млрд (+7,8%) — периметр шире, чем строка 2025 (только SPAR МВ 136 за год). Оценка года грубая: 136 × 1,078. https://www.kommersant.ru/doc/8923592</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: «Спар Миддл Волга, Smart» за полгода 103,57 млрд (+7,8%). Тут шире, чем строка 2025 (тогда только SPAR Миддл Волга — 136 за год). Грубая оценка года: 136 × 1,078. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
@@ -1251,22 +1251,22 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G20" s="3" t="n">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. Последнее: РСБУ 2025 = 127,5 млрд (+5%). На 1 июля 2026 — 1 303 магазина (штуки, не касса). Летом 2026 писали, что Лента смотрит покупку — сделка не подтверждена и цифры года не даёт. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+          <t>Прогноза выручки на 2026 нет. Последнее: российский отчёт за 2025 — 127,5 млрд (+5%). На 1 июля 2026 — 1 303 магазина (это штуки, не деньги). Летом 2026 писали, что «Лента» смотрит покупку — сделка не подтверждена и цифры года не даёт. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1291,32 +1291,32 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Своего прогноза на 2026 нет. INFOLine ставит оценку только по закрытому году. Последнее: ~111 млрд за 2025 (оценка, не МСФО).</t>
+          <t>Своего прогноза на 2026 нет. Агентство INFOLine считает оценку только когда год уже закрыт. Последнее: около 111 млрд за 2025 (оценка агентства, не официальный отчёт компании).</t>
         </is>
       </c>
     </row>
@@ -1333,32 +1333,32 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. В списках возможных M&amp;A 2026–2028 (Совкомбанк) — без суммы кассы. Последнее открытое: ~100 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+          <t>Прогноза выручки на 2026 нет. В списках возможных покупок 2026–2028 (Совкомбанк) — без суммы продаж. Последнее открытое: около 100 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П, 24.08.2026: 51,2 млрд (+7,2%), EBITDA 4,5, прибыль 0,8, точек 2 225 на 30.06 (2 222 на 30.09). Оценка года с темпа 1П: 95,1 × 1,072. 9М «продажи с НДС +24%» — это не IFRS-выручка, в ячейку не ставили. https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
+          <t>Официальный отчёт 24 августа 2026: за полгода 51,2 млрд (+7,2%), прибыль 0,8, точек 2 225 на 30 июня (2 222 на 30 сентября). Оценка года, если темп полугодия удержится: 95,1 × 1,072. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это не та выручка, что в таблице. https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -1409,32 +1409,32 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1451,32 +1451,32 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1493,32 +1493,32 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1535,32 +1535,32 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1577,32 +1577,32 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1619,32 +1619,32 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. Упоминается рядом с Победой / Ярче / Командором как возможный объект консолидации. Последнее: 31,3 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+          <t>Прогноза на 2026 нет. Упоминается рядом с «Победой», «Ярче» и «Командором» как сеть, которую крупный игрок может купить. Последнее: 31,3 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1661,32 +1661,32 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1703,32 +1703,32 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1745,32 +1745,32 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1787,32 +1787,32 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1829,32 +1829,32 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1871,32 +1871,32 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1913,32 +1913,32 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1955,32 +1955,32 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1997,32 +1997,32 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2039,32 +2039,32 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2081,32 +2081,32 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. РСБУ за 2026 выйдет весной 2027. Отраслевой фон INFOLine (топ-10 сетей +9–11% за год) — не персональный прогноз этой сети.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2153,17 +2153,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Период факта</t>
+          <t>За какой кусок года</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>YoY факта, %</t>
+          <t>Рост к тому же куску 2025, %</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Оценка / прогноз года 2026, млрд ₽</t>
+          <t>Оценка / прогноз на весь 2026, млрд ₽</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Откуда цифра / как считали оценку</t>
+          <t>Откуда цифра, простыми словами</t>
         </is>
       </c>
     </row>
@@ -2190,32 +2190,32 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>Российского прогноза в рублях нет (с 2022 глобальная PepsiCo не даёт локальный outlook). Глобально декабрь 2025 / весна 2026: органика +2–4% на 2026 — это мир, не «PepsiCo Россия». https://www.interfax.ru/business/1070847</t>
+          <t>Прогноза именно по России в рублях нет: с 2022 мировая PepsiCo российские планы не публикует. В декабре 2025 и весной 2026 мировой прогноз: рост продаж на 2–4% — это весь мир, не «PepsiCo Россия». https://www.interfax.ru/business/1070847</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2235,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -2246,12 +2246,12 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П: 183,0 млрд (+9,1%). У агро 2П обычно больше 1П, поэтому не умножали на 2. Оценка года: 396,5 × 1,091, если темп удержится. https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
+          <t>Официальный отчёт: за полгода 183,0 млрд (+9,1%). У растениеводства и сахара осень обычно сильнее весны, поэтому полугодие на два не умножали. Оценка года, если темп удержится: 396,5 × 1,091. https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
         </is>
       </c>
     </row>
@@ -2268,32 +2268,32 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
         <is>
-          <t>Цифры на 2026 нет. План на 2025 был 440 млрд — не взяли (факт 344, 0%). Весной 2026 менеджмент: новые проекты начнут окупаться в 2026–2027, ждут рост выручки и прибыли — без суммы. https://abireg.ru/newsitem/113897/</t>
+          <t>Цифры на 2026 нет. На 2025 сами планировали 440 млрд — не получилось (факт 344, рост ноль). Весной 2026 руководство: новые заводы начнут себя окупать в 2026–2027, ждут рост продаж и прибыли — без конкретной суммы. https://abireg.ru/newsitem/113897/</t>
         </is>
       </c>
     </row>
@@ -2310,17 +2310,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F5" s="3" t="n">
@@ -2328,12 +2328,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Полной выручки 1П 2026 в открытом виде нет. Президент Линник (ПМЭФ, июнь): ожидает рост выручки «на несколько процентов»; экспорт удержать ~58 млрд как в 2025 (план +20% по экспорту снят из‑за крепкого рубля). Оценка года ≈ 342 × 1,03. Прибыль МСФО 6 мес. 19,61 млрд (+26%) — это не выручка. https://echomsk.spb.ru/nws/5317198-miratorg-ogidaet-neznachitelnyj-rost-vyruchki-po-itogam-2026-goda.html</t>
+          <t>Полной выручки за январь–июнь 2026 в открытом виде нет. Глава компании Виктор Линник в июне на Петербургском экономическом форуме: ждать рост продаж «на несколько процентов»; продажи за границу удержать около 58 млрд, как в 2025 (план +20% сняли — рубль слишком крепкий). Оценка года ≈ 342 × 1,03. Прибыль за полгода 19,61 млрд (+26%) — это не выручка. https://echomsk.spb.ru/nws/5317198-miratorg-ogidaet-neznachitelnyj-rost-vyruchki-po-itogam-2026-goda.html</t>
         </is>
       </c>
     </row>
@@ -2350,32 +2350,32 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. INFOLine прямо ставит KDV в пример замедления: уже 2025 только +1%, в 2026 «динамика лидеров около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+          <t>Прогноза на 2026 нет. Агентство INFOLine берёт KDV как пример торможения: уже 2025 только +1%, а в 2026 у крупных производителей еды рост «около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -2406,12 +2406,12 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>МСФО 1П: 141,6 млрд (+3,5%). Свой рублёвый прогноз на год компания не давала — только «продолжим увеличивать выручку», капзатраты 2026 снова режут. Независимая оценка smart-lab: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
+          <t>Официальный отчёт: за полгода 141,6 млрд (+3,5%). Свой прогноз в рублях на год компания не давала — только «продолжим увеличивать выручку», деньги на стройки в 2026 снова режут. Независимая оценка на сайте для инвесторов: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
         </is>
       </c>
     </row>
@@ -2428,32 +2428,32 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>Рублёвого прогноза на 2026 нет. Июнь 2025 (ПМЭФ): трёхлетка капзатрат &gt;40 млрд, доп. объёмы птицы — в 2027. На 2025 обещали удержать выпуск ~1 070 тыс. т — факт 1 054. Это тонны, не касса 2026. https://www.agroinvestor.ru/investments/news/44400-gap-resurs-vlozhit-40-mlrd-rubley-v-rasshirenie-proizvodstva/</t>
+          <t>Прогноза в рублях на 2026 нет. В июне 2025 на Петербургском экономическом форуме: за три года вложат больше 40 млрд в новые птичники, добавка по мясу — в 2027. На 2025 обещали удержать выпуск около 1 070 тысяч тонн — вышло 1 054. Это тонны, не деньги 2026. https://www.agroinvestor.ru/investments/news/44400-gap-resurs-vlozhit-40-mlrd-rubley-v-rasshirenie-proizvodstva/</t>
         </is>
       </c>
     </row>
@@ -2470,32 +2470,32 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Выручки и прогноза по России на 2026 нет. Глобальный consensus аналитиков к Nestlé SA: органика ~3,5–3,7% на год — не российская цифра. https://www.nestle.com/sites/default/files/2026-10/nestle-sa-consensus-pre-Q32026.pdf</t>
+          <t>Выручки и прогноза по России на 2026 нет. Оценка аналитиков по всей мировой Nestlé: рост продаж около 3,5–3,7% за год — не российская цифра. https://www.nestle.com/sites/default/files/2026-10/nestle-sa-consensus-pre-Q32026.pdf</t>
         </is>
       </c>
     </row>
@@ -2512,32 +2512,32 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Локального прогноза выручки на 2026 не публиковали.</t>
+          <t>Своего прогноза выручки по России на 2026 не публиковали.</t>
         </is>
       </c>
     </row>
@@ -2554,32 +2554,32 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 не было. Открытое — сумма заводов за 2025 (~220–224 млрд по разным периметрам). РСБУ за 2026 выйдет весной 2027.</t>
+          <t>Прогноза выручки на 2026 не было. Открытое — сумма заводов за 2025 (около 220–224 млрд, считают по-разному). Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -2596,32 +2596,32 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Сводного прогноза группы на 2026 нет. INFOLine за 2025: 204,4 млрд (+15%). Отдельные юрлица (АПК-Курск и др.) отчитываются по РСБУ раз в год.</t>
+          <t>Прогноза всей группы на 2026 нет. Агентство INFOLine за 2025: 204,4 млрд (+15%). Отдельные компании группы (АПК-Курск и другие) отчитываются раз в год.</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Сама компания 16.07.2026: 84,5 млрд (+3,5%), молочка 510 тыс. т (+2,7%). Ориентир на год — не рубли, а «преодолеть 1 млн тонн готовой продукции». Инвестплан до 2030: 120 млрд. Оценка рублей на год: 167,1 × 1,035. https://logikamoloka.ru/press-centr/news/logika-moloka-podvodit-rezultaty-i-polugodiya-2026-goda/</t>
+          <t>Сама компания 16 июля 2026: за полгода продали на 84,5 млрд (+3,5%), молочки 510 тысяч тонн (+2,7%). Ориентир на год — не деньги, а «сделать больше 1 миллиона тонн готовой продукции». На стройки и оборудование до 2030 заложили 120 млрд. Оценка рублей на год: 167,1 × 1,035. https://logikamoloka.ru/press-centr/news/logika-moloka-podvodit-rezultaty-i-polugodiya-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -2672,32 +2672,32 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>Выручки 2026 нет. Стратегия без суммы: пиво &gt;30% рынка, безалкоголка &gt;8% портфеля в 1П, 700 млн в завод Саранск в 2026. https://napitkivmeste.ru/odin-god-pod-brendom-napitki-vmeste-bolee-30-novyh-produktov-i-rekordnye-vlozheniya-v-zavody/</t>
+          <t>Выручки 2026 нет. План без суммы: пиво — больше 30% рынка, напитки без алкоголя — больше 8% продаж за первое полугодие, 700 миллионов в завод в Саранске в 2026. https://napitkivmeste.ru/odin-god-pod-brendom-napitki-vmeste-bolee-30-novyh-produktov-i-rekordnye-vlozheniya-v-zavody/</t>
         </is>
       </c>
     </row>
@@ -2714,32 +2714,32 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. По 2025 выпуск пива −16% — компания сама назвала это запланированной модернизацией. https://www.kommersant.ru/doc/8401281</t>
+          <t>Прогноза выручки на 2026 нет. В 2025 выпуск пива упал на 16% — компания сама сказала, что так и задумала: обновляли заводы. Это про прошлый год, не про 2026. https://www.kommersant.ru/doc/8401281</t>
         </is>
       </c>
     </row>
@@ -2756,32 +2756,32 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Прогноза кассы на 2026 нет. После убытка 2025 (~4,2 млрд) холдинг сам сказал: масштабирование временно снимаем, фокус на рентабельности; точечно ~500 млн в Томскую птицефабрику. https://www.akm.ru/news/gruppa_kompaniy_sibagro_narastila_vyruchku_na_14_odnako_zakonchila_2025_god_s_chistym_ubytkom/</t>
+          <t>Прогноза выручки на 2026 нет. После убытка 2025 (около 4,2 млрд) группа сама сказала: новые большие стройки пока не начинаем, сначала надо выйти в плюс; точечно около 500 миллионов в Томскую птицефабрику. https://www.akm.ru/news/gruppa_kompaniy_sibagro_narastila_vyruchku_na_14_odnako_zakonchila_2025_god_s_chistym_ubytkom/</t>
         </is>
       </c>
     </row>
@@ -2798,32 +2798,32 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. В конце 2025 ходили слухи о продаже холдинга — «Гута» опровергла. Последнее открытое: ~113 млрд за 2025. https://www.kommersant.ru/doc/8339681</t>
+          <t>Прогноза на 2026 нет. В конце 2025 ходили слухи, что группу продадут — владельцы («Гута») опровергли. Последнее открытое: около 113 млрд за 2025. https://www.kommersant.ru/doc/8339681</t>
         </is>
       </c>
     </row>
@@ -2840,32 +2840,32 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. Последнее: ~88 млрд за 2025 (INFOLine).</t>
+          <t>Своего прогноза выручки на 2026 не публиковали. Последнее: около 88 млрд за 2025 (агентство INFOLine).</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>Пресс-служба 07.09.2026: 46,3 млрд (+19%), EBITDA 10. Оценка года: 82,8 × 1,19. https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
+          <t>Пресс-служба 7 сентября 2026: за полгода 46,3 млрд (+19%). Оценка года: 82,8 × 1,19. https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
         </is>
       </c>
     </row>
@@ -2918,32 +2918,32 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. INFOLine отмечает холдинг среди быстрорастущих молочников 2025, без цифры на этот год. Последнее: молочный контур 63,1 млрд за 2025.</t>
+          <t>Прогноза выручки на 2026 нет. Агентство INFOLine отмечает группу среди быстрорастущих молочников 2025, без цифры на этот год. Последнее: только молочная часть 63,1 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -2960,32 +2960,32 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
         <is>
-          <t>Локального прогноза на 2026 не публиковали. Последнее: 62,3 млрд за 2025.</t>
+          <t>Своего прогноза по России на 2026 не публиковали. Последнее: 62,3 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -3002,32 +3002,32 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3044,32 +3044,32 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>1 пол.</t>
+          <t>январь–июнь</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
@@ -3100,12 +3100,12 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>МСФО 6 мес.: 24,63 млрд (−6,4% к 26,31). Прибыль 1,99 (−40%). Оценка года: 56,4 × 0,936. Объём свинины +10% при падении цены. https://www.tbank.ru/invest/social/profile/Marten_Resting/cbc77ff8-2a7f-49ae-8534-59a60c86da65/</t>
+          <t>Официальный отчёт за полгода: 24,63 млрд — на 6,4% меньше, чем 26,31 годом раньше. Прибыль 1,99 (−40%). Оценка года: 56,4 × 0,936. Свинины в тоннах сделали на 10% больше, но она подешевела. https://www.tbank.ru/invest/social/profile/Marten_Resting/cbc77ff8-2a7f-49ae-8534-59a60c86da65/</t>
         </is>
       </c>
     </row>
@@ -3122,32 +3122,32 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. Март 2026 — это отчёт за 2025: выручка 52,1 (+8%), прибыль 10,2. https://www.kommersant.ru/doc/8552221</t>
+          <t>Прогноза на 2026 нет. В марте 2026 вышел отчёт за 2025: выручка 52,1 (+8%), прибыль 10,2. https://www.kommersant.ru/doc/8552221</t>
         </is>
       </c>
     </row>
@@ -3164,32 +3164,32 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>Рублёвого прогноза выручки на 2026 нет. Июль 2026: инвестпрограмма ~13 млрд до 2028 (глубокая переработка, ингредиенты) — это капзатраты, не касса года. https://milknews.ru/index/molochnye-produkty/molvest-13-mlrd-investicii.html</t>
+          <t>Прогноза выручки на 2026 нет. Июль 2026: до 2028 вложат около 13 млрд в новые линии (белки из молока и другие ингредиенты) — это деньги на стройку, не «сколько продадут за год». https://milknews.ru/index/molochnye-produkty/molvest-13-mlrd-investicii.html</t>
         </is>
       </c>
     </row>
@@ -3206,32 +3206,32 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. Отраслевой фон кондитеров: дорогое какао и упаковка, без персональной цифры. Последнее: 50,2 млрд за 2025.</t>
+          <t>Прогноза выручки на 2026 нет. У кондитеров в целом дорогое какао и упаковка — без цифры именно этой компании. Последнее: 50,2 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -3248,32 +3248,32 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3290,32 +3290,32 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>1 кв., только тонны</t>
+          <t>январь–март, только тонны</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
         <is>
-          <t>Выручку 2026 не публиковали. 1 кв.: продажи в натуральном выражении +7,5%, бренды «Сады Придонья» +11%, Nemoloko +19% (РБК Компании). Рублёвого прогноза года нет. https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
+          <t>Выручку 2026 в деньгах не публиковали. За январь–март продали на 7,5% больше в тоннах, бренды «Сады Придонья» +11%, Nemoloko +19%. Прогноза в рублях на год нет. https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
         </is>
       </c>
     </row>
@@ -3332,32 +3332,32 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3374,32 +3374,32 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3416,32 +3416,32 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3458,32 +3458,32 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>1 пол. весь холдинг</t>
+          <t>январь–июнь, вся группа</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
@@ -3511,17 +3511,17 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>МСФО холдинга 1П 45,2 млрд (−2,8%), прибыль 1,1. Это ВЕСЬ холдинг, не молочный контур рейтинга INFOLine 2025 (29,8) — сравнивать с 29,8 нельзя. Оценку года для контура не ставили. https://abireg.ru/newsitem/116916/</t>
+          <t>Официальный отчёт всей группы за полгода: 45,2 млрд (−2,8%), прибыль 1,1. Это ВСЯ компания, а не только молочная часть, которую агентство INFOLine считало за 2025 (29,8). С 29,8 сравнивать нельзя. Оценку года только для молочки не ставили. https://abireg.ru/newsitem/116916/</t>
         </is>
       </c>
     </row>
@@ -3538,32 +3538,32 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3580,32 +3580,32 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3622,32 +3622,32 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3664,32 +3664,32 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3748,32 +3748,32 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3790,32 +3790,32 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H41" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3832,32 +3832,32 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3874,32 +3874,32 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H43" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3916,32 +3916,32 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3958,32 +3958,32 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H45" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4000,32 +4000,32 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4042,32 +4042,32 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H47" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4084,32 +4084,32 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4126,32 +4126,32 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H49" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4168,32 +4168,32 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4210,32 +4210,32 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H51" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4252,32 +4252,32 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4294,32 +4294,32 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H53" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4336,32 +4336,32 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4378,32 +4378,32 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H55" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4420,32 +4420,32 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4462,32 +4462,32 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H57" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4504,32 +4504,32 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4546,32 +4546,32 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H59" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4588,32 +4588,32 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4630,32 +4630,32 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H61" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4672,32 +4672,32 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H62" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4714,32 +4714,32 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H63" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4756,32 +4756,32 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>н/д</t>
+          <t>нет данных</t>
         </is>
       </c>
       <c r="H64" s="11" t="inlineStr">
         <is>
-          <t>Своего рублёвого прогноза на 2026 не публиковали. INFOLine (сентябрь 2026): у лидеров пищепрома динамика «около нуля» — это отрасль, не эта компания. РСБУ за 2026 — весной 2027.</t>
+          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="B2" s="13" t="inlineStr">
         <is>
-          <t>Года ещё нет (сейчас октябрь 2026), полного МСФО за 2026 ни у кого нет. В столбце «факт» — уже опубликованный кусок: 9 месяцев, полугодие или квартал. «Оценка года» — не отчёт, а арифметика: либо прогноз самой компании, либо выручка-2025 × темп уже вышедшего куска 2026. Где куска нет — «н/д», ничего не додумано.</t>
+          <t>Года ещё нет (сейчас октябрь 2026), полного отчёта за весь 2026 ни у кого нет. В столбце «факт» — уже опубликованный кусок: девять месяцев, полгода или квартал. «Оценка года» — не отчёт, а арифметика: либо прогноз самой компании, либо выручка 2025, умноженная на рост уже вышедшего куска 2026. Где куска нет — «нет данных», ничего не додумано.</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
@@ -4849,12 +4849,12 @@
     <row r="3" ht="72" customHeight="1" s="6">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>X5 — 9 месяцев</t>
+          <t>X5 — январь–сентябрь</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Касса за январь–сентябрь 3,79 трлн ₽, на 11,4% больше, чем за те же 9 месяцев 2025-го. Третий квартал быстрее полугодия: +13% до 1,31 трлн. Чижик по-прежнему самый быстрый внутри группы (+31% за 9 мес., +35% за квартал). Компания свой прогноз на весь год не снимала: +12–16%.</t>
+          <t>Продали за январь–сентябрь на 3,79 триллиона рублей, на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь быстрее полугодия: +13% до 1,31 триллиона. Чижик по-прежнему самый быстрый внутри группы (+31% за девять месяцев, +35% за квартал). Компания свой прогноз на весь год не снимала: +12–16%.</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -4870,12 +4870,12 @@
     <row r="4" ht="72" customHeight="1" s="6">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>X5 — ориентир на год</t>
+          <t>X5 — свой прогноз на год</t>
         </is>
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>В марте и снова в июне президент Екатерина Лобачева: прогноз роста выручки 12–16% на 2026 держим. От базы 4,642 трлн это примерно 5,20–5,39 трлн за полный год. 9 месяцев идут ближе к нижней границе.</t>
+          <t>В марте и снова в июне президент Екатерина Лобачева: прогноз роста выручки 12–16% на 2026 держим. От выручки 2025 (4,642 триллиона) это примерно 5,20–5,39 триллиона за полный год. Девять месяцев идут ближе к нижней границе.</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
@@ -4891,12 +4891,12 @@
     <row r="5" ht="72" customHeight="1" s="6">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Магнит — полугодие</t>
+          <t>Магнит — полгода</t>
         </is>
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1 887 млрд ₽ за полгода, +12,8%. Магазины работают, касса растёт, по прибыли группа всё ещё в минусе по IFRS 16. Это тот же сюжет, что в 2025: полка живая, проценты тяжёлые.</t>
+          <t>1 887 млрд рублей за полгода, +12,8%. Магазины работают, продажи растут, по прибыли группа всё ещё в минусе: мешают проценты по кредитам. Это тот же сюжет, что в 2025: полка живая, кредиты тяжёлые.</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -4912,12 +4912,12 @@
     <row r="6" ht="72" customHeight="1" s="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Топ-10 сетей, 1 пол. 2026</t>
+          <t>Десять крупнейших сетей, январь–июнь 2026</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>INFOLine сложил десятку: 6,76 трлн ₽, +11,6% (годом раньше десятка росла на 17%). Лента +26% — самый быстрый из крупных. Светофор и Ашан в минусе. На весь 2026 INFOLine ждёт рост крупнейших сетей примерно 9–11%.</t>
+          <t>Агентство INFOLine сложила десятку: 6,76 триллиона рублей, +11,6% (годом раньше десятка росла на 17%). Лента +26% — самый быстрый из крупных. Светофор и Ашан продали меньше, чем год назад. На весь 2026 агентство ждёт рост крупнейших сетей примерно 9–11%.</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -4933,12 +4933,12 @@
     <row r="7" ht="72" customHeight="1" s="6">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Лента — полугодие</t>
+          <t>Лента — полгода</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>648 млрд ₽ за полгода, +26%. Драйверы — Супер Лента и Монетка. В августе забрала гипер «О’КЕЙ» — второе полугодие будет уже с чужими магазинами в периметре.</t>
+          <t>648 млрд рублей за полгода, +26%. Тянут «Супер Лента» и «Монетка». В августе купила большие магазины «О’КЕЙ» — со второго полугодия в цифрах будут ещё и эти магазины.</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -4954,12 +4954,12 @@
     <row r="8" ht="72" customHeight="1" s="6">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Fix Price — полугодие</t>
+          <t>Fix Price — полгода</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>155 млрд ₽, +4,8%. Медленнее продуктовых федералов: фиксированная цена и смешанный ассортимент.</t>
+          <t>155 млрд рублей, +4,8%. Медленнее больших продуктовых сетей: цены фиксированные, в ассортименте не только еда.</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -4975,12 +4975,12 @@
     <row r="9" ht="72" customHeight="1" s="6">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Винлаб — полугодие</t>
+          <t>Винлаб — полгода</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>51 млрд ₽ по МСФО, +7%. Отдельно компания хвалится продажами с НДС за 9 месяцев (+24%) — это восстановление после кибератаки 2025-го, не путать с выручкой в таблице.</t>
+          <t>51 млрд рублей по официальному отчёту, +7%. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это отскок после кибератаки 2025-го, не путать с выручкой в таблице.</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -4996,12 +4996,12 @@
     <row r="10" ht="72" customHeight="1" s="6">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Русагро — полугодие</t>
+          <t>Русагро — полгода</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>183 млрд ₽, +9%. Догнать PepsiCo по году ещё рано: полного 2026 нет ни у кого из заводов.</t>
+          <t>183 млрд рублей, +9%. Догнать PepsiCo по году ещё рано: полного 2026 нет ни у кого из заводов.</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -5017,12 +5017,12 @@
     <row r="11" ht="72" customHeight="1" s="6">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Черкизово — полугодие</t>
+          <t>Черкизово — полгода</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>142 млрд ₽, всего +3,5%. Слабее инфляции: дешевле свинина и меньше экспорта в Китай.</t>
+          <t>142 млрд рублей, всего +3,5%. Слабее роста цен в магазинах: дешевле свинина и меньше продаж в Китай.</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -5038,12 +5038,12 @@
     <row r="12" ht="72" customHeight="1" s="6">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Дамате — полугодие</t>
+          <t>Дамате — полгода</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>46 млрд ₽, +19% — один из немногих заводов с двузначным ростом кассы.</t>
+          <t>46 млрд рублей, +19% — один из немногих заводов, у кого продажи выросли сильно.</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Выручку за 2026 пока не раскрыли. Глава холдинга в июне: ждать роста «на несколько процентов», экспорт удержать около 58 млрд ₽.</t>
+          <t>Выручку за 2026 пока не раскрыли. Глава группы в июне: ждать роста «на несколько процентов», продажи за границу удержать около 58 млрд рублей.</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>По большинству региональных сетей и заводов своего рублёвого прогноза на 2026 не было ни в конце 2025, ни в начале 2026. Что находилось: отраслевой фон (INFOLine: топ-10 сетей за год +9–11%; пищепром «около нуля»), рынок e-grocery 1,83–1,84 трлн (Data Insight, это не Ozon и не Лавка), и качественные фразы вроде «проекты начнут окупаться» у ЭФКО. В ячейку это не ставили — это не выручка компании.</t>
+          <t>По большинству сетей из регионов и заводов своего прогноза «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год +9–11%; крупные производители еды почти без роста), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку выручки это не ставили — это не продажи компании.</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
@@ -5101,12 +5101,12 @@
     <row r="15" ht="72" customHeight="1" s="6">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>INFOLine — сети на весь 2026</t>
+          <t>Агентство INFOLine — сети на весь 2026</t>
         </is>
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (в 1П десятка уже +11,6%, годом раньше было +17%). Это прогноз десятки, не Мария-Ра и не Командор.</t>
+          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (за январь–июнь десятка уже +11,6%, годом раньше было +17%). Это прогноз десятки, не «Мария-Ра» и не «Командор».</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
@@ -5122,12 +5122,12 @@
     <row r="16" ht="72" customHeight="1" s="6">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>INFOLine — заводы</t>
+          <t>Агентство INFOLine — заводы</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Светлана Силенина, сентябрь 2026: после эмбарго-2014 крупные производители росли на 11–16% в год, в 2025 среднее уже +0,4%, в 2026 динамика лидеров «приблизилась к нулю». KDV как пример: уже 2025 только +1%.</t>
+          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже +0,4%, в 2026 рост лидеров «приблизился к нулю». KDV как пример: уже 2025 только +1%.</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
@@ -5143,12 +5143,12 @@
     <row r="17" ht="72" customHeight="1" s="6">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Data Insight — e-grocery, начало 2026</t>
+          <t>Доставка продуктов, начало 2026</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>В январе агентство заложило рынок доставки продуктов на 1,8 трлн ₽ за 2026 (+24%). К марту 1,83 трлн (+22%), к маю 1,84 трлн. Это весь рынок с НДС и доставкой, не выручка одной Лавки или Ozon Fresh.</t>
+          <t>В январе агентство Data Insight заложило всю доставку продуктов в России на 1,8 триллиона рублей за 2026 (+24%). К марту 1,83 триллиона (+22%), к маю 1,84. Это весь рынок вместе с налогом и платой за доставку, не выручка одной Лавки или Ozon Fresh.</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
@@ -5164,12 +5164,12 @@
     <row r="18" ht="72" customHeight="1" s="6">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Региональные сети — не прогноз кассы, а продажа</t>
+          <t>Сети из регионов — не прогноз продаж, а продажа самой сети</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Верный с октября 2025 ищут покупателя (оценка 25–35 млрд — цена бизнеса). Гулливер в начале 2026 писали как выставленный на продажу. Про Мария-Ра летом 2026 писали, что смотрит Лента. Цифры выручки на 2026 никто из них не давал.</t>
+          <t>«Верный» с октября 2025 ищут покупателя (оценка 25–35 млрд — цена всего бизнеса). «Гулливер» в начале 2026 писали как выставленный на продажу. Про «Мария-Ра» летом 2026 писали, что смотрит «Лента». Цифры выручки на 2026 никто из них не давал.</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Add 2026 H1 profit and margin columns where official reports exist
Keep the source comments in the same plain Russian. Fill profit and margin only for six chains and four manufacturers that published both figures for the same period; leave the rest as нет данных.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -42,6 +42,11 @@
     </font>
     <font>
       <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
       <sz val="11"/>
     </font>
     <font>
@@ -54,11 +59,6 @@
       <name val="Times New Roman"/>
       <b val="1"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -86,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -106,24 +106,30 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -417,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="6" min="1" max="1"/>
@@ -471,36 +477,48 @@
     <row r="9" ht="64" customHeight="1" s="6">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>Чего в ячейках нет</t>
+          <t>Что в столбцах «прибыль» и «маржа»</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных» (в таблице «н/д»). Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей +9–11%, производители еды около нуля, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
+          <t>Прибыль — сколько денег осталось после всех расходов за тот же кусок года, что и в столбце «факт». Маржа — какая это доля от продаж: 2% значит две копейки прибыли с каждого рубля. Цифры есть только там, где компания сама опубликовала и прибыль, и продажи за один период: шесть сетей и четыре завода. Исключение — X5: продажи уже за девять месяцев, прибыль пока только за январь–июнь. У остальных в этих столбцах «нет данных».</t>
         </is>
       </c>
     </row>
     <row r="11" ht="64" customHeight="1" s="6">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Были ли прогнозы в конце 2025 / начале 2026</t>
+          <t>Чего в ячейках нет</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Свои в рублях — почти ни у кого из тех, у кого в таблице «нет данных». X5 ещё в марте держала +12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «новые заводы начнут себя окупать», без суммы. У сетей из регионов вместо прогноза продаж были новости про продажу самой сети. Мировые PepsiCo и Nestlé дают прогноз на весь мир, не на Россию.</t>
+          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных». Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей +9–11%, производители еды около нуля, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="64" customHeight="1" s="6">
       <c r="A13" s="9" t="inlineStr">
         <is>
+          <t>Были ли прогнозы в конце 2025 / начале 2026</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Свои в рублях — почти ни у кого из тех, у кого в таблице «нет данных». X5 ещё в марте держала +12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «новые заводы начнут себя окупать», без суммы. У сетей из регионов вместо прогноза продаж были новости про продажу самой сети. Мировые PepsiCo и Nestlé дают прогноз на весь мир, не на Россию.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="64" customHeight="1" s="6">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
           <t>Формат файла</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Шрифт Times New Roman 11, шапка и столбец «Компания» — заливка #A2C4C9, как в вашей Google-таблице. Списки те же: сети и производители в том же порядке. Добавлен только этот лист и обновлён «Медиа».</t>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Шрифт Times New Roman 11, шапка и столбец «Компания» — заливка #A2C4C9, как в вашей Google-таблице. Списки те же: сети и производители в том же порядке. К выручке добавлены прибыль и маржа, плюс этот лист и обновлённый «Медиа».</t>
         </is>
       </c>
     </row>
@@ -515,7 +533,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="23.25" customWidth="1" style="6" min="1" max="1"/>
@@ -525,52 +543,64 @@
     <col width="12" customWidth="1" style="6" min="5" max="5"/>
     <col width="18" customWidth="1" style="6" min="6" max="6"/>
     <col width="14" customWidth="1" style="6" min="7" max="7"/>
-    <col width="78" customWidth="1" style="6" min="8" max="8"/>
+    <col width="16" customWidth="1" style="6" min="8" max="8"/>
+    <col width="12" customWidth="1" style="6" min="9" max="9"/>
+    <col width="78" customWidth="1" style="6" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" s="6">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1" s="6">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Компания</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Тип / формат</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Выручка 2026 факт, млрд ₽</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>За какой кусок года</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Рост к тому же куску 2025, %</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Оценка / прогноз на весь 2026, млрд ₽</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Магазины / заводы, шт</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Прибыль за тот же кусок, млрд ₽</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Маржа, %</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Откуда цифра, простыми словами</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1" s="6">
+    <row r="2" ht="98" customHeight="1" s="6">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>X5 Group (Пятёрочка, Перекрёсток, Чижик)</t>
@@ -600,13 +630,19 @@
       <c r="G2" s="3" t="n">
         <v>30981</v>
       </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>Сама компания 16 октября 2026, цифры ещё без проверки аудитора. За январь–сентябрь продали на 3 791,5 млрд рублей — на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь: 1 311 млрд (+13%). Пятёрочка за девять месяцев 2 918 (+9,4%), Перекрёсток 413 (+7,1%), Чижик 391 (+31,4%), доставка X5 — 257 (+28,4%). Магазинов 30 981 на конец сентября. Свой прогноз на весь год компания не снимала: рост 12–16%. От выручки 2025 (4 642) это 5 200–5 385. https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="48" customHeight="1" s="6">
+      <c r="H2" s="3" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="I2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>Сама компания 16 октября 2026, цифры ещё без проверки аудитора. За январь–сентябрь продали на 3 791,5 млрд рублей — на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь: 1 311 млрд (+13%). Пятёрочка за девять месяцев 2 918 (+9,4%), Перекрёсток 413 (+7,1%), Чижик 391 (+31,4%), доставка X5 — 257 (+28,4%). Магазинов 30 981 на конец сентября. Прибыль в таблице — 25,7 млрд, но это не за девять месяцев, а только за январь–июнь. За девять месяцев прибыль ещё не вышла (ждут 29 октября). Маржа 1% — это 25,7 от продаж за те же январь–июнь (2 481 млрд). От 3 792 за девять месяцев считать нельзя: куски года разные. Свой прогноз на весь год компания не снимала: рост 12–16%. От выручки 2025 (4 642) это 5 200–5 385. https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="87" customHeight="1" s="6">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Магнит (вкл. Дикси, Самбери, Азбука вкуса)</t>
@@ -634,13 +670,19 @@
       <c r="G3" s="3" t="n">
         <v>33652</v>
       </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт 28 августа 2026: за полгода продали на 1 887,2 млрд рублей (+12,8%). Из них магазины 1 871. Точек 33 652. Долги минус деньги на счетах ≈ 514,5 млрд. По прибыли группа всё ещё в минусе (около −9,5) — мешают проценты по кредитам. Оценка всего года, если второе полугодие будет как первое: 3 509 × 1,128. Это не отчёт за год. https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1" s="6">
+      <c r="H3" s="3" t="n">
+        <v>-1.9</v>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт 28 августа 2026: за полгода продали на 1 887,2 млрд рублей (+12,8%). Из них магазины 1 871. Точек 33 652. Долги минус деньги на счетах ≈ 514,5 млрд. Прибыль за те же январь–июнь в ячейке −1,9 млрд: сеть пока в минусе, мешают проценты по кредитам. Есть второй счёт того же минуса — около −9,5: там аренду магазинов считают как долг. В ячейке стоит −1,9, без этого правила. Оценка всего года, если второе полугодие будет как первое: 3 509 × 1,128. Это не отчёт за год. https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="61" customHeight="1" s="6">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Mercury Retail (Красное &amp; Белое, Бристоль)</t>
@@ -670,13 +712,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine в «Коммерсанте» 2 сентября 2026: за полгода 878 млрд (+11,2%). Своего сводного отчёта всей группы нет. Оценка года, если темп удержится: 1 660 × 1,112. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1" s="6">
+    <row r="5" ht="88" customHeight="1" s="6">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Группа Лента (Гипер/Супер Лента, Монетка, Улыбка радуги, Реми)</t>
@@ -704,13 +756,19 @@
       <c r="G5" s="3" t="n">
         <v>7456</v>
       </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт: за полгода 648,5 млрд (+26,2%); апрель–июнь 341,6 (+28,8%). Магазинов 7 456 на 30 июня. Быстрее всех внутри группы — «Супер Лента» (+30,2%) и «Монетка» (+26,1%), большие магазины +12,9%. В августе купила большие магазины «О’КЕЙ» — с осени в цифрах будут ещё и чужие точки. Оценка года без этой покупки: 1 104 × 1,262. К 2028 сама Лента хочет 2,2 триллиона — это цель на потом, не на 2026. https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="48" customHeight="1" s="6">
+      <c r="H5" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт: за полгода 648,5 млрд (+26,2%); апрель–июнь 341,6 (+28,8%). Магазинов 7 456 на 30 июня. Быстрее всех внутри группы — «Супер Лента» (+30,2%) и «Монетка» (+26,1%), большие магазины +12,9%. Прибыль за те же полгода 13 млрд — примерно 2 копейки с каждого рубля продаж. В августе купила большие магазины «О’КЕЙ» — с осени в цифрах будут ещё и чужие точки. Оценка года без этой покупки: 1 104 × 1,262. К 2028 сама Лента хочет 2,2 триллиона — это цель на потом, не на 2026. https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="57" customHeight="1" s="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Светофор / Маяк (ГК Торгсервис)</t>
@@ -740,13 +798,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine / «Коммерсантъ»: за полгода 189 млрд — на 4,5% меньше, чем годом раньше. Оценка года: 394 × 0,955. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" s="6">
+    <row r="7" ht="59" customHeight="1" s="6">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>ВкусВилл</t>
@@ -776,13 +844,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine / «Коммерсантъ»: за полгода 191,06 млрд (+7,8%). Обогнал «Светофор» среди пяти крупнейших. Оценка года: 359 × 1,078. https://www.infoline.spb.ru/news/?news=308855</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" s="6">
+    <row r="8" ht="73" customHeight="1" s="6">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Fix Price</t>
@@ -810,13 +888,19 @@
       <c r="G8" s="3" t="n">
         <v>8077</v>
       </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт 27 августа 2026: за полгода 155,3 млрд (+4,8%); апрель–июнь 82,2 (+6,9%). Магазины 138,2, опт 17,1. Точек 8 077. Оценка года: 313 × 1,048. https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1" s="6">
+      <c r="H8" s="3" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт 27 августа 2026: за полгода 155,3 млрд (+4,8%); апрель–июнь 82,2 (+6,9%). Магазины 138,2, опт 17,1. Точек 8 077. Прибыль за те же полгода 2,7 млрд — это 1,8% от продаж (почти 2 копейки с рубля). Оценка года: 313 × 1,048. https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1" s="6">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Самокат</t>
@@ -846,13 +930,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>Оценка агентства INFOLine / «Коммерсантъ»: за полгода 135 млрд (+15,5%). Оценка года: 279 × 1,155. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1" s="6">
+    <row r="10" ht="56" customHeight="1" s="6">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>METRO Россия</t>
@@ -882,13 +976,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine / «Коммерсантъ»: за полгода 118,9 млрд (+0,5%). Оценка года: 260 × 1,005. https://www.kommersant.ru/doc/8923610</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1" s="6">
+    <row r="11" ht="57" customHeight="1" s="6">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>АШАН Ритейл Россия</t>
@@ -918,13 +1022,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine / «Коммерсантъ»: за полгода 127 млрд — на 2,5% меньше, чем годом раньше. Оценка года: 250 × 0,975. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1" s="6">
+    <row r="12" ht="80" customHeight="1" s="6">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Ozon + Ozon Fresh</t>
@@ -960,13 +1074,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
         <is>
           <t>Сколько именно продуктов продал Ozon Fresh в 2026, компания не говорит — ни факта, ни своего прогноза. Что было в начале года: агентство Data Insight в январе ждало, что вся доставка продуктов в России за 2026 год будет около 1,8 триллиона рублей (+24% к 2025). К марту уточнили 1,83 триллиона (+22%), к маю 1,84. Это весь рынок доставки, не цифра Ozon. За апрель–июнь пять сервисов (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) вместе сделали 260 млрд; заказы Ozon Fresh +65%. https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1" s="6">
+    <row r="13" ht="72" customHeight="1" s="6">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Яндекс Лавка</t>
@@ -1002,13 +1126,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
         <is>
           <t>Выручку Лавки отдельно не публикуют, своего прогноза по ней тоже не было. Весь интернет-блок Яндекса (Лавка + Маркет + Еда + Деливери) за полгода 247 млрд (+19%) — туда входят не только продукты. Заказов у Лавки за апрель–июнь +5%. Прогноз агентства Data Insight на 2026 — вся доставка продуктов в стране 1,83–1,84 триллиона. Это не цифра Лавки. https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1" s="6">
+    <row r="14" ht="72" customHeight="1" s="6">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>ГК О'КЕЙ / Да!</t>
@@ -1036,13 +1170,19 @@
       <c r="G14" s="3" t="n">
         <v>236</v>
       </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>Большие магазины «О’КЕЙ» в конце 2025 продали. У оставшейся компании на бирже теперь только «ДА!»: за полгода 43,3 млрд (+10,4%), 236 магазинов. Оценка года именно «ДА!»: 80 × 1,104. Большие магазины ООО «О’КЕЙ» за полгода 68,2 (−5,6%) — это уже Лента, с «ДА!» не складывать. https://okeygroup.lu/upload/IFRS%201H2026_RUS_final_.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="48" customHeight="1" s="6">
+      <c r="H14" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I14" s="12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Большие магазины «О’КЕЙ» в конце 2025 продали. У оставшейся компании на бирже теперь только «ДА!»: за полгода 43,3 млрд (+10,4%), 236 магазинов. Прибыль только «ДА!» за те же полгода 1,2 млрд — 2,8% от продаж. Оценка года именно «ДА!»: 80 × 1,104. Большие магазины ООО «О’КЕЙ» за полгода 68,2 (−5,6%) — это уже Лента, с «ДА!» не складывать. https://okeygroup.lu/upload/IFRS%201H2026_RUS_final_.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1" s="6">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>ТС Победа / Гулливер / Народный амбар (ТК Лето)</t>
@@ -1078,13 +1218,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не было. В начале 2026 про «Гулливер» из той же группы писали: сеть выставлена на продажу. Аналитик Совкомбанка: независимые сети, которые в 2025 продали больше чем на 100 млрд (Победа, Командор, Ярче, Аникс), в ближайшие 2–3 года могут сменить хозяина. Это не цифра выручки. Последнее открытое: 176 млрд за 2025. https://www.kommersant.ru/doc/8364093</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1" s="6">
+    <row r="16" ht="65" customHeight="1" s="6">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Ярче! (Камелот-А, Томск)</t>
@@ -1120,13 +1270,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. В обзорах конца 2025 и 2026 сеть называют как возможную покупку для крупного игрока — не как компанию со своим прогнозом. Последнее открытое: 168 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1" s="6">
+    <row r="17" ht="70" customHeight="1" s="6">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Гиперглобус (Globus)</t>
@@ -1154,13 +1314,23 @@
       <c r="G17" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="H17" s="11" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine / «Коммерсантъ»: за полгода 80,6 млрд без налога (+2,7%). В тех же магазинах, что были год назад, продажи +5,7%, средний чек +7,5%. Своего прогноза выручки на 2026 нет. Новый большой магазин планируют на 2027 (больше 4 млрд на стройку) — это не цифра продаж на этот год. Оценка года: 165,6 × 1,027. https://www.kommersant.ru/doc/9005166</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1" s="6">
+    <row r="18" ht="66" customHeight="1" s="6">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Верный (Союз Святого Иоанна Воина)</t>
@@ -1196,13 +1366,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. В октябре 2025 основатель искал покупателя: сеть оценивали в 25–35 млрд рублей. Это цена всего бизнеса, если его продадут, а не «сколько продадут за год». Российский отчёт за 2025 вышел 1 апреля 2026: 154,4 млрд — это прошлый год. https://www.kommersant.ru/doc/8158706</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1" s="6">
+    <row r="19" ht="62" customHeight="1" s="6">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>SPAR Миддл Волга (SPAR, EUROSPAR)</t>
@@ -1232,13 +1412,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>Агентство INFOLine / «Коммерсантъ»: «Спар Миддл Волга, Smart» за полгода 103,57 млрд (+7,8%). Тут шире, чем строка 2025 (тогда только SPAR Миддл Волга — 136 за год). Грубая оценка года: 136 × 1,078. https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1" s="6">
+    <row r="20" ht="68" customHeight="1" s="6">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Мария-Ра (Розница К-1)</t>
@@ -1272,13 +1462,23 @@
       <c r="G20" s="3" t="n">
         <v>1303</v>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. Последнее: российский отчёт за 2025 — 127,5 млрд (+5%). На 1 июля 2026 — 1 303 магазина (это штуки, не деньги). Летом 2026 писали, что «Лента» смотрит покупку — сделка не подтверждена и цифры года не даёт. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1" s="6">
+    <row r="21" ht="59" customHeight="1" s="6">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Ермолино (оценка INFOLine, производство + своя розница)</t>
@@ -1314,13 +1514,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза на 2026 нет. Агентство INFOLine считает оценку только когда год уже закрыт. Последнее: около 111 млрд за 2025 (оценка агентства, не официальный отчёт компании).</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1" s="6">
+    <row r="22" ht="62" customHeight="1" s="6">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>ГК Командор (Командор, Аллея, Хороший)</t>
@@ -1356,13 +1566,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. В списках возможных покупок 2026–2028 (Совкомбанк) — без суммы продаж. Последнее открытое: около 100 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1" s="6">
+    <row r="23" ht="78" customHeight="1" s="6">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Винлаб (ПАО ВинЛаб / Novabev)</t>
@@ -1390,9 +1610,15 @@
       <c r="G23" s="3" t="n">
         <v>2222</v>
       </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт 24 августа 2026: за полгода 51,2 млрд (+7,2%), прибыль 0,8, точек 2 225 на 30 июня (2 222 на 30 сентября). Оценка года, если темп полугодия удержится: 95,1 × 1,072. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это не та выручка, что в таблице. https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
+      <c r="H23" s="3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт 24 августа 2026: за полгода 51,2 млрд (+7,2%), прибыль 0,79 млрд (1,5% от продаж — полторы копейки с рубля), точек 2 225 на 30 июня (2 222 на 30 сентября). Оценка года, если темп полугодия удержится: 95,1 × 1,072. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это не та выручка, что в таблице. https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1658,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H24" s="11" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1474,7 +1710,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1516,7 +1762,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1558,7 +1814,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1600,13 +1866,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="48" customHeight="1" s="6">
+    <row r="29" ht="63" customHeight="1" s="6">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Аникс (ТС Аникс + Прайд-А)</t>
@@ -1642,7 +1918,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
         <is>
           <t>Прогноза на 2026 нет. Упоминается рядом с «Победой», «Ярче» и «Командором» как сеть, которую крупный игрок может купить. Последнее: 31,3 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
@@ -1684,7 +1970,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1726,7 +2022,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1768,7 +2074,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1810,7 +2126,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1852,7 +2178,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H34" s="11" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I34" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J34" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1894,7 +2230,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1936,7 +2282,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -1978,7 +2334,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -2020,7 +2386,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H38" s="11" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -2062,7 +2438,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H39" s="11" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J39" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -2104,7 +2490,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H40" s="11" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
         </is>
@@ -2122,7 +2518,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="17.75" customWidth="1" style="6" min="1" max="1"/>
@@ -2132,52 +2528,64 @@
     <col width="12" customWidth="1" style="6" min="5" max="5"/>
     <col width="18" customWidth="1" style="6" min="6" max="6"/>
     <col width="14" customWidth="1" style="6" min="7" max="7"/>
-    <col width="78" customWidth="1" style="6" min="8" max="8"/>
+    <col width="16" customWidth="1" style="6" min="8" max="8"/>
+    <col width="12" customWidth="1" style="6" min="9" max="9"/>
+    <col width="78" customWidth="1" style="6" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" s="6">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1" s="6">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Компания</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Тип / формат</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Выручка 2026 факт, млрд ₽</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>За какой кусок года</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Рост к тому же куску 2025, %</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Оценка / прогноз на весь 2026, млрд ₽</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Магазины / заводы, шт</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Прибыль за тот же кусок, млрд ₽</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Маржа, %</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Откуда цифра, простыми словами</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1" s="6">
+    <row r="2" ht="62" customHeight="1" s="6">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>PepsiCo Россия (вкл. Вимм-Билль-Данн)</t>
@@ -2213,13 +2621,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
         <is>
           <t>Прогноза именно по России в рублях нет: с 2022 мировая PepsiCo российские планы не публикует. В декабре 2025 и весной 2026 мировой прогноз: рост продаж на 2–4% — это весь мир, не «PepsiCo Россия». https://www.interfax.ru/business/1070847</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1" s="6">
+    <row r="3" ht="72" customHeight="1" s="6">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Русагро</t>
@@ -2249,13 +2667,19 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт: за полгода 183,0 млрд (+9,1%). У растениеводства и сахара осень обычно сильнее весны, поэтому полугодие на два не умножали. Оценка года, если темп удержится: 396,5 × 1,091. https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="48" customHeight="1" s="6">
+      <c r="H3" s="3" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт: за полгода 183,0 млрд (+9,1%). Прибыль почти ноль: 56 миллионов рублей, это 0,056 млрд — меньше одной десятой копейки с рубля продаж. У растениеводства и сахара осень обычно сильнее весны, поэтому полугодие на два не умножали. Оценка года, если темп удержится: 396,5 × 1,091. https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="63" customHeight="1" s="6">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ЭФКО</t>
@@ -2291,13 +2715,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>Цифры на 2026 нет. На 2025 сами планировали 440 млрд — не получилось (факт 344, рост ноль). Весной 2026 руководство: новые заводы начнут себя окупать в 2026–2027, ждут рост продаж и прибыли — без конкретной суммы. https://abireg.ru/newsitem/113897/</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1" s="6">
+    <row r="5" ht="76" customHeight="1" s="6">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>АПХ Мираторг</t>
@@ -2331,13 +2765,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Полной выручки за январь–июнь 2026 в открытом виде нет. Глава компании Виктор Линник в июне на Петербургском экономическом форуме: ждать рост продаж «на несколько процентов»; продажи за границу удержать около 58 млрд, как в 2025 (план +20% сняли — рубль слишком крепкий). Оценка года ≈ 342 × 1,03. Прибыль за полгода 19,61 млрд (+26%) — это не выручка. https://echomsk.spb.ru/nws/5317198-miratorg-ogidaet-neznachitelnyj-rost-vyruchki-po-itogam-2026-goda.html</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1" s="6">
+    <row r="6" ht="65" customHeight="1" s="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>KDV Group</t>
@@ -2373,13 +2817,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
         <is>
           <t>Прогноза на 2026 нет. Агентство INFOLine берёт KDV как пример торможения: уже 2025 только +1%, а в 2026 у крупных производителей еды рост «около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" s="6">
+    <row r="7" ht="77" customHeight="1" s="6">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Черкизово</t>
@@ -2409,13 +2863,19 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт: за полгода 141,6 млрд (+3,5%). Свой прогноз в рублях на год компания не давала — только «продолжим увеличивать выручку», деньги на стройки в 2026 снова режут. Независимая оценка на сайте для инвесторов: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1" s="6">
+      <c r="H7" s="3" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт: за полгода 141,6 млрд (+3,5%). Прибыль за те же полгода 14,1 млрд — почти 10 копеек с каждого рубля продаж. Свой прогноз в рублях на год компания не давала — только «продолжим увеличивать выручку», деньги на стройки в 2026 снова режут. Независимая оценка на сайте для инвесторов: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="71" customHeight="1" s="6">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ГАП Ресурс</t>
@@ -2451,13 +2911,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
         <is>
           <t>Прогноза в рублях на 2026 нет. В июне 2025 на Петербургском экономическом форуме: за три года вложат больше 40 млрд в новые птичники, добавка по мясу — в 2027. На 2025 обещали удержать выпуск около 1 070 тысяч тонн — вышло 1 054. Это тонны, не деньги 2026. https://www.agroinvestor.ru/investments/news/44400-gap-resurs-vlozhit-40-mlrd-rubley-v-rasshirenie-proizvodstva/</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1" s="6">
+    <row r="9" ht="62" customHeight="1" s="6">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Nestlé Россия</t>
@@ -2493,13 +2963,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>Выручки и прогноза по России на 2026 нет. Оценка аналитиков по всей мировой Nestlé: рост продаж около 3,5–3,7% за год — не российская цифра. https://www.nestle.com/sites/default/files/2026-10/nestle-sa-consensus-pre-Q32026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1" s="6">
+    <row r="10" ht="51" customHeight="1" s="6">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Mars Россия</t>
@@ -2535,13 +3015,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза выручки по России на 2026 не публиковали.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1" s="6">
+    <row r="11" ht="57" customHeight="1" s="6">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Продимекс (сумма предприятий группы)</t>
@@ -2577,13 +3067,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 не было. Открытое — сумма заводов за 2025 (около 220–224 млрд, считают по-разному). Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1" s="6">
+    <row r="12" ht="57" customHeight="1" s="6">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Агропромкомплектация</t>
@@ -2619,13 +3119,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
         <is>
           <t>Прогноза всей группы на 2026 нет. Агентство INFOLine за 2025: 204,4 млрд (+15%). Отдельные компании группы (АПК-Курск и другие) отчитываются раз в год.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1" s="6">
+    <row r="13" ht="71" customHeight="1" s="6">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Логика молока (ex-Danone / Health&amp;Nutrition)</t>
@@ -2653,13 +3163,23 @@
       <c r="G13" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="H13" s="11" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
         <is>
           <t>Сама компания 16 июля 2026: за полгода продали на 84,5 млрд (+3,5%), молочки 510 тысяч тонн (+2,7%). Ориентир на год — не деньги, а «сделать больше 1 миллиона тонн готовой продукции». На стройки и оборудование до 2030 заложили 120 млрд. Оценка рублей на год: 167,1 × 1,035. https://logikamoloka.ru/press-centr/news/logika-moloka-podvodit-rezultaty-i-polugodiya-2026-goda/</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1" s="6">
+    <row r="14" ht="65" customHeight="1" s="6">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Напитки вместе (ex-AB InBev Efes)</t>
@@ -2695,13 +3215,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H14" s="11" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
         <is>
           <t>Выручки 2026 нет. План без суммы: пиво — больше 30% рынка, напитки без алкоголя — больше 8% продаж за первое полугодие, 700 миллионов в завод в Саранске в 2026. https://napitkivmeste.ru/odin-god-pod-brendom-napitki-vmeste-bolee-30-novyh-produktov-i-rekordnye-vlozheniya-v-zavody/</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1" s="6">
+    <row r="15" ht="60" customHeight="1" s="6">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Балтика (ООО ПК Балтика)</t>
@@ -2737,13 +3267,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H15" s="11" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. В 2025 выпуск пива упал на 16% — компания сама сказала, что так и задумала: обновляли заводы. Это про прошлый год, не про 2026. https://www.kommersant.ru/doc/8401281</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1" s="6">
+    <row r="16" ht="68" customHeight="1" s="6">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Сибагро (совокупность компаний группы)</t>
@@ -2779,13 +3319,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. После убытка 2025 (около 4,2 млрд) группа сама сказала: новые большие стройки пока не начинаем, сначала надо выйти в плюс; точечно около 500 миллионов в Томскую птицефабрику. https://www.akm.ru/news/gruppa_kompaniy_sibagro_narastila_vyruchku_na_14_odnako_zakonchila_2025_god_s_chistym_ubytkom/</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1" s="6">
+    <row r="17" ht="59" customHeight="1" s="6">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Объединённые кондитеры (ООО, дистрибуция группы)</t>
@@ -2821,13 +3371,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H17" s="11" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>Прогноза на 2026 нет. В конце 2025 ходили слухи, что группу продадут — владельцы («Гута») опровергли. Последнее открытое: около 113 млрд за 2025. https://www.kommersant.ru/doc/8339681</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1" s="6">
+    <row r="18" ht="54" customHeight="1" s="6">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>АБИ (ABI Product)</t>
@@ -2863,13 +3423,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза выручки на 2026 не публиковали. Последнее: около 88 млрд за 2025 (агентство INFOLine).</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1" s="6">
+    <row r="19" ht="61" customHeight="1" s="6">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Дамате</t>
@@ -2899,13 +3469,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H19" s="11" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>Пресс-служба 7 сентября 2026: за полгода 46,3 млрд (+19%). Оценка года: 82,8 × 1,19. https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1" s="6">
+    <row r="20" ht="59" customHeight="1" s="6">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Комос Групп (молочный контур рейтинга)</t>
@@ -2941,13 +3521,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. Агентство INFOLine отмечает группу среди быстрорастущих молочников 2025, без цифры на этот год. Последнее: только молочная часть 63,1 млрд за 2025.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1" s="6">
+    <row r="21" ht="52" customHeight="1" s="6">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Орими Трейд (Tess, Greenfield, Jardin)</t>
@@ -2983,7 +3573,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза по России на 2026 не публиковали. Последнее: 62,3 млрд за 2025.</t>
         </is>
@@ -3025,7 +3625,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3067,13 +3677,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1" s="6">
+    <row r="24" ht="68" customHeight="1" s="6">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Агроэко</t>
@@ -3103,13 +3723,19 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт за полгода: 24,63 млрд — на 6,4% меньше, чем 26,31 годом раньше. Прибыль 1,99 (−40%). Оценка года: 56,4 × 0,936. Свинины в тоннах сделали на 10% больше, но она подешевела. https://www.tbank.ru/invest/social/profile/Marten_Resting/cbc77ff8-2a7f-49ae-8534-59a60c86da65/</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1" s="6">
+      <c r="H24" s="3" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт за полгода: 24,63 млрд — на 6,4% меньше, чем 26,31 годом раньше. Прибыль 1,99 млрд (−40% к прошлому году) — это 8,1% от продаж. Оценка года: 56,4 × 0,936. Свинины в тоннах сделали на 10% больше, но она подешевела. https://www.tbank.ru/invest/social/profile/Marten_Resting/cbc77ff8-2a7f-49ae-8534-59a60c86da65/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="55" customHeight="1" s="6">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Прогресс (ФрутоНяня / Малышам)</t>
@@ -3145,13 +3771,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
         <is>
           <t>Прогноза на 2026 нет. В марте 2026 вышел отчёт за 2025: выручка 52,1 (+8%), прибыль 10,2. https://www.kommersant.ru/doc/8552221</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="48" customHeight="1" s="6">
+    <row r="26" ht="63" customHeight="1" s="6">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>ГК Молвест</t>
@@ -3187,13 +3823,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. Июль 2026: до 2028 вложат около 13 млрд в новые линии (белки из молока и другие ингредиенты) — это деньги на стройку, не «сколько продадут за год». https://milknews.ru/index/molochnye-produkty/molvest-13-mlrd-investicii.html</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="48" customHeight="1" s="6">
+    <row r="27" ht="56" customHeight="1" s="6">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Эссен Продакшн (Махеевъ)</t>
@@ -3229,7 +3875,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
         <is>
           <t>Прогноза выручки на 2026 нет. У кондитеров в целом дорогое какао и упаковка — без цифры именно этой компании. Последнее: 50,2 млрд за 2025.</t>
         </is>
@@ -3271,13 +3927,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H28" s="11" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="48" customHeight="1" s="6">
+    <row r="29" ht="65" customHeight="1" s="6">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Сады Придонья</t>
@@ -3313,7 +3979,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H29" s="11" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
         <is>
           <t>Выручку 2026 в деньгах не публиковали. За январь–март продали на 7,5% больше в тоннах, бренды «Сады Придонья» +11%, Nemoloko +19%. Прогноза в рублях на год нет. https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
         </is>
@@ -3355,7 +4031,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3397,7 +4083,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H31" s="11" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3439,7 +4135,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H32" s="11" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I32" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3481,13 +4187,23 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I33" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="48" customHeight="1" s="6">
+    <row r="34" ht="67" customHeight="1" s="6">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>ГК ЭкоНива (молочный контур рейтинга)</t>
@@ -3519,9 +4235,15 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H34" s="11" t="inlineStr">
-        <is>
-          <t>Официальный отчёт всей группы за полгода: 45,2 млрд (−2,8%), прибыль 1,1. Это ВСЯ компания, а не только молочная часть, которую агентство INFOLine считало за 2025 (29,8). С 29,8 сравнивать нельзя. Оценку года только для молочки не ставили. https://abireg.ru/newsitem/116916/</t>
+      <c r="H34" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I34" s="12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J34" s="13" t="inlineStr">
+        <is>
+          <t>Официальный отчёт всей группы за полгода: 45,2 млрд (−2,8%), прибыль 1,1 млрд — 2,4% от продаж всей группы. Это ВСЯ компания, а не только молочная часть, которую агентство INFOLine считало за 2025 (29,8). С 29,8 сравнивать нельзя. Оценку года только для молочки не ставили. https://abireg.ru/newsitem/116916/</t>
         </is>
       </c>
     </row>
@@ -3561,7 +4283,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H35" s="11" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I35" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J35" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3603,7 +4335,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H36" s="11" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I36" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J36" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3645,7 +4387,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H37" s="11" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J37" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3687,7 +4439,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H38" s="11" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J38" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3729,7 +4491,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H39" s="11" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J39" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3771,7 +4543,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H40" s="11" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J40" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3813,7 +4595,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H41" s="11" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3855,7 +4647,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H42" s="11" t="inlineStr">
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J42" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3897,7 +4699,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I43" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J43" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3939,7 +4751,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H44" s="11" t="inlineStr">
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -3981,7 +4803,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I45" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J45" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4023,7 +4855,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H46" s="11" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I46" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J46" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4065,7 +4907,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H47" s="11" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I47" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4107,7 +4959,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H48" s="11" t="inlineStr">
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I48" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4149,7 +5011,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H49" s="11" t="inlineStr">
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J49" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4191,7 +5063,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H50" s="11" t="inlineStr">
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J50" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4233,7 +5115,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I51" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J51" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4275,7 +5167,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H52" s="11" t="inlineStr">
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I52" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J52" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4317,7 +5219,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H53" s="11" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J53" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4359,7 +5271,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H54" s="11" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J54" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4401,7 +5323,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I55" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J55" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4443,7 +5375,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H56" s="11" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I56" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J56" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4485,7 +5427,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I57" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J57" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4527,7 +5479,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H58" s="11" t="inlineStr">
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I58" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J58" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4569,7 +5531,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H59" s="11" t="inlineStr">
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I59" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J59" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4611,7 +5583,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H60" s="11" t="inlineStr">
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I60" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J60" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4653,7 +5635,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H61" s="11" t="inlineStr">
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J61" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4695,7 +5687,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H62" s="11" t="inlineStr">
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I62" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J62" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4737,7 +5739,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H63" s="11" t="inlineStr">
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I63" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J63" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4779,7 +5791,17 @@
           <t>нет данных</t>
         </is>
       </c>
-      <c r="H64" s="11" t="inlineStr">
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="I64" s="12" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+      <c r="J64" s="13" t="inlineStr">
         <is>
           <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
         </is>
@@ -4796,7 +5818,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" style="6" min="1" max="1"/>
@@ -4826,17 +5848,17 @@
       <c r="G1" s="4" t="n"/>
     </row>
     <row r="2" ht="72" customHeight="1" s="6">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Как читать цифру 2026</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>Года ещё нет (сейчас октябрь 2026), полного отчёта за весь 2026 ни у кого нет. В столбце «факт» — уже опубликованный кусок: девять месяцев, полгода или квартал. «Оценка года» — не отчёт, а арифметика: либо прогноз самой компании, либо выручка 2025, умноженная на рост уже вышедшего куска 2026. Где куска нет — «нет данных», ничего не додумано.</t>
-        </is>
-      </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Года ещё нет (сейчас октябрь 2026), полного отчёта за весь 2026 ни у кого нет. В столбце «факт» — уже опубликованный кусок: девять месяцев, полгода или квартал. «Оценка года» — не отчёт, а арифметика: либо прогноз самой компании, либо выручка 2025, умноженная на рост уже вышедшего куска 2026. Где куска нет — «нет данных», ничего не додумано. Прибыль и маржа стоят только там, где компания сама их опубликовала за тот же кусок года.</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
         <is>
           <t>https://www.x5.ru/ru/investors/financial-and-operational-results/</t>
         </is>
@@ -4847,17 +5869,17 @@
       <c r="G2" s="3" t="n"/>
     </row>
     <row r="3" ht="72" customHeight="1" s="6">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>X5 — январь–сентябрь</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Продали за январь–сентябрь на 3,79 триллиона рублей, на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь быстрее полугодия: +13% до 1,31 триллиона. Чижик по-прежнему самый быстрый внутри группы (+31% за девять месяцев, +35% за квартал). Компания свой прогноз на весь год не снимала: +12–16%.</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
         </is>
@@ -4868,17 +5890,17 @@
       <c r="G3" s="3" t="n"/>
     </row>
     <row r="4" ht="72" customHeight="1" s="6">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>X5 — свой прогноз на год</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>В марте и снова в июне президент Екатерина Лобачева: прогноз роста выручки 12–16% на 2026 держим. От выручки 2025 (4,642 триллиона) это примерно 5,20–5,39 триллиона за полный год. Девять месяцев идут ближе к нижней границе.</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>https://www.x5.ru/ru/news/x5-predstavila-prognozy-i-orientiry-na-2026-god/</t>
         </is>
@@ -4889,17 +5911,17 @@
       <c r="G4" s="3" t="n"/>
     </row>
     <row r="5" ht="72" customHeight="1" s="6">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Магнит — полгода</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>1 887 млрд рублей за полгода, +12,8%. Магазины работают, продажи растут, по прибыли группа всё ещё в минусе: мешают проценты по кредитам. Это тот же сюжет, что в 2025: полка живая, кредиты тяжёлые.</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>1 887 млрд рублей за полгода, +12,8%. Магазины работают, продажи растут, по прибыли группа всё ещё в минусе: −1,9 млрд (без правила «аренда как долг»). Если аренду магазинов считать долгом, минус около −9,5. Мешают проценты по кредитам. Это тот же сюжет, что в 2025: полка живая, кредиты тяжёлые.</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
         </is>
@@ -4910,19 +5932,19 @@
       <c r="G5" s="3" t="n"/>
     </row>
     <row r="6" ht="72" customHeight="1" s="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Десять крупнейших сетей, январь–июнь 2026</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Агентство INFOLine сложила десятку: 6,76 триллиона рублей, +11,6% (годом раньше десятка росла на 17%). Лента +26% — самый быстрый из крупных. Светофор и Ашан продали меньше, чем год назад. На весь 2026 агентство ждёт рост крупнейших сетей примерно 9–11%.</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>https://www.kommersant.ru/doc/8923592</t>
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Прибыль и маржа — у кого уже есть</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Официальную прибыль за январь–июнь 2026 опубликовали шесть сетей и четыре завода. Сети: X5 25,7 млрд (маржа 1% — от продаж за январь–июнь 2 481, не от девяти месяцев), Магнит −1,9, Лента 13 (2%), Fix Price 2,7 (1,8%), «ДА!» 1,2 (2,8%), Винлаб 0,79 (1,5%). Заводы: Черкизово 14,1 (почти 10 копеек с рубля), Русагро почти ноль (0,056), Агроэко 1,99 (8,1%), ЭкоНива 1,1 (2,4% от всей группы). У остальных в этих столбцах «нет данных»: отчёта с прибылью за 2026 ещё нет. Мираторг писал прибыль 19,61 без полной выручки — в ячейку не ставили, маржу от этого не посчитать.</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>https://www.x5.ru/ru/investors/financial-and-operational-results/</t>
         </is>
       </c>
       <c r="D6" s="3" t="n"/>
@@ -4931,19 +5953,19 @@
       <c r="G6" s="3" t="n"/>
     </row>
     <row r="7" ht="72" customHeight="1" s="6">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Лента — полгода</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>648 млрд рублей за полгода, +26%. Тянут «Супер Лента» и «Монетка». В августе купила большие магазины «О’КЕЙ» — со второго полугодия в цифрах будут ещё и эти магазины.</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Десять крупнейших сетей, январь–июнь 2026</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Агентство INFOLine сложила десятку: 6,76 триллиона рублей, +11,6% (годом раньше десятка росла на 17%). Лента +26% — самый быстрый из крупных. Светофор и Ашан продали меньше, чем год назад. На весь 2026 агентство ждёт рост крупнейших сетей примерно 9–11%.</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
       <c r="D7" s="3" t="n"/>
@@ -4952,19 +5974,19 @@
       <c r="G7" s="3" t="n"/>
     </row>
     <row r="8" ht="72" customHeight="1" s="6">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Fix Price — полгода</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>155 млрд рублей, +4,8%. Медленнее больших продуктовых сетей: цены фиксированные, в ассортименте не только еда.</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Лента — полгода</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>648 млрд рублей за полгода, +26%. Тянут «Супер Лента» и «Монетка». В августе купила большие магазины «О’КЕЙ» — со второго полугодия в цифрах будут ещё и эти магазины.</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
         </is>
       </c>
       <c r="D8" s="3" t="n"/>
@@ -4973,19 +5995,19 @@
       <c r="G8" s="3" t="n"/>
     </row>
     <row r="9" ht="72" customHeight="1" s="6">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Винлаб — полгода</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>51 млрд рублей по официальному отчёту, +7%. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это отскок после кибератаки 2025-го, не путать с выручкой в таблице.</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Fix Price — полгода</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>155 млрд рублей, +4,8%. Медленнее больших продуктовых сетей: цены фиксированные, в ассортименте не только еда.</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
         </is>
       </c>
       <c r="D9" s="3" t="n"/>
@@ -4994,19 +6016,19 @@
       <c r="G9" s="3" t="n"/>
     </row>
     <row r="10" ht="72" customHeight="1" s="6">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Русагро — полгода</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>183 млрд рублей, +9%. Догнать PepsiCo по году ещё рано: полного 2026 нет ни у кого из заводов.</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Винлаб — полгода</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>51 млрд рублей по официальному отчёту, +7%. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это отскок после кибератаки 2025-го, не путать с выручкой в таблице.</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
         </is>
       </c>
       <c r="D10" s="3" t="n"/>
@@ -5015,19 +6037,19 @@
       <c r="G10" s="3" t="n"/>
     </row>
     <row r="11" ht="72" customHeight="1" s="6">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Черкизово — полгода</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>142 млрд рублей, всего +3,5%. Слабее роста цен в магазинах: дешевле свинина и меньше продаж в Китай.</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>https://www.interfax.ru/business/1111410</t>
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Русагро — полгода</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>183 млрд рублей, +9%. Догнать PepsiCo по году ещё рано: полного 2026 нет ни у кого из заводов.</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
         </is>
       </c>
       <c r="D11" s="3" t="n"/>
@@ -5036,19 +6058,19 @@
       <c r="G11" s="3" t="n"/>
     </row>
     <row r="12" ht="72" customHeight="1" s="6">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Дамате — полгода</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>46 млрд рублей, +19% — один из немногих заводов, у кого продажи выросли сильно.</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Черкизово — полгода</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>142 млрд рублей, всего +3,5%. Слабее роста цен в магазинах: дешевле свинина и меньше продаж в Китай.</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>https://www.interfax.ru/business/1111410</t>
         </is>
       </c>
       <c r="D12" s="3" t="n"/>
@@ -5057,19 +6079,19 @@
       <c r="G12" s="3" t="n"/>
     </row>
     <row r="13" ht="72" customHeight="1" s="6">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Мираторг — прогноз, не факт</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Выручку за 2026 пока не раскрыли. Глава группы в июне: ждать роста «на несколько процентов», продажи за границу удержать около 58 млрд рублей.</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>https://news.mail.ru/economics/71212403/</t>
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Дамате — полгода</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="inlineStr">
+        <is>
+          <t>46 млрд рублей, +19% — один из немногих заводов, у кого продажи выросли сильно.</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
         </is>
       </c>
       <c r="D13" s="3" t="n"/>
@@ -5078,19 +6100,19 @@
       <c r="G13" s="3" t="n"/>
     </row>
     <row r="14" ht="72" customHeight="1" s="6">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Что было вместо цифры, если её нет</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>По большинству сетей из регионов и заводов своего прогноза «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год +9–11%; крупные производители еды почти без роста), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку выручки это не ставили — это не продажи компании.</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Мираторг — прогноз, не факт</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Выручку за 2026 пока не раскрыли. Глава группы в июне: ждать роста «на несколько процентов», продажи за границу удержать около 58 млрд рублей.</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>https://news.mail.ru/economics/71212403/</t>
         </is>
       </c>
       <c r="D14" s="3" t="n"/>
@@ -5099,19 +6121,19 @@
       <c r="G14" s="3" t="n"/>
     </row>
     <row r="15" ht="72" customHeight="1" s="6">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Агентство INFOLine — сети на весь 2026</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (за январь–июнь десятка уже +11,6%, годом раньше было +17%). Это прогноз десятки, не «Мария-Ра» и не «Командор».</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>https://www.kommersant.ru/doc/8923592</t>
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Что было вместо цифры, если её нет</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>По большинству сетей из регионов и заводов своего прогноза «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год +9–11%; крупные производители еды почти без роста), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку выручки это не ставили — это не продажи компании.</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
       <c r="D15" s="3" t="n"/>
@@ -5120,19 +6142,19 @@
       <c r="G15" s="3" t="n"/>
     </row>
     <row r="16" ht="72" customHeight="1" s="6">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Агентство INFOLine — заводы</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже +0,4%, в 2026 рост лидеров «приблизился к нулю». KDV как пример: уже 2025 только +1%.</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
-        <is>
-          <t>https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Агентство INFOLine — сети на весь 2026</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (за январь–июнь десятка уже +11,6%, годом раньше было +17%). Это прогноз десятки, не «Мария-Ра» и не «Командор».</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>https://www.kommersant.ru/doc/8923592</t>
         </is>
       </c>
       <c r="D16" s="3" t="n"/>
@@ -5141,19 +6163,19 @@
       <c r="G16" s="3" t="n"/>
     </row>
     <row r="17" ht="72" customHeight="1" s="6">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Доставка продуктов, начало 2026</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>В январе агентство Data Insight заложило всю доставку продуктов в России на 1,8 триллиона рублей за 2026 (+24%). К марту 1,83 триллиона (+22%), к маю 1,84. Это весь рынок вместе с налогом и платой за доставку, не выручка одной Лавки или Ozon Fresh.</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
-        <is>
-          <t>https://datainsight.ru/DI_eGrocery_april_2026</t>
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>Агентство INFOLine — заводы</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже +0,4%, в 2026 рост лидеров «приблизился к нулю». KDV как пример: уже 2025 только +1%.</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
       <c r="D17" s="3" t="n"/>
@@ -5162,25 +6184,46 @@
       <c r="G17" s="3" t="n"/>
     </row>
     <row r="18" ht="72" customHeight="1" s="6">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Сети из регионов — не прогноз продаж, а продажа самой сети</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>«Верный» с октября 2025 ищут покупателя (оценка 25–35 млрд — цена всего бизнеса). «Гулливер» в начале 2026 писали как выставленный на продажу. Про «Мария-Ра» летом 2026 писали, что смотрит «Лента». Цифры выручки на 2026 никто из них не давал.</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
-        <is>
-          <t>https://www.kommersant.ru/doc/8158706</t>
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Доставка продуктов, начало 2026</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>В январе агентство Data Insight заложило всю доставку продуктов в России на 1,8 триллиона рублей за 2026 (+24%). К марту 1,83 триллиона (+22%), к маю 1,84. Это весь рынок вместе с налогом и платой за доставку, не выручка одной Лавки или Ozon Fresh.</t>
+        </is>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>https://datainsight.ru/DI_eGrocery_april_2026</t>
         </is>
       </c>
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
+    </row>
+    <row r="19" ht="72" customHeight="1" s="6">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Сети из регионов — не прогноз продаж, а продажа самой сети</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>«Верный» с октября 2025 ищут покупателя (оценка 25–35 млрд — цена всего бизнеса). «Гулливер» в начале 2026 писали как выставленный на продажу. Про «Мария-Ра» летом 2026 писали, что смотрит «Лента». Цифры выручки на 2026 никто из них не давал.</t>
+        </is>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>https://www.kommersant.ru/doc/8158706</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -5201,6 +6244,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rewrite SPAR Kaliningrad comment in plain spoken Russian
Keep the same facts and source link; drop the stiff report phrasing
so the Excel note reads as a short explanation, not a briefing.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -5983,7 +5983,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="90" customHeight="1" s="6">
+    <row r="4" ht="98" customHeight="1" s="6">
       <c r="A4" s="18" t="inlineStr">
         <is>
           <t>SPAR Калининград (ООО Евроритейл)</t>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="J4" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025 у ООО «Евроритейл»: 32,68 млрд (+15%), прибыль 0,563 млрд, маржа 1,7 копейки с рубля. Не путать с ООО «Спар-Калининград» (54 млн и 2 человека — это не магазины). Апрель 2026, замгендиректора: больше 100 магазинов, «Пятёрочка» уже около 200, с ней по числу точек и по цене в массовом сегменте не гонятся. В 2025 открыли шесть магазинов. В 2025 директор говорила: каждый год +10 точек и 20–25 реконструкций, электронные ценники уже стоят. Сигнал для ИТ: не урезают «под закрытие». Деньги скорее на реконструкцию, ценники и логистику через паром, чем на гонку с «Пятёрочкой». https://kaliningrad-news.net/society/2026/04/17/281609.html</t>
+          <t>За 2026 продаж компания не публиковала. Что есть — весь 2025 у ООО «Евроритейл»: 32,68 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 563 миллиона — это 1,7 копейки с каждого рубля. Рядом есть другое ООО — «Спар-Калининград»: 54 миллиона выручки и двое сотрудников. Это не магазины, их цифры сюда не относятся. В апреле 2026 замгендиректора сказал: магазинов уже больше ста. «Пятёрочка» в области около двухсот — по числу точек и по цене с ней не соревнуются. За 2025 открыли шесть магазинов. Директор раньше говорила: каждый год плюс десять новых и 20–25 ремонтов старых. Электронные ценники уже стоят. Для ИТ это значит: сеть живая, не сворачивается. Деньги скорее на ремонт магазинов, ценники и доставку через паром, чем на то, чтобы догнать «Пятёрочку». https://kaliningrad-news.net/society/2026/04/17/281609.html</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite all 2026 table notes in spoken Russian
Replace «кусок» with «период» in headers and comments. Keep the same
facts, numbers, and links; drop the briefing tone in chain, plant,
regional, media, and how-to text.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -460,12 +460,12 @@
     <row r="3" ht="64" customHeight="1" s="6">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Почему нет колонки «выручка за весь 2026»</t>
+          <t>Почему нет колонки «продажи за весь 2026»</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Сегодня 29 октября 2026. Год закроется 31 декабря. Полные годовые отчёты компании обычно публикуют весной 2027. Поэтому в таблице два разных числа: уже вышедший кусок года и, где можно, оценка полного года.</t>
+          <t>Сегодня 29 октября 2026. Год закроется 31 декабря. Полные годовые отчёты компании обычно публикуют весной 2027. Поэтому в таблице два разных числа: уже вышедший период и, где можно, оценка полного года.</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Только опубликованная выручка за девять месяцев, полгода или (редко) квартал. X5 — единственная из крупных, у кого на октябрь уже есть девять месяцев. Магнит, Лента, Fix Price, Русагро, Черкизово — полгода. Светофор, Mercury, Самокат, Ашан, Metro — оценки агентства INFOLine за полгода, не их собственный отчёт.</t>
+          <t>Только опубликованные продажи за девять месяцев, полгода или (редко) квартал. X5 — единственная из крупных, у кого на октябрь уже есть девять месяцев. Магнит, Лента, Fix Price, Русагро, Черкизово — полгода. Светофор, Mercury, Самокат, Ашан, Metro — оценки агентства INFOLine за полгода, не их собственный отчёт.</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Либо слова самой компании (X5: рост 12–16%; Мираторг: «несколько процентов»), либо простая арифметика: выручка 2025, умноженная на рост уже вышедшего куска 2026. Это не отчёт и не гарантия. У «Русагро» осень обычно сильнее весны — поэтому полугодие на два не умножали.</t>
+          <t>Либо слова самой компании (X5: рост 12–16%; Мираторг: «несколько процентов»), либо простая арифметика: продажи 2025, умноженные на рост уже вышедшего периода 2026. Это не отчёт и не гарантия. У «Русагро» осень обычно сильнее весны — поэтому полугодие на два не умножали.</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Прибыль — сколько денег осталось после всех расходов за тот же кусок года, что и в столбце «факт». Маржа — какая это доля от продаж: 2% значит две копейки прибыли с каждого рубля. Цифры есть только там, где компания сама опубликовала и прибыль, и продажи за один период: шесть сетей и четыре завода. Исключение — X5: продажи уже за девять месяцев, прибыль пока только за январь–июнь. У остальных в этих столбцах «нет данных».</t>
+          <t>Прибыль — сколько денег осталось после всех расходов за тот же период, что и в столбце «факт». Маржа — какая это доля от продаж: 2% значит две копейки прибыли с каждого рубля. Цифры есть только там, где компания сама опубликовала и прибыль, и продажи за один период: шесть сетей и четыре завода. Исключение — X5: продажи уже за девять месяцев, прибыль пока только за январь–июнь. У остальных в этих столбцах «нет данных».</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных». Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей +9–11%, производители еды около нуля, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
+          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных». Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей плюс 9–11%, производители еды около нуля, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Свои в рублях — почти ни у кого из тех, у кого в таблице «нет данных». X5 ещё в марте держала +12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «новые заводы начнут себя окупать», без суммы. У сетей из регионов вместо прогноза продаж были новости про продажу самой сети. Мировые PepsiCo и Nestlé дают прогноз на весь мир, не на Россию.</t>
+          <t>Свои в рублях — почти ни у кого из тех, у кого в таблице «нет данных». X5 ещё в марте держала плюс 12–16% (это уже в таблице). Мираторг в июне сказал «несколько процентов». ЭФКО — «новые заводы начнут себя окупать», без суммы. У сетей из регионов вместо прогноза продаж были новости про продажу самой сети. Мировые PepsiCo и Nestlé дают прогноз на весь мир, не на Россию.</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Шрифт Times New Roman 11, шапка и столбец «Компания» — заливка #A2C4C9, как в вашей Google-таблице. Те же десять колонок на листах «Сети», «Производители» и «Регионы». К выручке добавлены прибыль и маржа, плюс этот лист и обновлённый «Медиа».</t>
+          <t>Шрифт Times New Roman 11, шапка и столбец «Компания» — заливка #A2C4C9, как в вашей Google-таблице. Те же десять колонок на листах «Сети», «Производители» и «Регионы». К продажам добавлены прибыль и маржа, плюс этот лист и обновлённый «Медиа».</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Это сети на 30–200 точек и заводы поменьше. Выручки за кусок 2026 у них почти нет — в столбцах денег стоит «нет данных», чтобы не подменять 2026 закрытым 2025-м. В комментарии два слоя: последний закрытый год (чтобы видеть маржу и прибыль) и что видно на 2026–27 (открывают, склеивают сети, режут издержки, закрывают магазин). Никто из них не публикует «бюджет ИТ в рублях». Сигнал такой: растёт и строит склад / склеивает юрлица после сделки — ИТ скорее не режут; продажи уже падали, убыток, закрывают гипермаркет — скорее заморозка; тонкая маржа и «год эффективности» — ИТ только если окупается на издержках.</t>
+          <t>Это сети на 30–200 точек и заводы поменьше. Продаж за период 2026 у них почти нет — в столбцах денег стоит «нет данных», чтобы не подменять 2026 закрытым 2025-м. В комментарии два слоя: закрытый год (чтобы видеть прибыль) и что видно на 2026–27 (открывают, склеивают сети, режут расходы, закрывают магазин). Никто из них не публикует «бюджет ИТ в рублях». Читать так: растёт и строит склад / склеивает компании после сделки — ИТ скорее не режут; продажи уже падали, убыток, закрывают гипермаркет — скорее заморозка; прибыли мало и «год эффективности» — ИТ только если окупается на расходах.</t>
         </is>
       </c>
     </row>
@@ -597,12 +597,12 @@
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>За какой кусок года</t>
+          <t>За какой период</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Рост к тому же куску 2025, %</t>
+          <t>Рост к тому же периоду 2025, %</t>
         </is>
       </c>
       <c r="F1" s="11" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="H1" s="11" t="inlineStr">
         <is>
-          <t>Прибыль за тот же кусок, млрд ₽</t>
+          <t>Прибыль за тот же период, млрд ₽</t>
         </is>
       </c>
       <c r="I1" s="11" t="inlineStr">
@@ -631,7 +631,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="98" customHeight="1" s="6">
+    <row r="2" ht="101" customHeight="1" s="6">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>X5 Group (Пятёрочка, Перекрёсток, Чижик)</t>
@@ -669,11 +669,11 @@
       </c>
       <c r="J2" s="13" t="inlineStr">
         <is>
-          <t>Сама компания 16 октября 2026, цифры ещё без проверки аудитора. За январь–сентябрь продали на 3 791,5 млрд рублей — на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь: 1 311 млрд (+13%). Пятёрочка за девять месяцев 2 918 (+9,4%), Перекрёсток 413 (+7,1%), Чижик 391 (+31,4%), доставка X5 — 257 (+28,4%). Магазинов 30 981 на конец сентября. Прибыль в таблице — 25,7 млрд, но это не за девять месяцев, а только за январь–июнь. За девять месяцев прибыль ещё не вышла (ждут 29 октября). Маржа 1% — это 25,7 от продаж за те же январь–июнь (2 481 млрд). От 3 792 за девять месяцев считать нельзя: куски года разные. Свой прогноз на весь год компания не снимала: рост 12–16%. От выручки 2025 (4 642) это 5 200–5 385. https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="87" customHeight="1" s="6">
+          <t>Сама компания 16 октября 2026, аудитор эти цифры ещё не проверял. За январь–сентябрь продали на 3 791,5 млрд рублей — на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь: 1 311 млрд, на 13% больше. Пятёрочка за девять месяцев 2 918 млрд (на 9,4% больше), Перекрёсток 413 (на 7,1% больше), Чижик 391 (на 31,4% больше), доставка X5 — 257 (на 28,4% больше). Магазинов 30 981 на конец сентября. Прибыль в таблице — 25,7 млрд, но это не за девять месяцев, а только за январь–июнь. Прибыль за девять месяцев ещё не вышла (ждали 29 октября). 1% в столбце маржи — это 25,7 от продаж за те же январь–июнь (2 481 млрд). От 3 792 за девять месяцев считать нельзя: это разные периоды. Свой прогноз на весь год компания не меняла: рост 12–16%. От продаж 2025 (4 642) это 5 200–5 385. https://www.x5.ru/wp-content/uploads/2026/10/q3_2026_trading_update_rus.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1" s="6">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Магнит (вкл. Дикси, Самбери, Азбука вкуса)</t>
@@ -709,11 +709,11 @@
       </c>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт 28 августа 2026: за полгода продали на 1 887,2 млрд рублей (+12,8%). Из них магазины 1 871. Точек 33 652. Долги минус деньги на счетах ≈ 514,5 млрд. Прибыль за те же январь–июнь в ячейке −1,9 млрд: сеть пока в минусе, мешают проценты по кредитам. Есть второй счёт того же минуса — около −9,5: там аренду магазинов считают как долг. В ячейке стоит −1,9, без этого правила. Оценка всего года, если второе полугодие будет как первое: 3 509 × 1,128. Это не отчёт за год. https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="61" customHeight="1" s="6">
+          <t>Официальный отчёт 28 августа 2026: за полгода продали на 1 887,2 млрд рублей — на 12,8% больше, чем годом раньше. Из них магазины 1 871. Точек 33 652. Долги минус деньги на счетах примерно 514,5 млрд. Прибыль за те же январь–июнь в ячейке −1,9 млрд: сеть пока в минусе, мешают проценты по кредитам. Есть другой способ считать тот же минус — около −9,5: там аренду магазинов считают как долг. В ячейке стоит −1,9, без этого правила. Оценка всего года, если второе полугодие будет как первое: 3 509 × 1,128. Это не отчёт за год. https://www.magnit.com/ru/media/press-releases/magnit-obyavlyaet-operatstionnye-i-finansovye-rezultaty-deyatelnosti-za-pervoe-polugodie-2026-goda/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="63" customHeight="1" s="6">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Mercury Retail (Красное &amp; Белое, Бристоль)</t>
@@ -755,11 +755,11 @@
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
-          <t>Агентство INFOLine в «Коммерсанте» 2 сентября 2026: за полгода 878 млрд (+11,2%). Своего сводного отчёта всей группы нет. Оценка года, если темп удержится: 1 660 × 1,112. https://www.kommersant.ru/doc/8923592</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="88" customHeight="1" s="6">
+          <t>Агентство INFOLine в «Коммерсанте» 2 сентября 2026: за полгода 878 млрд — на 11,2% больше, чем годом раньше. Своего сводного отчёта всей группы нет. Оценка года, если тот же темп удержится: 1 660 × 1,112. https://www.kommersant.ru/doc/8923592</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="92" customHeight="1" s="6">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Группа Лента (Гипер/Супер Лента, Монетка, Улыбка радуги, Реми)</t>
@@ -795,7 +795,7 @@
       </c>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт: за полгода 648,5 млрд (+26,2%); апрель–июнь 341,6 (+28,8%). Магазинов 7 456 на 30 июня. Быстрее всех внутри группы — «Супер Лента» (+30,2%) и «Монетка» (+26,1%), большие магазины +12,9%. Прибыль за те же полгода 13 млрд — примерно 2 копейки с каждого рубля продаж. В августе купила большие магазины «О’КЕЙ» — с осени в цифрах будут ещё и чужие точки. Оценка года без этой покупки: 1 104 × 1,262. К 2028 сама Лента хочет 2,2 триллиона — это цель на потом, не на 2026. https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
+          <t>Официальный отчёт: за полгода 648,5 млрд — на 26,2% больше, чем годом раньше; апрель–июнь 341,6 млрд, на 28,8% больше. Магазинов 7 456 на 30 июня. Быстрее всех внутри группы — «Супер Лента» (на 30,2% больше) и «Монетка» (на 26,1% больше), большие магазины — на 12,9% больше. Прибыль за те же полгода 13 млрд — примерно 2 копейки с каждого рубля продаж. В августе купила большие магазины «О’КЕЙ» — с осени в цифрах будут ещё и эти точки. Оценка года без этой покупки: 1 104 × 1,262. К 2028 сама Лента хочет 2,2 триллиона — это цель на потом, не на 2026. https://www.lentagroup.ru/ru/media/news-and-press-releases/gruppa-lenta-obyavlyaet-o-roste-vyruchki-na-28-8-roste-lfl-prodazh-na-6-5-vo-2-kvartale-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="59" customHeight="1" s="6">
+    <row r="7" ht="61" customHeight="1" s="6">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>ВкусВилл</t>
@@ -887,11 +887,11 @@
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 191,06 млрд (+7,8%). Обогнал «Светофор» среди пяти крупнейших. Оценка года: 359 × 1,078. https://www.infoline.spb.ru/news/?news=308855</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="73" customHeight="1" s="6">
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 191,06 млрд — на 7,8% больше, чем годом раньше. Обогнал «Светофор» среди пяти крупнейших. Оценка года: 359 × 1,078. https://www.infoline.spb.ru/news/?news=308855</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1" s="6">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Fix Price</t>
@@ -927,11 +927,11 @@
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт 27 августа 2026: за полгода 155,3 млрд (+4,8%); апрель–июнь 82,2 (+6,9%). Магазины 138,2, опт 17,1. Точек 8 077. Прибыль за те же полгода 2,7 млрд — это 1,8% от продаж (почти 2 копейки с рубля). Оценка года: 313 × 1,048. https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="56" customHeight="1" s="6">
+          <t>Официальный отчёт 27 августа 2026: за полгода 155,3 млрд — на 4,8% больше, чем годом раньше; апрель–июнь 82,2 млрд, на 6,9% больше. Магазины 138,2, опт 17,1. Точек 8 077. Прибыль за те же полгода 2,7 млрд — это 1,8% от продаж (почти 2 копейки с рубля). Оценка года: 313 × 1,048. https://investors.fix-price.ru/upload/iblock/927/qomfciov5lu66hurwrrsb5bn5wkxeut0/PJSC_Fix_Price_announces_key_operating_and_financial_results_for_Q2_2026_RUS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1" s="6">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Самокат</t>
@@ -973,11 +973,11 @@
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>Оценка агентства INFOLine / «Коммерсантъ»: за полгода 135 млрд (+15,5%). Оценка года: 279 × 1,155. https://www.kommersant.ru/doc/8923592</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="56" customHeight="1" s="6">
+          <t>Оценка агентства INFOLine / «Коммерсантъ»: за полгода 135 млрд — на 15,5% больше, чем годом раньше. Оценка года: 279 × 1,155. https://www.kommersant.ru/doc/8923592</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="57" customHeight="1" s="6">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>METRO Россия</t>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 118,9 млрд (+0,5%). Оценка года: 260 × 1,005. https://www.kommersant.ru/doc/8923610</t>
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 118,9 млрд — на 0,5% больше, чем годом раньше. Оценка года: 260 × 1,005. https://www.kommersant.ru/doc/8923610</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="80" customHeight="1" s="6">
+    <row r="12" ht="83" customHeight="1" s="6">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Ozon + Ozon Fresh</t>
@@ -1117,11 +1117,11 @@
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>Сколько именно продуктов продал Ozon Fresh в 2026, компания не говорит — ни факта, ни своего прогноза. Что было в начале года: агентство Data Insight в январе ждало, что вся доставка продуктов в России за 2026 год будет около 1,8 триллиона рублей (+24% к 2025). К марту уточнили 1,83 триллиона (+22%), к маю 1,84. Это весь рынок доставки, не цифра Ozon. За апрель–июнь пять сервисов (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) вместе сделали 260 млрд; заказы Ozon Fresh +65%. https://datainsight.ru/DI_eGrocery_april_2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="72" customHeight="1" s="6">
+          <t>Сколько именно продуктов продал Ozon Fresh в 2026, компания не говорит — ни факта, ни своего прогноза. Что было в начале года: агентство Data Insight в январе ждало, что вся доставка продуктов в России за 2026 год будет около 1,8 триллиона рублей (на 24% больше, чем в 2025). К марту уточнили 1,83 триллиона (на 22% больше), к маю 1,84. Это весь рынок доставки, не цифра Ozon. За апрель–июнь пять сервисов (Самокат, ВкусВилл, Лавка, Пятёрочка, Ozon Fresh) вместе сделали 260 млрд; заказы Ozon Fresh выросли на 65%. https://datainsight.ru/DI_eGrocery_april_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1" s="6">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Яндекс Лавка</t>
@@ -1169,11 +1169,11 @@
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>Выручку Лавки отдельно не публикуют, своего прогноза по ней тоже не было. Весь интернет-блок Яндекса (Лавка + Маркет + Еда + Деливери) за полгода 247 млрд (+19%) — туда входят не только продукты. Заказов у Лавки за апрель–июнь +5%. Прогноз агентства Data Insight на 2026 — вся доставка продуктов в стране 1,83–1,84 триллиона. Это не цифра Лавки. https://datainsight.ru/DI_eGrocery_april_2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="72" customHeight="1" s="6">
+          <t>Продажи Лавки отдельно не публикуют, своего прогноза по ней тоже не было. Весь интернет-блок Яндекса (Лавка + Маркет + Еда + Деливери) за полгода 247 млрд — на 19% больше, чем годом раньше. Туда входят не только продукты. Заказов у Лавки за апрель–июнь на 5% больше. Прогноз агентства Data Insight на 2026 — вся доставка продуктов в стране 1,83–1,84 триллиона. Это не цифра Лавки. https://datainsight.ru/DI_eGrocery_april_2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="76" customHeight="1" s="6">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>ГК О'КЕЙ / Да!</t>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>Большие магазины «О’КЕЙ» в конце 2025 продали. У оставшейся компании на бирже теперь только «ДА!»: за полгода 43,3 млрд (+10,4%), 236 магазинов. Прибыль только «ДА!» за те же полгода 1,2 млрд — 2,8% от продаж. Оценка года именно «ДА!»: 80 × 1,104. Большие магазины ООО «О’КЕЙ» за полгода 68,2 (−5,6%) — это уже Лента, с «ДА!» не складывать. https://okeygroup.lu/upload/IFRS%201H2026_RUS_final_.pdf</t>
+          <t>Большие магазины «О’КЕЙ» в конце 2025 продали. У оставшейся компании на бирже теперь только «ДА!»: за полгода 43,3 млрд — на 10,4% больше, чем годом раньше, 236 магазинов. Прибыль только «ДА!» за те же полгода 1,2 млрд — 2,8% от продаж. Оценка года именно «ДА!»: 80 × 1,104. Большие магазины ООО «О’КЕЙ» за полгода 68,2 млрд — на 5,6% меньше, чем годом раньше. Это уже Лента, с «ДА!» не складывать. https://okeygroup.lu/upload/IFRS%201H2026_RUS_final_.pdf</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не было. В начале 2026 про «Гулливер» из той же группы писали: сеть выставлена на продажу. Аналитик Совкомбанка: независимые сети, которые в 2025 продали больше чем на 100 млрд (Победа, Командор, Ярче, Аникс), в ближайшие 2–3 года могут сменить хозяина. Это не цифра выручки. Последнее открытое: 176 млрд за 2025. https://www.kommersant.ru/doc/8364093</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не было. В начале 2026 про «Гулливер» из той же группы писали: сеть выставлена на продажу. Аналитик Совкомбанка: независимые сети, которые в 2025 продали больше чем на 100 млрд (Победа, Командор, Ярче, Аникс), в ближайшие 2–3 года могут сменить хозяина. Это не цифра продаж. Последнее открытое: 176 млрд за 2025. https://www.kommersant.ru/doc/8364093</t>
         </is>
       </c>
     </row>
@@ -1313,11 +1313,11 @@
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. В обзорах конца 2025 и 2026 сеть называют как возможную покупку для крупного игрока — не как компанию со своим прогнозом. Последнее открытое: 168 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="70" customHeight="1" s="6">
+          <t>Прогноза продаж на 2026 нет. В обзорах конца 2025 и 2026 сеть называют как возможную покупку для крупного игрока — не как компанию со своим прогнозом. Последнее открытое: 168 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1" s="6">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Гиперглобус (Globus)</t>
@@ -1357,11 +1357,11 @@
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 80,6 млрд без налога (+2,7%). В тех же магазинах, что были год назад, продажи +5,7%, средний чек +7,5%. Своего прогноза выручки на 2026 нет. Новый большой магазин планируют на 2027 (больше 4 млрд на стройку) — это не цифра продаж на этот год. Оценка года: 165,6 × 1,027. https://www.kommersant.ru/doc/9005166</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="66" customHeight="1" s="6">
+          <t>Агентство INFOLine / «Коммерсантъ»: за полгода 80,6 млрд без налога — на 2,7% больше, чем годом раньше. В тех же магазинах, что были год назад, продажи выросли на 5,7%, средний чек — на 7,5%. Своего прогноза продаж на 2026 нет. Новый большой магазин планируют на 2027 (больше 4 млрд на стройку) — это не цифра продаж на этот год. Оценка года: 165,6 × 1,027. https://www.kommersant.ru/doc/9005166</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="65" customHeight="1" s="6">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Верный (Союз Святого Иоанна Воина)</t>
@@ -1409,11 +1409,11 @@
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. В октябре 2025 основатель искал покупателя: сеть оценивали в 25–35 млрд рублей. Это цена всего бизнеса, если его продадут, а не «сколько продадут за год». Российский отчёт за 2025 вышел 1 апреля 2026: 154,4 млрд — это прошлый год. https://www.kommersant.ru/doc/8158706</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="62" customHeight="1" s="6">
+          <t>Прогноза продаж на 2026 нет. В октябре 2025 основатель искал покупателя: сеть оценивали в 25–35 млрд рублей. Это цена всего бизнеса, если его продадут, а не «сколько продадут за год». Отчёт за 2025 вышел 1 апреля 2026: 154,4 млрд — это прошлый год. https://www.kommersant.ru/doc/8158706</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="64" customHeight="1" s="6">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>SPAR Миддл Волга (SPAR, EUROSPAR)</t>
@@ -1455,11 +1455,11 @@
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Агентство INFOLine / «Коммерсантъ»: «Спар Миддл Волга, Smart» за полгода 103,57 млрд (+7,8%). Тут шире, чем строка 2025 (тогда только SPAR Миддл Волга — 136 за год). Грубая оценка года: 136 × 1,078. https://www.kommersant.ru/doc/8923592</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="68" customHeight="1" s="6">
+          <t>Агентство INFOLine / «Коммерсантъ»: «Спар Миддл Волга, Smart» за полгода 103,57 млрд — на 7,8% больше, чем годом раньше. Тут шире, чем строка 2025 (тогда только SPAR Миддл Волга — 136 за год). Грубая оценка года: 136 × 1,078. https://www.kommersant.ru/doc/8923592</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="69" customHeight="1" s="6">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Мария-Ра (Розница К-1)</t>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. Последнее: российский отчёт за 2025 — 127,5 млрд (+5%). На 1 июля 2026 — 1 303 магазина (это штуки, не деньги). Летом 2026 писали, что «Лента» смотрит покупку — сделка не подтверждена и цифры года не даёт. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+          <t>Прогноза продаж на 2026 нет. Последнее: отчёт за 2025 — 127,5 млрд, на 5% больше, чем годом раньше. На 1 июля 2026 — 1 303 магазина (это штуки, не деньги). Летом 2026 писали, что «Лента» смотрит покупку — сделка не подтверждена и цифры года не даёт. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -1609,11 +1609,11 @@
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. В списках возможных покупок 2026–2028 (Совкомбанк) — без суммы продаж. Последнее открытое: около 100 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="78" customHeight="1" s="6">
+          <t>Прогноза продаж на 2026 нет. В списках возможных покупок 2026–2028 (Совкомбанк) — без суммы продаж. Последнее открытое: около 100 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1" s="6">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Винлаб (ПАО ВинЛаб / Novabev)</t>
@@ -1649,7 +1649,7 @@
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт 24 августа 2026: за полгода 51,2 млрд (+7,2%), прибыль 0,79 млрд (1,5% от продаж — полторы копейки с рубля), точек 2 225 на 30 июня (2 222 на 30 сентября). Оценка года, если темп полугодия удержится: 95,1 × 1,072. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это не та выручка, что в таблице. https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
+          <t>Официальный отчёт 24 августа 2026: за полгода 51,2 млрд — на 7,2% больше, чем годом раньше, прибыль 0,79 млрд (1,5% от продаж — полторы копейки с рубля), точек 2 225 на 30 июня (2 222 на 30 сентября). Оценка года, если темп полугодия удержится: 95,1 × 1,072. Отдельно компания хвалится продажами с налогом за девять месяцев (на 24% больше) — это не те продажи, что в таблице. https://corp.winelab.ru/ru/press-center/news-and-press-releases/vyruchka-vinlab-vyrosla-na-7-2-i-prevysila-51-mlrd-rubley-v-pervom-polugodii-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="J24" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="J28" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. Упоминается рядом с «Победой», «Ярче» и «Командором» как сеть, которую крупный игрок может купить. Последнее: 31,3 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
+          <t>Прогноза на 2026 нет. Упоминается рядом с «Победой», «Ярче» и «Командором» как сеть, которую крупный игрок может купить. Последнее открытое: 31,3 млрд за 2025. https://iz.ru/2152177/denis-kuznetcov/lenta-mozhet-poglotit-krupneyshego-riteylera-sibiri</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2169,7 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — выручка 2025. Российский отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей +9–11% за год) — не прогноз именно этой сети.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали — ни в конце 2025, ни в начале 2026. Последняя открытая цифра — продажи за 2025. Отчёт за 2026 выйдет весной 2027. Общий фон рынка (десять крупнейших сетей за год плюс 9–11%) — не прогноз именно этой сети.</t>
         </is>
       </c>
     </row>
@@ -2582,12 +2582,12 @@
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>За какой кусок года</t>
+          <t>За какой период</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Рост к тому же куску 2025, %</t>
+          <t>Рост к тому же периоду 2025, %</t>
         </is>
       </c>
       <c r="F1" s="11" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="H1" s="11" t="inlineStr">
         <is>
-          <t>Прибыль за тот же кусок, млрд ₽</t>
+          <t>Прибыль за тот же период, млрд ₽</t>
         </is>
       </c>
       <c r="I1" s="11" t="inlineStr">
@@ -2668,7 +2668,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="72" customHeight="1" s="6">
+    <row r="3" ht="74" customHeight="1" s="6">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Русагро</t>
@@ -2706,7 +2706,7 @@
       </c>
       <c r="J3" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт: за полгода 183,0 млрд (+9,1%). Прибыль почти ноль: 56 миллионов рублей, это 0,056 млрд — меньше одной десятой копейки с рубля продаж. У растениеводства и сахара осень обычно сильнее весны, поэтому полугодие на два не умножали. Оценка года, если темп удержится: 396,5 × 1,091. https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
+          <t>Официальный отчёт: за полгода 183,0 млрд — на 9,1% больше, чем годом раньше. Прибыль почти ноль: 56 миллионов рублей, это 0,056 млрд — меньше одной десятой копейки с рубля продаж. У растениеводства и сахара осень обычно сильнее весны, поэтому полугодие на два не умножали. Оценка года, если тот же темп удержится: 396,5 × 1,091. https://www.rusagrogroup.ru/fileadmin/files/reports/ru/pdf/Rusagro_Group_PJSC_IFRS_6m_2026_RUS.pdf</t>
         </is>
       </c>
     </row>
@@ -2758,11 +2758,11 @@
       </c>
       <c r="J4" s="13" t="inlineStr">
         <is>
-          <t>Цифры на 2026 нет. На 2025 сами планировали 440 млрд — не получилось (факт 344, рост ноль). Весной 2026 руководство: новые заводы начнут себя окупать в 2026–2027, ждут рост продаж и прибыли — без конкретной суммы. https://abireg.ru/newsitem/113897/</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="76" customHeight="1" s="6">
+          <t>Цифр на 2026 нет. На 2025 сами планировали 440 млрд — не получилось (факт 344, рост ноль). Весной 2026 руководство: новые заводы начнут себя окупать в 2026–2027, ждут рост продаж и прибыли — без конкретной суммы. https://abireg.ru/newsitem/113897/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="79" customHeight="1" s="6">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>АПХ Мираторг</t>
@@ -2808,7 +2808,7 @@
       </c>
       <c r="J5" s="13" t="inlineStr">
         <is>
-          <t>Полной выручки за январь–июнь 2026 в открытом виде нет. Глава компании Виктор Линник в июне на Петербургском экономическом форуме: ждать рост продаж «на несколько процентов»; продажи за границу удержать около 58 млрд, как в 2025 (план +20% сняли — рубль слишком крепкий). Оценка года ≈ 342 × 1,03. Прибыль за полгода 19,61 млрд (+26%) — это не выручка. https://echomsk.spb.ru/nws/5317198-miratorg-ogidaet-neznachitelnyj-rost-vyruchki-po-itogam-2026-goda.html</t>
+          <t>Полных продаж за январь–июнь 2026 в открытом виде нет. Глава компании Виктор Линник в июне на Петербургском экономическом форуме: ждать рост продаж «на несколько процентов»; продажи за границу удержать около 58 млрд, как в 2025 (план «плюс 20%» сняли — рубль слишком крепкий). Оценка года примерно 342 × 1,03. Прибыль за полгода 19,61 млрд — на 26% больше, чем годом раньше. Это не продажи. https://echomsk.spb.ru/nws/5317198-miratorg-ogidaet-neznachitelnyj-rost-vyruchki-po-itogam-2026-goda.html</t>
         </is>
       </c>
     </row>
@@ -2860,11 +2860,11 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. Агентство INFOLine берёт KDV как пример торможения: уже 2025 только +1%, а в 2026 у крупных производителей еды рост «около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="77" customHeight="1" s="6">
+          <t>Прогноза на 2026 нет. Агентство INFOLine берёт KDV как пример торможения: уже 2025 только на 1% больше, а в 2026 у крупных производителей еды рост «около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="79" customHeight="1" s="6">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Черкизово</t>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт: за полгода 141,6 млрд (+3,5%). Прибыль за те же полгода 14,1 млрд — почти 10 копеек с каждого рубля продаж. Свой прогноз в рублях на год компания не давала — только «продолжим увеличивать выручку», деньги на стройки в 2026 снова режут. Независимая оценка на сайте для инвесторов: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
+          <t>Официальный отчёт: за полгода 141,6 млрд — на 3,5% больше, чем годом раньше. Прибыль за те же полгода 14,1 млрд — почти 10 копеек с каждого рубля продаж. Свой прогноз в рублях на год компания не давала — только «продолжим увеличивать продажи», деньги на стройки в 2026 снова режут. Независимая оценка на сайте для инвесторов: 305–315 млрд за год (это не отчёт компании). В ячейке оценки — 288,7 × 1,035. https://cherkizovo-group.com/press/gruppa-cherkizovo-obyavlyaet-finansovye-rezultaty-za-2025-god/</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>Выручки и прогноза по России на 2026 нет. Оценка аналитиков по всей мировой Nestlé: рост продаж около 3,5–3,7% за год — не российская цифра. https://www.nestle.com/sites/default/files/2026-10/nestle-sa-consensus-pre-Q32026.pdf</t>
+          <t>Продаж и прогноза по России на 2026 нет. Оценка аналитиков по всей мировой Nestlé: рост продаж около 3,5–3,7% за год — не российская цифра. https://www.nestle.com/sites/default/files/2026-10/nestle-sa-consensus-pre-Q32026.pdf</t>
         </is>
       </c>
     </row>
@@ -3058,11 +3058,11 @@
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза выручки по России на 2026 не публиковали.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="57" customHeight="1" s="6">
+          <t>Своего прогноза продаж по России на 2026 не публиковали.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1" s="6">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Продимекс (сумма предприятий группы)</t>
@@ -3110,11 +3110,11 @@
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 не было. Открытое — сумма заводов за 2025 (около 220–224 млрд, считают по-разному). Российский отчёт за 2026 выйдет весной 2027.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="57" customHeight="1" s="6">
+          <t>Прогноза продаж на 2026 не было. Открытое — сумма заводов за 2025 (около 220–224 млрд, считают по-разному). Отчёт за 2026 выйдет весной 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="59" customHeight="1" s="6">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Агропромкомплектация</t>
@@ -3162,11 +3162,11 @@
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>Прогноза всей группы на 2026 нет. Агентство INFOLine за 2025: 204,4 млрд (+15%). Отдельные компании группы (АПК-Курск и другие) отчитываются раз в год.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="71" customHeight="1" s="6">
+          <t>Прогноза всей группы на 2026 нет. Агентство INFOLine за 2025: 204,4 млрд — на 15% больше, чем годом раньше. Отдельные компании группы (АПК-Курск и другие) отчитываются раз в год.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="73" customHeight="1" s="6">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Логика молока (ex-Danone / Health&amp;Nutrition)</t>
@@ -3206,7 +3206,7 @@
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>Сама компания 16 июля 2026: за полгода продали на 84,5 млрд (+3,5%), молочки 510 тысяч тонн (+2,7%). Ориентир на год — не деньги, а «сделать больше 1 миллиона тонн готовой продукции». На стройки и оборудование до 2030 заложили 120 млрд. Оценка рублей на год: 167,1 × 1,035. https://logikamoloka.ru/press-centr/news/logika-moloka-podvodit-rezultaty-i-polugodiya-2026-goda/</t>
+          <t>Сама компания 16 июля 2026: за полгода продали на 84,5 млрд — на 3,5% больше, чем годом раньше, молочки 510 тысяч тонн (на 2,7% больше). Ориентир на год — не деньги, а «сделать больше 1 миллиона тонн готовой продукции». На стройки и оборудование до 2030 заложили 120 млрд. Оценка рублей на год: 167,1 × 1,035. https://logikamoloka.ru/press-centr/news/logika-moloka-podvodit-rezultaty-i-polugodiya-2026-goda/</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>Выручки 2026 нет. План без суммы: пиво — больше 30% рынка, напитки без алкоголя — больше 8% продаж за первое полугодие, 700 миллионов в завод в Саранске в 2026. https://napitkivmeste.ru/odin-god-pod-brendom-napitki-vmeste-bolee-30-novyh-produktov-i-rekordnye-vlozheniya-v-zavody/</t>
+          <t>Продаж за 2026 нет. План без суммы: пиво — больше 30% рынка, напитки без алкоголя — больше 8% продаж за первое полугодие, 700 миллионов в завод в Саранске в 2026. https://napitkivmeste.ru/odin-god-pod-brendom-napitki-vmeste-bolee-30-novyh-produktov-i-rekordnye-vlozheniya-v-zavody/</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. В 2025 выпуск пива упал на 16% — компания сама сказала, что так и задумала: обновляли заводы. Это про прошлый год, не про 2026. https://www.kommersant.ru/doc/8401281</t>
+          <t>Прогноза продаж на 2026 нет. В 2025 выпуск пива упал на 16% — компания сама сказала, что так и задумала: обновляли заводы. Это про прошлый год, не про 2026. https://www.kommersant.ru/doc/8401281</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. После убытка 2025 (около 4,2 млрд) группа сама сказала: новые большие стройки пока не начинаем, сначала надо выйти в плюс; точечно около 500 миллионов в Томскую птицефабрику. https://www.akm.ru/news/gruppa_kompaniy_sibagro_narastila_vyruchku_na_14_odnako_zakonchila_2025_god_s_chistym_ubytkom/</t>
+          <t>Прогноза продаж на 2026 нет. После убытка 2025 (около 4,2 млрд) группа сама сказала: новые большие стройки пока не начинаем, сначала надо выйти в плюс; точечно около 500 миллионов в Томскую птицефабрику. https://www.akm.ru/news/gruppa_kompaniy_sibagro_narastila_vyruchku_na_14_odnako_zakonchila_2025_god_s_chistym_ubytkom/</t>
         </is>
       </c>
     </row>
@@ -3466,11 +3466,11 @@
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза выручки на 2026 не публиковали. Последнее: около 88 млрд за 2025 (агентство INFOLine).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="61" customHeight="1" s="6">
+          <t>Своего прогноза продаж на 2026 не публиковали. Последнее: около 88 млрд за 2025 (агентство INFOLine).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="62" customHeight="1" s="6">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Дамате</t>
@@ -3512,7 +3512,7 @@
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Пресс-служба 7 сентября 2026: за полгода 46,3 млрд (+19%). Оценка года: 82,8 × 1,19. https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
+          <t>Пресс-служба 7 сентября 2026: за полгода 46,3 млрд — на 19% больше, чем годом раньше. Оценка года: 82,8 × 1,19. https://www.acdamate.com/press-center/press/vyruchka-damate-v-i-polugodii-2026-goda-vyrosla-na-19-i-prevysila-46-mlrd-rubley/</t>
         </is>
       </c>
     </row>
@@ -3564,11 +3564,11 @@
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. Агентство INFOLine отмечает группу среди быстрорастущих молочников 2025, без цифры на этот год. Последнее: только молочная часть 63,1 млрд за 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="52" customHeight="1" s="6">
+          <t>Прогноза продаж на 2026 нет. Агентство INFOLine отмечает группу среди быстрорастущих молочников 2025, без цифры на этот год. Последнее: только молочная часть 63,1 млрд за 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="53" customHeight="1" s="6">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Орими Трейд (Tess, Greenfield, Jardin)</t>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза по России на 2026 не публиковали. Последнее: 62,3 млрд за 2025.</t>
+          <t>Своего прогноза по России на 2026 не публиковали. Последнее открытое: 62,3 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3762,11 +3762,11 @@
       </c>
       <c r="J24" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт за полгода: 24,63 млрд — на 6,4% меньше, чем 26,31 годом раньше. Прибыль 1,99 млрд (−40% к прошлому году) — это 8,1% от продаж. Оценка года: 56,4 × 0,936. Свинины в тоннах сделали на 10% больше, но она подешевела. https://www.tbank.ru/invest/social/profile/Marten_Resting/cbc77ff8-2a7f-49ae-8534-59a60c86da65/</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="55" customHeight="1" s="6">
+          <t>Официальный отчёт за полгода: 24,63 млрд — на 6,4% меньше, чем 26,31 годом раньше. Прибыль 1,99 млрд (на 40% меньше, чем год назад) — это 8,1% от продаж. Оценка года: 56,4 × 0,936. Свинины в тоннах сделали на 10% больше, но она подешевела. https://www.tbank.ru/invest/social/profile/Marten_Resting/cbc77ff8-2a7f-49ae-8534-59a60c86da65/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="57" customHeight="1" s="6">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Прогресс (ФрутоНяня / Малышам)</t>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. В марте 2026 вышел отчёт за 2025: выручка 52,1 (+8%), прибыль 10,2. https://www.kommersant.ru/doc/8552221</t>
+          <t>Прогноза на 2026 нет. В марте 2026 вышел отчёт за 2025: продажи 52,1 млрд — на 8% больше, чем годом раньше, прибыль 10,2. https://www.kommersant.ru/doc/8552221</t>
         </is>
       </c>
     </row>
@@ -3866,11 +3866,11 @@
       </c>
       <c r="J26" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. Июль 2026: до 2028 вложат около 13 млрд в новые линии (белки из молока и другие ингредиенты) — это деньги на стройку, не «сколько продадут за год». https://milknews.ru/index/molochnye-produkty/molvest-13-mlrd-investicii.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="56" customHeight="1" s="6">
+          <t>Прогноза продаж на 2026 нет. Июль 2026: до 2028 вложат около 13 млрд в новые линии (белки из молока и другие ингредиенты) — это деньги на стройку, не «сколько продадут за год». https://milknews.ru/index/molochnye-produkty/molvest-13-mlrd-investicii.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="57" customHeight="1" s="6">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Эссен Продакшн (Махеевъ)</t>
@@ -3918,7 +3918,7 @@
       </c>
       <c r="J27" s="13" t="inlineStr">
         <is>
-          <t>Прогноза выручки на 2026 нет. У кондитеров в целом дорогое какао и упаковка — без цифры именно этой компании. Последнее: 50,2 млрд за 2025.</t>
+          <t>Прогноза продаж на 2026 нет. У кондитеров в целом дорогое какао и упаковка — без цифры именно этой компании. Последнее открытое: 50,2 млрд за 2025.</t>
         </is>
       </c>
     </row>
@@ -3970,11 +3970,11 @@
       </c>
       <c r="J28" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="65" customHeight="1" s="6">
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="66" customHeight="1" s="6">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Сады Придонья</t>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="J29" s="13" t="inlineStr">
         <is>
-          <t>Выручку 2026 в деньгах не публиковали. За январь–март продали на 7,5% больше в тоннах, бренды «Сады Придонья» +11%, Nemoloko +19%. Прогноза в рублях на год нет. https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
+          <t>Продажи 2026 в деньгах не публиковали. За январь–март продали на 7,5% больше в тоннах, бренды «Сады Придонья» — на 11% больше, Nemoloko — на 19% больше. Прогноза в рублях на год нет. https://companies.rbc.ru/news/kwQXFC9CLJ/kak-sadyi-pridonya-adaptiruyutsya-v-usloviyah-ryinochnoj-neopredelennosti/</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4230,11 +4230,11 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="67" customHeight="1" s="6">
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="68" customHeight="1" s="6">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>ГК ЭкоНива (молочный контур рейтинга)</t>
@@ -4274,7 +4274,7 @@
       </c>
       <c r="J34" s="13" t="inlineStr">
         <is>
-          <t>Официальный отчёт всей группы за полгода: 45,2 млрд (−2,8%), прибыль 1,1 млрд — 2,4% от продаж всей группы. Это ВСЯ компания, а не только молочная часть, которую агентство INFOLine считало за 2025 (29,8). С 29,8 сравнивать нельзя. Оценку года только для молочки не ставили. https://abireg.ru/newsitem/116916/</t>
+          <t>Официальный отчёт всей группы за полгода: 45,2 млрд — на 2,8% меньше, чем годом раньше, прибыль 1,1 млрд — 2,4% от продаж всей группы. Это вся компания, а не только молочная часть, которую агентство INFOLine считало за 2025 (29,8). С 29,8 сравнивать нельзя. Оценку года только для молочки не ставили. https://abireg.ru/newsitem/116916/</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4898,7 +4898,7 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5158,7 @@
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5418,7 +5418,7 @@
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5730,7 +5730,7 @@
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>Своего прогноза «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Российский отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5883,12 +5883,12 @@
       </c>
       <c r="D1" s="17" t="inlineStr">
         <is>
-          <t>За какой кусок года</t>
+          <t>За какой период</t>
         </is>
       </c>
       <c r="E1" s="17" t="inlineStr">
         <is>
-          <t>Рост к тому же куску 2025, %</t>
+          <t>Рост к тому же периоду 2025, %</t>
         </is>
       </c>
       <c r="F1" s="17" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="H1" s="17" t="inlineStr">
         <is>
-          <t>Прибыль за тот же кусок, млрд ₽</t>
+          <t>Прибыль за тот же период, млрд ₽</t>
         </is>
       </c>
       <c r="I1" s="17" t="inlineStr">
@@ -5933,7 +5933,7 @@
       <c r="I2" s="17" t="n"/>
       <c r="J2" s="17" t="n"/>
     </row>
-    <row r="3" ht="83" customHeight="1" s="6">
+    <row r="3" ht="85" customHeight="1" s="6">
       <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Семишагофф (ООО ТК Прогресс)</t>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="J3" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 компания не публиковала. Последний закрытый год — весь 2025: 70,67 млрд (+29%), прибыль 0,955 млрд, маржа 1,4 копейки с рубля. К 2025–началу 2026 около 190 магазинов. В 2025 купили склад в Шушарах почти на 1,5 млрд — это не «сворачиваемся». В августе 2026 агентство INFOLine: с метра площади в 2025-м впервые больше 1 млн рублей, второе место в стране после «Азбуки вкуса». Сигнал для ИТ на 2026–27: резать незачем. Сеть растёт, склад свой, кассы и учёт будут нужны на большом обороте. https://checko.ru/company/tk-progress-1127847102338</t>
+          <t>За 2026 продаж компания не публиковала. Что есть — весь 2025: 70,67 млрд рублей, на 29% больше, чем годом раньше. После расходов осталось 955 миллионов — это 1,4 копейки с каждого рубля. К началу 2026 около 190 магазинов. В 2025 купили склад в Шушарах почти за 1,5 млрд — так не делают, если собираются сворачиваться. В августе 2026 агентство INFOLine: с квадратного метра в 2025-м впервые больше миллиона рублей, второе место в стране после «Азбуки вкуса». Для ИТ это значит: резать незачем. Сеть растёт, склад свой, кассы и учёт будут нужны. https://checko.ru/company/tk-progress-1127847102338</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="88" customHeight="1" s="6">
+    <row r="5" ht="90" customHeight="1" s="6">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Лама (SPAR / Первоцен / F City; сумма 4 юрлиц)</t>
@@ -6079,11 +6079,11 @@
       </c>
       <c r="J5" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — сумма четырёх магазинных юрлиц за 2025: 5,6 + 7 + 8,7 + 11 = 32,3 млрд, прибыль 0,335 млрд, маржа около 1 копейки с рубля. Управляющую «Ламу» (134 млн) с магазинами не складывали. ФАС 20 октября 2025 согласовала, чтобы «Лама» полностью управляла SPAR, «Первоценом» и F City в Томской и Новосибирской областях. У самой «Ламы» тогда 103 магазина. Сигнал для ИТ на 2026–27: скорее потратят на склейку касс, справочников и склада после сделки, чем выкинут систему. Своего «в 2026 продадим на столько-то» не было. https://retailer.ru/fas-soglasovala-pokupku-lamoj-seti-spar-v-tomskoj-i-novosibirskoj-oblastjah/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="81" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — сумма четырёх магазинных компаний за 2025: 5,6 + 7 + 8,7 + 11 = 32,3 млрд рублей. После расходов осталось 335 миллионов — около одной копейки с рубля. Управляющую компанию «Лама» (134 млн) с магазинами не складывали. 20 октября 2025 антимонопольная служба разрешила «Ламе» полностью управлять SPAR, «Первоценом» и F City в Томской и Новосибирской областях. Тогда у «Ламы» было 103 магазина. Для ИТ это значит: скорее потратят на то, чтобы склеить кассы, справочники и склад после сделки, чем выкинут систему. Своего плана «в 2026 продадим на столько-то» не было. https://retailer.ru/fas-soglasovala-pokupku-lamoj-seti-spar-v-tomskoj-i-novosibirskoj-oblastjah/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="79" customHeight="1" s="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Аникс (ТС Аникс + Прайд-А)</t>
@@ -6129,11 +6129,11 @@
       </c>
       <c r="J6" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — два юрлица за 2025: 18,3 + 13,0 = 31,3 млрд, прибыль 0,414 млрд, маржа 1,3 копейки с рубля. Своих магазинов 165, ещё 109 франшиза «Корзинка». В 2025 прибыль выросла. Своего плана продаж на 2026 не публиковали. Сигнал для ИТ: живой региональный игрок с прибылью, не «режим выживания». Но и программы «тратим на цифру столько-то» нет — бюджет ИТ в рублях никто не раскрывал. https://tolknews.ru/ekonomika/214569-skolko-zarabotali-krupneyshie-seti-altaya-mariya-ra-i-aniks-v-godu</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — две компании за 2025: 18,3 + 13,0 = 31,3 млрд рублей. После расходов осталось 414 миллионов — 1,3 копейки с рубля. Своих магазинов 165, ещё 109 работают как франшиза «Корзинка». В 2025 прибыль выросла. Плана продаж на 2026 не публиковали. Для ИТ это значит: сеть живая и с прибылью, не экономит на всём. Но сколько именно тратят на ИТ — никто не говорит. https://tolknews.ru/ekonomika/214569-skolko-zarabotali-krupneyshie-seti-altaya-mariya-ra-i-aniks-v-godu</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="82" customHeight="1" s="6">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Европа (ООО Европа, Курск)</t>
@@ -6179,11 +6179,11 @@
       </c>
       <c r="J7" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 31 млрд (+2,7%), прибыль 1,1 млрд, маржа 3,6 копейки с рубля — для продуктов густо. Директор: 47 магазинов (34 гипер, 7 супер, 6 у дома). На сайте компании «около 60 предприятий». Рост продаж слабый. Своего прогноза на 2026 нет. Сигнал для ИТ: сеть на ногах и не продаётся федералам (слова директора). Больших строек и «режем всё» в открытом виде тоже нет — скорее держат текущие системы. https://www.audit-it.ru/contragent/1074632016205_ooo-evropa</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="90" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 31 млрд рублей, на 2,7% больше, чем годом раньше. После расходов осталось 1,1 млрд — 3,6 копейки с рубля, для продуктов это много. Директор говорит: 47 магазинов (34 больших, 7 супермаркетов, 6 у дома). На сайте компании «около 60 предприятий». Продажи почти не растут. Прогноза на 2026 нет. Для ИТ это значит: сеть на ногах и, по словам директора, федералам не продаётся. Больших строек и «режем всё» тоже не видно — скорее держат то, что уже есть. https://www.audit-it.ru/contragent/1074632016205_ooo-evropa</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="92" customHeight="1" s="6">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Бегемаг / SPAR Кузбасс (ООО Универсамы Бегемаг)</t>
@@ -6229,11 +6229,11 @@
       </c>
       <c r="J8" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 12,87 млрд (+1%), прибыль всего 65 млн, маржа полкопейки с рубля. На начало 2026: 74 магазина, закрытий не было. В 2025 новые точки почти не открывали: эффективность, аренда, тарифы. Запустили SPAR-Express и кассы самообслуживания. Июль 2026: в нацпроекте «Производительность труда» — торты пекут вдвое быстрее, выработка на человека +27%. Сигнал для ИТ: не на открытие сети, а на то, что режет издержки (самообслуживание, бережливое производство). Большой «бюджет на цифровизацию» не обещали. https://www.retail.ru/articles/kak-rosli-riteylery-v-2025-godu-ekspansiya-optimizatsiya-i-znachimye-resheniya-vedushchikh-setey/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="73" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 12,87 млрд рублей, почти как годом раньше (на 1% больше). После расходов осталось всего 65 миллионов — полкопейки с рубля. На начало 2026: 74 магазина, закрытий не было. В 2025 новые точки почти не открывали: смотрели эффективность, аренду, тарифы. Запустили SPAR-Express и кассы, где покупатель бьёт товар сам. В июле 2026 участвовали в нацпроекте «Производительность труда»: торты пекут вдвое быстрее, один человек делает на 27% больше. Для ИТ это значит: деньги не на новые магазины, а на то, что снижает расходы. Большого «тратим на программы» не обещали. https://www.retail.ru/articles/kak-rosli-riteylery-v-2025-godu-ekspansiya-optimizatsiya-i-znachimye-resheniya-vedushchikh-setey/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1" s="6">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Низкоцен (ООО Холлифуд)</t>
@@ -6279,11 +6279,11 @@
       </c>
       <c r="J9" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 9,5 млрд (−2%), прибыль 61 млн, маржа 0,6 копейки с рубля. На сайте 71 магазин, новые объекты ищут. Сигнал для ИТ: осторожно. Продажи уже не росли, маржа тонкая. Скорее заморозка лишнего, чем новая платформа. Своего плана на 2026 нет. https://ksonline.ru/605083/skolko-zarabotali-krupnye-sibirskie-produktovye-seti-v-2025-godu/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 9,5 млрд рублей, на 2% меньше, чем годом раньше. После расходов осталось 61 миллион — 0,6 копейки с рубля. На сайте 71 магазин, новые помещения ищут. Для ИТ это значит: осторожно. Продажи уже не росли, прибыли мало. Скорее заморозят лишнее, чем купят новую платформу. Своего плана на 2026 нет. https://ksonline.ru/605083/skolko-zarabotali-krupnye-sibirskie-produktovye-seti-v-2025-godu/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="73" customHeight="1" s="6">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>OFFPRICE (ООО Оффпрайс)</t>
@@ -6329,11 +6329,11 @@
       </c>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>Это не продукты. Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 4,85 млрд (+1,8%), прибыль 0,113 млрд, маржа 2,3 копейки с рубля. На сайте «30+ аутлетов»; вы называли 40. Рост почти остановился. Сигнал для ИТ: слабый рост, не FMCG. Большого «режем / строим» в открытом виде нет. https://firmoteka.ru/7725844967</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="76" customHeight="1" s="6">
+          <t>Это одежда, не продукты. За 2026 продаж нет. Что есть — весь 2025: 4,85 млрд рублей, на 1,8% больше, чем годом раньше. После расходов осталось 113 миллионов — 2,3 копейки с рубля. На сайте «30+ аутлетов»; вы называли 40. Рост почти остановился. Для ИТ это значит: слабый рост, и это не продуктовая сеть. Ни «режем», ни «строим» в открытом виде не видно. https://firmoteka.ru/7725844967</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="79" customHeight="1" s="6">
       <c r="A11" s="18" t="inlineStr">
         <is>
           <t>КЗВС (вет. аптеки, Краснодарский край)</t>
@@ -6379,11 +6379,11 @@
       </c>
       <c r="J11" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — ООО «КЗВС» весь 2025: 1,13 млрд (+2,6%), прибыль 0,108 млрд, маржа почти 10 копеек с рубля — для розницы жирно. На сайте 200 вет. аптек, в штате юрлица 92 человека: часть точек, скорее всего, партнёры. Сигнал для ИТ: маржа позволяет не резать всё подряд, но это одно юрлицо, не холдинг. Своего плана «в 2026 откроем столько-то» не нашли. https://www.testfirm.ru/result/2312208833_ooo-kzvs</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="74" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — ООО «КЗВС» за весь 2025: 1,13 млрд рублей, на 2,6% больше, чем годом раньше. После расходов осталось 108 миллионов — почти 10 копеек с рубля, для розницы это много. На сайте 200 вет. аптек, в штате этой компании 92 человека: часть точек, скорее всего, партнёры. Для ИТ это значит: прибыль позволяет не резать всё подряд, но это одна компания, не большая группа. Плана «в 2026 откроем столько-то» не нашли. https://www.testfirm.ru/result/2312208833_ooo-kzvs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1" s="6">
       <c r="A12" s="18" t="inlineStr">
         <is>
           <t>АО «Иркутская аптека»</t>
@@ -6429,14 +6429,14 @@
       </c>
       <c r="J12" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 1,1 млрд (−2%), убыток 4,5 млн. На 1 января 2026 — 43 точки (вы называли 44). Городская сеть, в 2025-м из МУП сделали АО. Сигнал для ИТ на 2026–27: скорее заморозка и обязательные госсистемы, чем новая коммерческая платформа. Убыток и муниципальный хозяин — плохой фон для лишних проектов. https://ircity.ru/text/business/2026/09/07/76621885/</t>
+          <t>За 2026 продаж нет. Что есть — весь 2025: 1,1 млрд рублей, на 2% меньше, чем годом раньше. После расходов минус 4,5 миллиона — сеть в убытке. На 1 января 2026 — 43 точки (вы называли 44). Это городская сеть: в 2025-м из муниципального предприятия сделали акционерное общество. Для ИТ на 2026–27 это значит: скорее заморозка и обязательные государственные системы, чем новая коммерческая программа. Убыток и город как хозяин — плохой фон для лишних проектов. https://ircity.ru/text/business/2026/09/07/76621885/</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1" s="6">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Заводы поменьше: 2026 почти не раскрывают, смотрим стройки и прибыль 2025</t>
+          <t>Заводы поменьше: продаж за 2026 почти нет, смотрим стройки и прибыль 2025</t>
         </is>
       </c>
       <c r="B13" s="17" t="n"/>
@@ -6449,7 +6449,7 @@
       <c r="I13" s="17" t="n"/>
       <c r="J13" s="17" t="n"/>
     </row>
-    <row r="14" ht="79" customHeight="1" s="6">
+    <row r="14" ht="81" customHeight="1" s="6">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Любятово (ООО; ГК Черноголовка)</t>
@@ -6495,11 +6495,11 @@
       </c>
       <c r="J14" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 13,2 млрд (+25%), прибыль 0,847 млрд, маржа 6,4 копейки с рубля. Площадки: Воронеж, Псков, Вязьма. Февраль 2026: в Воронеже обсуждали производственно-складской комплекс, в прессе оценка около 4 млрд. Сентябрь 2026: в Вязьме — новые линии и склад на 2026–2027. Сигнал для ИТ: капекс точно не режут. Заводу, который строит корпус и склад, учёт и линии будут нужны. Это не прогноз выручки на год. https://www.kommersant.ru/doc/8476994</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="78" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 13,2 млрд рублей, на 25% больше, чем годом раньше. После расходов осталось 847 миллионов — 6,4 копейки с рубля. Площадки: Воронеж, Псков, Вязьма. В феврале 2026 в Воронеже обсуждали новый производственно-складской комплекс, в прессе оценка около 4 млрд. В сентябре 2026 в Вязьме — новые линии и склад на 2026–2027. Для ИТ это значит: стройки не режут. Заводу, который ставит корпус и склад, учёт и линии будут нужны. Это не прогноз продаж на год. https://www.kommersant.ru/doc/8476994</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="82" customHeight="1" s="6">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Иркутский масложиркомбинат</t>
@@ -6545,11 +6545,11 @@
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 16,35 млрд (−0,9%), прибыль 2,33 млрд. Маржа 14 копеек с рубля, но заметная часть — проценты по деньгам на счетах, не от продажи масла. Агентство INFOLine, сентябрь 2026: у крупных производителей еды рост «около нуля» — это рынок, не этот завод. Сигнал для ИТ: денег после 2025 много, своего плана строек на 2026 не нашли. Не «режим порезок», но и не анонс цифры. https://finscanner.ru/company/3811185573/finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="68" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 16,35 млрд рублей, почти как годом раньше (на 0,9% меньше). После расходов осталось 2,33 млрд. Это 14 копеек с рубля, но заметная часть — проценты по деньгам на счетах, не от продажи масла. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не этот завод. Для ИТ это значит: денег после 2025 много, своего плана строек на 2026 не нашли. Не похоже на режим порезок, но и анонса «тратим на программы» нет. https://finscanner.ru/company/3811185573/finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1" s="6">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Каравай (ОАО, Санкт-Петербург)</t>
@@ -6595,11 +6595,11 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 11,12 млрд (+15%), прибыль 0,709 млрд, маржа 6,4 копейки с рубля. Не путать с ангарским «Караваем». Сигнал для ИТ: 2025 прибыльный. Своего плана на 2026 нет. По рынку заводов рост около нуля. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="67" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 11,12 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 709 миллионов — 6,4 копейки с рубля. Есть ещё ангарский «Каравай» — это другая компания, сюда не относится. Для ИТ это значит: 2025 был прибыльным. Своего плана на 2026 нет. По рынку заводов рост около нуля. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="69" customHeight="1" s="6">
       <c r="A17" s="18" t="inlineStr">
         <is>
           <t>СМАК (АО, Екатеринбург)</t>
@@ -6645,11 +6645,11 @@
       </c>
       <c r="J17" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 9,79 млрд (+18%), прибыль 1,11 млрд, маржа 11 копеек с рубля. Три площадки, включая Раменское. Сигнал для ИТ: маржа высокая, 2025 сильный. Своего «в 2026 продадим на столько-то» нет. https://www.smakhleb.ru/predpriyatie</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="70" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 9,79 млрд рублей, на 18% больше, чем годом раньше. После расходов осталось 1,11 млрд — 11 копеек с рубля. Три площадки, включая Раменское. Для ИТ это значит: прибыль высокая, 2025 сильный. Своего «в 2026 продадим на столько-то» нет. https://www.smakhleb.ru/predpriyatie</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1" s="6">
       <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Лимак (АО, Липецк)</t>
@@ -6695,11 +6695,11 @@
       </c>
       <c r="J18" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 8,93 млрд (+8%), прибыль 0,22 млрд, маржа 2,5 копейки с рубля — для хлеба скромно. Девять хлебозаводов плюс мельница. Сигнал для ИТ: сеть площадок живая, но маржа тонкая. Лишнего ИТ без окупаемости, скорее всего, не купят. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="66" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 8,93 млрд рублей, на 8% больше, чем годом раньше. После расходов осталось 220 миллионов — 2,5 копейки с рубля, для хлеба скромно. Девять хлебозаводов плюс мельница. Для ИТ это значит: площадки живые, но прибыли мало. Лишний софт без понятной экономии, скорее всего, не купят. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="67" customHeight="1" s="6">
       <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Первый хлебокомбинат (АО, Челябинск)</t>
@@ -6747,11 +6747,11 @@
       </c>
       <c r="J19" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 8,00 млрд (+10%), прибыль 1,16 млрд, маржа 14,5 копейки с рубля. Сколько площадок — не нашли. Сигнал для ИТ: прибыль 2025 большая, плана 2026 нет. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="73" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 8,00 млрд рублей, на 10% больше, чем годом раньше. После расходов осталось 1,16 млрд — 14,5 копейки с рубля. Сколько площадок — не нашли. Для ИТ это значит: прибыль 2025 большая, плана на 2026 нет. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="75" customHeight="1" s="6">
       <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Вологодское мороженое (ООО)</t>
@@ -6797,11 +6797,11 @@
       </c>
       <c r="J20" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 6,63 млрд (−7%), прибыль 2,78 млрд, маржа 42 копейки с рубля — для мороженого необычно много, причину компания не объясняла. Сигнал для ИТ: продажи падали, прибыль огромная. На «режем ИТ из-за дыры» не похоже, на «строим новую цифру» тоже ничего не анонсировали. https://nalogovaya.ru/egrul/companies/1033500071505/</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="66" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 6,63 млрд рублей, на 7% меньше, чем годом раньше. После расходов осталось 2,78 млрд — 42 копейки с рубля. Для мороженого это необычно много, причину компания не объясняла. Для ИТ это значит: продажи падали, но дыры в деньгах нет. На «режем ИТ из-за убытка» не похоже, на «строим новую систему» тоже ничего не анонсировали. https://nalogovaya.ru/egrul/companies/1033500071505/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="68" customHeight="1" s="6">
       <c r="A21" s="18" t="inlineStr">
         <is>
           <t>Покровский хлеб (АО, Пермь)</t>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="J21" s="19" t="inlineStr">
         <is>
-          <t>Выручки за кусок 2026 нет. Последний закрытый год — весь 2025: 5,5 млрд (+17%), прибыль 0,82 млрд, маржа почти 15 копеек с рубля. Три пермских завода. Сигнал для ИТ: 2025 сильный. Своего плана капекса на 2026–27 не нашли. https://www.kommersant.ru/doc/8552543</t>
+          <t>За 2026 продаж нет. Что есть — весь 2025: 5,5 млрд рублей, на 17% больше, чем годом раньше. После расходов осталось 820 миллионов — почти 15 копеек с рубля. Три завода в Перми. Для ИТ это значит: 2025 сильный. Своего плана строек на 2026–27 не нашли. https://www.kommersant.ru/doc/8552543</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       <c r="I22" s="17" t="n"/>
       <c r="J22" s="17" t="n"/>
     </row>
-    <row r="23" ht="76" customHeight="1" s="6">
+    <row r="23" ht="80" customHeight="1" s="6">
       <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Дружба (Рыбинск, Ярославская область)</t>
@@ -6913,11 +6913,11 @@
       </c>
       <c r="J23" s="19" t="inlineStr">
         <is>
-          <t>Сводной выручки сети нет — ни за 2026, ни за 2025. Сайт: 28 точек, 12 500 м², 1 700 человек. Юрлицо ООО «Дружба» (66 млн и 14 человек) — не эта сеть, в таблицу не ставили. Июнь 2026: закрывают гипермаркет в ТЦ «Космос» (работал ~15 лет), дата около 20 июля. Сигнал для ИТ: сжимаются, не расширяются. Новый дорогой софт на этом фоне маловероятен. https://ngs76.ru/gorod/v-rybinske-zakroetsya-gipermarket-druzhba-magazin-prorabotal-15-let-id341441/</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="72" customHeight="1" s="6">
+          <t>Сводных продаж сети нет — ни за 2026, ни за 2025. Сайт: 28 точек, 12 500 квадратных метров, 1 700 человек. Есть ООО «Дружба» с 66 миллионами выручки и 14 людьми — это не эта сеть, в таблицу не ставили. В июне 2026 объявили, что закрывают гипермаркет в ТЦ «Космос» (работал около 15 лет), дата около 20 июля. Для ИТ это значит: сеть сжимается, не расширяется. Новый дорогой софт на этом фоне маловероятен. https://ngs76.ru/gorod/v-rybinske-zakroetsya-gipermarket-druzhba-magazin-prorabotal-15-let-id341441/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="71" customHeight="1" s="6">
       <c r="A24" s="18" t="inlineStr">
         <is>
           <t>Ёвар (Таджикистан)</t>
@@ -6963,7 +6963,7 @@
       </c>
       <c r="J24" s="19" t="inlineStr">
         <is>
-          <t>Выручки в открытом виде нет. Октябрь 2025: сеть писала про 30 супермаркетов и новый зал в City Mall. Вы называли 62 — 62 в открытых текстах не подтвердили. Сигнал для ИТ: по словам самой сети — расширение географии, не сжатие. Суммы и ИТ-бюджет неизвестны. https://koinotinav.tj/news/set-supermarketov-evar-ukreplyaet-pozicii-i-rasshiryaet-geografiyu-prisutstviya</t>
+          <t>Открытых цифр продаж нет. В октябре 2025 сеть писала про 30 супермаркетов и новый зал в City Mall. Вы называли 62 — в открытых текстах 62 не нашли. Для ИТ это значит: по словам самой сети — расширение, не сжатие. Суммы и бюджет ИТ неизвестны. https://koinotinav.tj/news/set-supermarketov-evar-ukreplyaet-pozicii-i-rasshiryaet-geografiyu-prisutstviya</t>
         </is>
       </c>
     </row>
@@ -7013,7 +7013,7 @@
       </c>
       <c r="J25" s="19" t="inlineStr">
         <is>
-          <t>62 точки — как вы указали. Открытой выручки нет. Попадаются «Fayz» и «Kredit Fayz» (техника) — это не обязательно та же сеть, деньги не ставили. Сигнал для ИТ: по открытым источникам ничего; ни «режем», ни «строим» подтвердить нельзя.</t>
+          <t>62 точки — как вы указали. Открытых продаж нет. Попадаются «Fayz» и «Kredit Fayz» (техника) — это не обязательно та же сеть, деньги не ставили. Для ИТ по открытым источникам ничего не видно: ни «режем», ни «строим» подтвердить нельзя.</t>
         </is>
       </c>
     </row>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>Года ещё нет (сейчас октябрь 2026), полного отчёта за весь 2026 ни у кого нет. В столбце «факт» — уже опубликованный кусок: девять месяцев, полгода или квартал. «Оценка года» — не отчёт, а арифметика: либо прогноз самой компании, либо выручка 2025, умноженная на рост уже вышедшего куска 2026. Где куска нет — «нет данных», ничего не додумано. Прибыль и маржа стоят только там, где компания сама их опубликовала за тот же кусок года.</t>
+          <t>Года ещё нет (сейчас октябрь 2026), полного отчёта за весь 2026 ни у кого нет. В столбце «факт» — уже опубликованный период: девять месяцев, полгода или квартал. «Оценка года» — не отчёт, а арифметика: либо прогноз самой компании, либо продажи 2025, умноженные на рост уже вышедшего периода 2026. Где периода нет — «нет данных», ничего не додумано. Прибыль и маржа стоят только там, где компания сама их опубликовала за тот же период.</t>
         </is>
       </c>
       <c r="C2" s="16" t="inlineStr">
@@ -7087,7 +7087,7 @@
       </c>
       <c r="B3" s="15" t="inlineStr">
         <is>
-          <t>Продали за январь–сентябрь на 3,79 триллиона рублей, на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь быстрее полугодия: +13% до 1,31 триллиона. Чижик по-прежнему самый быстрый внутри группы (+31% за девять месяцев, +35% за квартал). Компания свой прогноз на весь год не снимала: +12–16%.</t>
+          <t>Продали за январь–сентябрь на 3,79 триллиона рублей, на 11,4% больше, чем за те же девять месяцев 2025-го. Июль–сентябрь быстрее полугодия: на 13% больше, до 1,31 триллиона. Чижик по-прежнему самый быстрый внутри группы (на 31% больше за девять месяцев, на 35% больше за квартал). Компания свой прогноз на весь год не меняла: плюс 12–16%.</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>В марте и снова в июне президент Екатерина Лобачева: прогноз роста выручки 12–16% на 2026 держим. От выручки 2025 (4,642 триллиона) это примерно 5,20–5,39 триллиона за полный год. Девять месяцев идут ближе к нижней границе.</t>
+          <t>В марте и снова в июне президент Екатерина Лобачева: прогноз роста продаж 12–16% на 2026 держим. От продаж 2025 (4,642 триллиона) это примерно 5,20–5,39 триллиона за полный год. Девять месяцев идут ближе к нижней границе.</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
@@ -7129,7 +7129,7 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>1 887 млрд рублей за полгода, +12,8%. Магазины работают, продажи растут, по прибыли группа всё ещё в минусе: −1,9 млрд (без правила «аренда как долг»). Если аренду магазинов считать долгом, минус около −9,5. Мешают проценты по кредитам. Это тот же сюжет, что в 2025: полка живая, кредиты тяжёлые.</t>
+          <t>1 887 млрд рублей за полгода, на 12,8% больше, чем годом раньше. Магазины работают, продажи растут, по прибыли группа всё ещё в минусе: −1,9 млрд (без правила «аренда как долг»). Если аренду магазинов считать долгом, минус около −9,5. Мешают проценты по кредитам. Это тот же сюжет, что в 2025: полка живая, кредиты тяжёлые.</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Официальную прибыль за январь–июнь 2026 опубликовали шесть сетей и четыре завода. Сети: X5 25,7 млрд (маржа 1% — от продаж за январь–июнь 2 481, не от девяти месяцев), Магнит −1,9, Лента 13 (2%), Fix Price 2,7 (1,8%), «ДА!» 1,2 (2,8%), Винлаб 0,79 (1,5%). Заводы: Черкизово 14,1 (почти 10 копеек с рубля), Русагро почти ноль (0,056), Агроэко 1,99 (8,1%), ЭкоНива 1,1 (2,4% от всей группы). У остальных в этих столбцах «нет данных»: отчёта с прибылью за 2026 ещё нет. Мираторг писал прибыль 19,61 без полной выручки — в ячейку не ставили, маржу от этого не посчитать.</t>
+          <t>Официальную прибыль за январь–июнь 2026 опубликовали шесть сетей и четыре завода. Сети: X5 25,7 млрд (1% — от продаж за январь–июнь 2 481, не от девяти месяцев), Магнит −1,9, Лента 13 (2%), Fix Price 2,7 (1,8%), «ДА!» 1,2 (2,8%), Винлаб 0,79 (1,5%). Заводы: Черкизово 14,1 (почти 10 копеек с рубля), Русагро почти ноль (0,056), Агроэко 1,99 (8,1%), ЭкоНива 1,1 (2,4% от всей группы). У остальных в этих столбцах «нет данных»: отчёта с прибылью за 2026 ещё нет. Мираторг писал прибыль 19,61 без полных продаж — в ячейку не ставили, долю от этого не посчитать.</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
@@ -7171,7 +7171,7 @@
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Агентство INFOLine сложила десятку: 6,76 триллиона рублей, +11,6% (годом раньше десятка росла на 17%). Лента +26% — самый быстрый из крупных. Светофор и Ашан продали меньше, чем год назад. На весь 2026 агентство ждёт рост крупнейших сетей примерно 9–11%.</t>
+          <t>Агентство INFOLine сложила десятку: 6,76 триллиона рублей, на 11,6% больше (годом раньше десятка росла на 17%). Лента — на 26% больше, самый быстрый из крупных. Светофор и Ашан продали меньше, чем год назад. На весь 2026 агентство ждёт рост крупнейших сетей примерно 9–11%.</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>648 млрд рублей за полгода, +26%. Тянут «Супер Лента» и «Монетка». В августе купила большие магазины «О’КЕЙ» — со второго полугодия в цифрах будут ещё и эти магазины.</t>
+          <t>648 млрд рублей за полгода, на 26% больше, чем годом раньше. Тянут «Супер Лента» и «Монетка». В августе купила большие магазины «О’КЕЙ» — со второго полугодия в цифрах будут ещё и эти магазины.</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
@@ -7213,7 +7213,7 @@
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>155 млрд рублей, +4,8%. Медленнее больших продуктовых сетей: цены фиксированные, в ассортименте не только еда.</t>
+          <t>155 млрд рублей, на 4,8% больше, чем годом раньше. Медленнее больших продуктовых сетей: цены фиксированные, в ассортименте не только еда.</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>51 млрд рублей по официальному отчёту, +7%. Отдельно компания хвалится продажами с налогом за девять месяцев (+24%) — это отскок после кибератаки 2025-го, не путать с выручкой в таблице.</t>
+          <t>51 млрд рублей по официальному отчёту, на 7% больше, чем годом раньше. Отдельно компания хвалится продажами с налогом за девять месяцев (на 24% больше) — это отскок после кибератаки 2025-го, не те продажи, что в таблице.</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
@@ -7255,7 +7255,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>183 млрд рублей, +9%. Догнать PepsiCo по году ещё рано: полного 2026 нет ни у кого из заводов.</t>
+          <t>183 млрд рублей, на 9% больше, чем годом раньше. Догнать PepsiCo по году ещё рано: полного 2026 нет ни у кого из заводов.</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
@@ -7276,7 +7276,7 @@
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>142 млрд рублей, всего +3,5%. Слабее роста цен в магазинах: дешевле свинина и меньше продаж в Китай.</t>
+          <t>142 млрд рублей, всего на 3,5% больше, чем годом раньше. Слабее роста цен в магазинах: дешевле свинина и меньше продаж в Китай.</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
@@ -7297,7 +7297,7 @@
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>46 млрд рублей, +19% — один из немногих заводов, у кого продажи выросли сильно.</t>
+          <t>46 млрд рублей, на 19% больше, чем годом раньше — один из немногих заводов, у кого продажи выросли сильно.</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
@@ -7318,7 +7318,7 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Выручку за 2026 пока не раскрыли. Глава группы в июне: ждать роста «на несколько процентов», продажи за границу удержать около 58 млрд рублей.</t>
+          <t>Продажи за 2026 пока не раскрыли. Глава группы в июне: ждать роста «на несколько процентов», продажи за границу удержать около 58 млрд рублей.</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
@@ -7339,7 +7339,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>По большинству сетей из регионов и заводов своего прогноза «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год +9–11%; крупные производители еды почти без роста), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку выручки это не ставили — это не продажи компании. Регионы меньшего масштаба и сигнал «режут ли ИТ» — на листе «Регионы».</t>
+          <t>По большинству сетей из регионов и заводов своего плана «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год плюс 9–11%; крупные производители еды почти без роста), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку продаж это не ставили — это не продажи компании. Сети поменьше и то, режут ли они ИТ, — на листе «Регионы».</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
@@ -7355,12 +7355,12 @@
     <row r="16" ht="72" customHeight="1" s="6">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Регионы меньшего масштаба — 2026 и ИТ</t>
+          <t>Регионы поменьше — 2026 и ИТ</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>У сетей на 30–200 точек своего отчёта за кусок 2026 почти нет. На листе «Регионы» те же десять колонок, что у крупных. В деньгах за 2026 чаще «нет данных». В комментарии — последний закрытый 2025 и что видно на 2026–27: открывают, склеивают сети, режут издержки или закрывают магазин. Это не «бюджет ИТ в рублях», такого никто не публикует.</t>
+          <t>У сетей на 30–200 точек своего отчёта за период 2026 почти нет. На листе «Регионы» те же десять колонок, что у крупных. В деньгах за 2026 чаще «нет данных». В комментарии — закрытый 2025 и что видно на 2026–27: открывают, склеивают сети, режут расходы или закрывают магазин. Это не «бюджет ИТ в рублях», такого никто не публикует.</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
@@ -7381,7 +7381,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>Агентство INFOLine: у крупнейших сетей за год до июня 2026 точек стало больше только на 4,9% (годом раньше было +10,8%). Новый магазин дороже на 8–12%. Часть денег уходит в доставку и цифру. Это фон рынка, не строка «Семишагофф».</t>
+          <t>Агентство INFOLine: у крупнейших сетей за год до июня 2026 точек стало больше только на 4,9% (годом раньше было на 10,8% больше). Новый магазин дороже на 8–12%. Часть денег уходит в доставку и программы. Это фон рынка, не строка «Семишагофф».</t>
         </is>
       </c>
       <c r="C17" s="16" t="inlineStr">
@@ -7397,12 +7397,12 @@
     <row r="18" ht="72" customHeight="1" s="6">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>SPAR Калининград — не путать юрлица</t>
+          <t>SPAR Калининград — две разные компании</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Операционная компания ООО «Евроритейл»: за 2025 продали на 32,7 млрд (+15%), прибыль 0,56 млрд. ООО «Спар-Калининград» — другое юрлицо, 54 млн выручки: это не магазины. Директор сети в июне 2025: 105 магазинов.</t>
+          <t>Магазины — это ООО «Евроритейл»: за 2025 продали на 32,7 млрд, на 15% больше, чем годом раньше, прибыль 0,56 млрд. ООО «Спар-Калининград» — другая компания, 54 млн продаж: это не магазины. Директор сети в июне 2025: 105 магазинов.</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>«Континент Сибирь» разобрал российские отчёты: «Лама» — сумма четырёх магазинных юрлиц 32,3 млрд, «Аникс» отдельно, «Бегемаг» 13 млрд при прибыли всего 65 млн, «Низкоцен» 9,5 млрд. Управляющую компанию «Лама» (134 млн) с магазинами складывать нельзя.</t>
+          <t>«Континент Сибирь» разобрал российские отчёты: «Лама» — сумма четырёх магазинных компаний 32,3 млрд, «Аникс» отдельно, «Бегемаг» 13 млрд при прибыли всего 65 млн, «Низкоцен» 9,5 млрд. Управляющую компанию «Лама» (134 млн) с магазинами складывать нельзя.</t>
         </is>
       </c>
       <c r="C19" s="16" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (за январь–июнь десятка уже +11,6%, годом раньше было +17%). Это прогноз десятки, не «Мария-Ра» и не «Командор».</t>
+          <t>После полугодия агентство ждало рост крупнейших продуктовых сетей примерно 9–11% за полный год (за январь–июнь десятка уже на 11,6% больше, годом раньше было на 17% больше). Это прогноз десятки, не «Мария-Ра» и не «Командор».</t>
         </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
@@ -7461,7 +7461,7 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже +0,4%, в 2026 рост лидеров «приблизился к нулю». KDV как пример: уже 2025 только +1%.</t>
+          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже плюс 0,4%, в 2026 рост лидеров «приблизился к нулю». KDV как пример: уже 2025 только на 1% больше.</t>
         </is>
       </c>
       <c r="C21" s="16" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>В январе агентство Data Insight заложило всю доставку продуктов в России на 1,8 триллиона рублей за 2026 (+24%). К марту 1,83 триллиона (+22%), к маю 1,84. Это весь рынок вместе с налогом и платой за доставку, не выручка одной Лавки или Ozon Fresh.</t>
+          <t>В январе агентство Data Insight заложило всю доставку продуктов в России на 1,8 триллиона рублей за 2026 (на 24% больше). К марту 1,83 триллиона (на 22% больше), к маю 1,84. Это весь рынок вместе с налогом и платой за доставку, не продажи одной Лавки или Ozon Fresh.</t>
         </is>
       </c>
       <c r="C22" s="16" t="inlineStr">
@@ -7495,7 +7495,7 @@
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>«Верный» с октября 2025 ищут покупателя (оценка 25–35 млрд — цена всего бизнеса). «Гулливер» в начале 2026 писали как выставленный на продажу. Про «Мария-Ра» летом 2026 писали, что смотрит «Лента». Цифры выручки на 2026 никто из них не давал.</t>
+          <t>«Верный» с октября 2025 ищут покупателя (оценка 25–35 млрд — цена всего бизнеса). «Гулливер» в начале 2026 писали как выставленный на продажу. Про «Мария-Ра» летом 2026 писали, что смотрит «Лента». Цифры продаж на 2026 никто из них не давал.</t>
         </is>
       </c>
       <c r="C23" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Explain why SPAR-Kaliningrad is not the store chain
The 54 million and two staff belong to a trademark-licensing company,
not Euroretail's 100 stores. Say that in the note so the headcount is
a reason to ignore the row, not a fact about SPAR.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -5983,7 +5983,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="98" customHeight="1" s="6">
+    <row r="4" ht="107" customHeight="1" s="6">
       <c r="A4" s="18" t="inlineStr">
         <is>
           <t>SPAR Калининград (ООО Евроритейл)</t>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="J4" s="19" t="inlineStr">
         <is>
-          <t>За 2026 продаж компания не публиковала. Что есть — весь 2025 у ООО «Евроритейл»: 32,68 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 563 миллиона — это 1,7 копейки с каждого рубля. Рядом есть другое ООО — «Спар-Калининград»: 54 миллиона выручки и двое сотрудников. Это не магазины, их цифры сюда не относятся. В апреле 2026 замгендиректора сказал: магазинов уже больше ста. «Пятёрочка» в области около двухсот — по числу точек и по цене с ней не соревнуются. За 2025 открыли шесть магазинов. Директор раньше говорила: каждый год плюс десять новых и 20–25 ремонтов старых. Электронные ценники уже стоят. Для ИТ это значит: сеть живая, не сворачивается. Деньги скорее на ремонт магазинов, ценники и доставку через паром, чем на то, чтобы догнать «Пятёрочку». https://kaliningrad-news.net/society/2026/04/17/281609.html</t>
+          <t>За 2026 продаж компания не публиковала. Что есть — весь 2025 у ООО «Евроритейл»: 32,68 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 563 миллиона — это 1,7 копейки с каждого рубля. Есть ещё фирма с похожим именем — ООО «Спар-Калининград». Это не магазины: она сдаёт в аренду товарные знаки и за 2025 показала 54 миллиона продаж. В налоговой у неё в штате в среднем двое людей. У сети SPAR больше ста магазинов — такие цифры к ней не относятся, в таблицу их не ставили. В апреле 2026 замгендиректора сказал: магазинов уже больше ста. «Пятёрочка» в области около двухсот — по числу точек и по цене с ней не соревнуются. За 2025 открыли шесть магазинов. Директор раньше говорила: каждый год плюс десять новых и 20–25 ремонтов старых. Электронные ценники уже стоят. Для ИТ это значит: сеть живая, не сворачивается. Деньги скорее на ремонт магазинов, ценники и доставку через паром, чем на то, чтобы догнать «Пятёрочку». https://kaliningrad-news.net/society/2026/04/17/281609.html</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6867,7 @@
       <c r="I22" s="17" t="n"/>
       <c r="J22" s="17" t="n"/>
     </row>
-    <row r="23" ht="80" customHeight="1" s="6">
+    <row r="23" ht="83" customHeight="1" s="6">
       <c r="A23" s="18" t="inlineStr">
         <is>
           <t>Дружба (Рыбинск, Ярославская область)</t>
@@ -6913,7 +6913,7 @@
       </c>
       <c r="J23" s="19" t="inlineStr">
         <is>
-          <t>Сводных продаж сети нет — ни за 2026, ни за 2025. Сайт: 28 точек, 12 500 квадратных метров, 1 700 человек. Есть ООО «Дружба» с 66 миллионами выручки и 14 людьми — это не эта сеть, в таблицу не ставили. В июне 2026 объявили, что закрывают гипермаркет в ТЦ «Космос» (работал около 15 лет), дата около 20 июля. Для ИТ это значит: сеть сжимается, не расширяется. Новый дорогой софт на этом фоне маловероятен. https://ngs76.ru/gorod/v-rybinske-zakroetsya-gipermarket-druzhba-magazin-prorabotal-15-let-id341441/</t>
+          <t>Сводных продаж сети нет — ни за 2026, ни за 2025. Сайт: 28 точек, 12 500 квадратных метров, 1 700 человек. Есть ООО «Дружба» с 66 миллионами продаж и 14 людьми в налоговой. На сайте сети — 28 магазинов и 1 700 человек. Это разные фирмы, 66 миллионов в таблицу не ставили. В июне 2026 объявили, что закрывают гипермаркет в ТЦ «Космос» (работал около 15 лет), дата около 20 июля. Для ИТ это значит: сеть сжимается, не расширяется. Новый дорогой софт на этом фоне маловероятен. https://ngs76.ru/gorod/v-rybinske-zakroetsya-gipermarket-druzhba-magazin-prorabotal-15-let-id341441/</t>
         </is>
       </c>
     </row>
@@ -7402,12 +7402,12 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Магазины — это ООО «Евроритейл»: за 2025 продали на 32,7 млрд, на 15% больше, чем годом раньше, прибыль 0,56 млрд. ООО «Спар-Калининград» — другая компания, 54 млн продаж: это не магазины. Директор сети в июне 2025: 105 магазинов.</t>
+          <t>Магазины — это ООО «Евроритейл»: за 2025 продали на 32,7 млрд, на 15% больше, чем годом раньше, прибыль 0,56 млрд. ООО «Спар-Калининград» — другая фирма: сдаёт в аренду товарные знаки, 54 млн продаж и двое в штате по налоговой. Это не сто магазинов SPAR. Директор сети в июне 2025: 105 магазинов.</t>
         </is>
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>https://firmoteka.ru/3906321175</t>
+          <t>https://checko.ru/company/spar-kaliningrad-1133926040819</t>
         </is>
       </c>
       <c r="D18" s="12" t="n"/>

</xml_diff>

<commit_message>
Tighten Aniks note: grocery yes, IT spend unknown
Keep 2025 sales and profit. Drop the claim that the chain is not
cutting costs — that did not follow from a thin grocery margin.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -6083,7 +6083,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="79" customHeight="1" s="6">
+    <row r="6" ht="97" customHeight="1" s="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Аникс (ТС Аникс + Прайд-А)</t>
@@ -6091,7 +6091,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>у дома, Алтай</t>
+          <t>продукты у дома, Алтай</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="J6" s="19" t="inlineStr">
         <is>
-          <t>За 2026 продаж нет. Что есть — две компании за 2025: 18,3 + 13,0 = 31,3 млрд рублей. После расходов осталось 414 миллионов — 1,3 копейки с рубля. Своих магазинов 165, ещё 109 работают как франшиза «Корзинка». В 2025 прибыль выросла. Плана продаж на 2026 не публиковали. Для ИТ это значит: сеть живая и с прибылью, не экономит на всём. Но сколько именно тратят на ИТ — никто не говорит. https://tolknews.ru/ekonomika/214569-skolko-zarabotali-krupneyshie-seti-altaya-mariya-ra-i-aniks-v-godu</t>
+          <t>Да, продукты: магазины у дома в Алтайском крае, Республике Алтай и Новосибирской области. За 2026 продаж нет. Что есть — две компании за 2025. ООО «ТС Аникс» (сами магазины): 18,3 млрд, на 10% больше, чем годом раньше, прибыль 305 млн. ООО «Прайд-А» (опт продуктов на ту же сеть): 13,0 млрд, на 10% больше, прибыль 109 млн. Вместе 31,3 млрд и 414 млн — 1,3 копейки с рубля, для продуктов обычно. Местная пресса в апреле 2026: прибыль выросла больше чем на 70 млн, «повысили эффективность». Своих магазинов 165, ещё франшиза «Корзинка». Плана продаж на 2026 нет. Для ИТ это значит: по закрытому 2025 сеть не в убытке и продажи росли. Из этого не следует, что «не экономят»: сколько тратят на ИТ, никто не публиковал. https://tolknews.ru/ekonomika/214569-skolko-zarabotali-krupneyshie-seti-altaya-mariya-ra-i-aniks-v-godu</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separate OFFPRICE margin from stalled sales growth
2.3 kopecks per ruble is profit share, not expansion. Spell out that
2025 sales grew only 1.8% and profit fell 15%, and that store openings
were not the claim.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -6283,7 +6283,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="73" customHeight="1" s="6">
+    <row r="10" ht="89" customHeight="1" s="6">
       <c r="A10" s="18" t="inlineStr">
         <is>
           <t>OFFPRICE (ООО Оффпрайс)</t>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>Это одежда, не продукты. За 2026 продаж нет. Что есть — весь 2025: 4,85 млрд рублей, на 1,8% больше, чем годом раньше. После расходов осталось 113 миллионов — 2,3 копейки с рубля. На сайте «30+ аутлетов»; вы называли 40. Рост почти остановился. Для ИТ это значит: слабый рост, и это не продуктовая сеть. Ни «режем», ни «строим» в открытом виде не видно. https://firmoteka.ru/7725844967</t>
+          <t>Это одежда, не продукты. За 2026 продаж нет. Что есть — весь 2025: 4,85 млрд рублей, всего на 1,8% больше, чем годом раньше — продажи почти не выросли. После расходов осталось 113 миллионов — 2,3 копейки с рубля. Для розницы это хорошо (у продуктов обычно около одной копейки), противоречия тут нет: с каждого рубля оставляют нормально, но сам оборот почти не растёт. Прибыль даже чуть села: на 15% меньше, чем в 2024-м. На сайте «30+ аутлетов»; вы называли 40. Сколько точек открыли за год — в открытом виде не нашли. Для ИТ это значит: не «режим порезок из-за дыры», но и не история про быстрое расширение. Бюджет ИТ никто не публиковал. https://firmoteka.ru/7725844967</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Spell out INFOLine zero-growth as industry, not Karavay
The short 'factory market near zero' line read as this plant's 2026
outlook. Say it is the INFOLine food-producer average, not Каравай.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -6549,7 +6549,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="72" customHeight="1" s="6">
+    <row r="16" ht="86" customHeight="1" s="6">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Каравай (ОАО, Санкт-Петербург)</t>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>За 2026 продаж нет. Что есть — весь 2025: 11,12 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 709 миллионов — 6,4 копейки с рубля. Есть ещё ангарский «Каравай» — это другая компания, сюда не относится. Для ИТ это значит: 2025 был прибыльным. Своего плана на 2026 нет. По рынку заводов рост около нуля. https://firmoteka.ru/rating-by-revenue-10_71_1</t>
+          <t>За 2026 продаж нет. Что есть — весь 2025: 11,12 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 709 миллионов — 6,4 копейки с рубля. Есть ещё ангарский «Каравай» — это другая компания, сюда не относится. Для ИТ это значит: 2025 был прибыльным. Своего плана на 2026 нет. Фраза про «рост около нуля» — не про этот завод. Агентство INFOLine в сентябре 2026: у крупных производителей еды продажи в 2026 почти стоят (ни плюс, ни минус). Это весь рынок, не цифра «Каравая». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Say INFOLine 2026 factory slowdown is H1, not a full year
The 'near zero' line is Silenina's September 2026 reading of published
first-half figures for large plants, not a closed 2026 report.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных». Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей плюс 9–11%, производители еды около нуля, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
+          <t>Пустых «примерно» без источника. Если открытой цифры нет — «нет данных». Сети из регионов и большинство молочных заводов так и стоят: они отчитаются в 2027-м. Общий фон рынка (десять крупнейших сетей плюс 9–11%, у крупных заводов за полгода 2026 рост уже слабый, вся доставка продуктов 1,83 триллиона) в строку конкретной компании не ставили.</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2812,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="65" customHeight="1" s="6">
+    <row r="6" ht="73" customHeight="1" s="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>KDV Group</t>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>Прогноза на 2026 нет. Агентство INFOLine берёт KDV как пример торможения: уже 2025 только на 1% больше, а в 2026 у крупных производителей еды рост «около нуля». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+          <t>Прогноза на 2026 нет. Агентство INFOLine берёт KDV как пример торможения: уже 2025 только на 1% больше. В сентябре 2026 они смотрели полгода у крупных (Русагро плюс 9%, Черкизово плюс 3,5%) и сказали, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра KDV. https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -3970,7 +3970,7 @@
       </c>
       <c r="J28" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="J30" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="J32" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="J35" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4378,7 +4378,7 @@
       </c>
       <c r="J36" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J37" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J38" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="J39" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="J40" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="J41" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="J42" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="J43" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="J44" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4846,7 @@
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4898,7 +4898,7 @@
       </c>
       <c r="J46" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -4950,7 +4950,7 @@
       </c>
       <c r="J47" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5054,7 @@
       </c>
       <c r="J49" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="J50" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5158,7 @@
       </c>
       <c r="J51" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="J52" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5262,7 +5262,7 @@
       </c>
       <c r="J53" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5314,7 +5314,7 @@
       </c>
       <c r="J54" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="J55" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5418,7 +5418,7 @@
       </c>
       <c r="J56" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="J57" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="J58" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="J59" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="J60" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="J61" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5730,7 +5730,7 @@
       </c>
       <c r="J62" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="J64" s="13" t="inlineStr">
         <is>
-          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не эта компания. Отчёт за 2026 выйдет весной 2027.</t>
+          <t>Своего плана «в 2026 продадим на столько-то» не публиковали. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных заводов и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этой компании. Отчёт за 2026 выйдет весной 2027.</t>
         </is>
       </c>
     </row>
@@ -6499,7 +6499,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="82" customHeight="1" s="6">
+    <row r="15" ht="89" customHeight="1" s="6">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Иркутский масложиркомбинат</t>
@@ -6545,11 +6545,11 @@
       </c>
       <c r="J15" s="19" t="inlineStr">
         <is>
-          <t>За 2026 продаж нет. Что есть — весь 2025: 16,35 млрд рублей, почти как годом раньше (на 0,9% меньше). После расходов осталось 2,33 млрд. Это 14 копеек с рубля, но заметная часть — проценты по деньгам на счетах, не от продажи масла. Агентство INFOLine в сентябре 2026: у крупных производителей еды рост «около нуля» — это весь рынок, не этот завод. Для ИТ это значит: денег после 2025 много, своего плана строек на 2026 не нашли. Не похоже на режим порезок, но и анонса «тратим на программы» нет. https://finscanner.ru/company/3811185573/finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="86" customHeight="1" s="6">
+          <t>За 2026 продаж нет. Что есть — весь 2025: 16,35 млрд рублей, почти как годом раньше (на 0,9% меньше). После расходов осталось 2,33 млрд. Это 14 копеек с рубля, но заметная часть — проценты по деньгам на счетах, не от продажи масла. Агентство INFOLine в сентябре 2026 смотрело уже вышедшие полгода у крупных заводов (Русагро плюс 9%, Черкизово плюс 3,5%, ЭкоНива минус 2,4%) и сказало, что рост лидеров «приблизился к нулю». Это не отчёт за весь 2026 и не цифра этого завода. Для ИТ это значит: денег после 2025 много, своего плана строек на 2026 не нашли. Не похоже на режим порезок, но и анонса «тратим на программы» нет. https://finscanner.ru/company/3811185573/finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1" s="6">
       <c r="A16" s="18" t="inlineStr">
         <is>
           <t>Каравай (ОАО, Санкт-Петербург)</t>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>За 2026 продаж нет. Что есть — весь 2025: 11,12 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 709 миллионов — 6,4 копейки с рубля. Есть ещё ангарский «Каравай» — это другая компания, сюда не относится. Для ИТ это значит: 2025 был прибыльным. Своего плана на 2026 нет. Фраза про «рост около нуля» — не про этот завод. Агентство INFOLine в сентябре 2026: у крупных производителей еды продажи в 2026 почти стоят (ни плюс, ни минус). Это весь рынок, не цифра «Каравая». https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
+          <t>За 2026 продаж нет. Что есть — весь 2025: 11,12 млрд рублей, на 15% больше, чем годом раньше. После расходов осталось 709 миллионов — 6,4 копейки с рубля. Есть ещё ангарский «Каравай» — это другая компания, сюда не относится. Для ИТ это значит: 2025 был прибыльным. Своего плана на 2026 нет. Фраза про «рост около нуля» — не про этот завод и не отчёт за весь 2026. Агентство INFOLine в сентябре 2026 смотрело полгода у крупных: Русагро плюс 9%, Черкизово плюс 3,5%, ЭкоНива минус 2,4% — и отсюда сказало, что рост лидеров «приблизился к нулю». К «Караваю» это не цифра. https://www.retail.ru/news/infoline-vyruchka-krupneyshikh-proizvoditeley-produktov-pitaniya-padaet-16-sentyabrya-2026-282211/</t>
         </is>
       </c>
     </row>
@@ -7461,7 +7461,7 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже плюс 0,4%, в 2026 рост лидеров «приблизился к нулю». KDV как пример: уже 2025 только на 1% больше.</t>
+          <t>Светлана Силенина, сентябрь 2026: после запрета на ввоз еды в 2014 году крупные производители росли на 11–16% в год, в 2025 среднее уже плюс 0,4%. За весь 2026 отчёта нет — они смотрели первое полугодие: Русагро плюс 9% (годом раньше за весь год было плюс 16,6%), Черкизово плюс 3,5% (было плюс 11,4%), «Логика молока» плюс 3,5%, ЭкоНива минус 2,4%. Отсюда слова, что рост лидеров «приблизился к нулю». KDV как пример торможения ещё по 2025: только плюс 1%.</t>
         </is>
       </c>
       <c r="C21" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Add regional 2026 reading: cautious spend, kit not expansion
No mid-size chain published an aggressive store-opening plan for 2026.
Record that as the working IT lens, with warehouse/capex exceptions
and federals as a separate layer.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_vyruchka_2026.xlsx
+++ b/FMCG_RF_vyruchka_2026.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="6" min="1" max="1"/>
@@ -493,7 +493,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="64" customHeight="1" s="6">
+    <row r="9" ht="100" customHeight="1" s="6">
       <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Что в столбцах «прибыль» и «маржа»</t>
@@ -549,7 +549,19 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Это сети на 30–200 точек и заводы поменьше. Продаж за период 2026 у них почти нет — в столбцах денег стоит «нет данных», чтобы не подменять 2026 закрытым 2025-м. В комментарии два слоя: закрытый год (чтобы видеть прибыль) и что видно на 2026–27 (открывают, склеивают сети, режут расходы, закрывают магазин). Никто из них не публикует «бюджет ИТ в рублях». Читать так: растёт и строит склад / склеивает компании после сделки — ИТ скорее не режут; продажи уже падали, убыток, закрывают гипермаркет — скорее заморозка; прибыли мало и «год эффективности» — ИТ только если окупается на расходах.</t>
+          <t>Это сети на 30–200 точек и заводы поменьше. Продаж за период 2026 у них почти нет — в столбцах денег стоит «нет данных», чтобы не подменять 2026 закрытым 2025-м. В комментарии: закрытый год и что видно на 2026–27. Бюджет ИТ в рублях никто не публикует.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="100" customHeight="1" s="6">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Что видно по регионам на 2026</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Никто из этих сетей не заявил план активно открывать точки в 2026. По закрытому 2025 картина осторожная: кто-то чуть подрос в продажах, кто-то чуть в прибыли с рубля, кто-то почти ноль или минус по объёму («Низкоцен», «Иркутская аптека», гипермаркет «Дружбы»). Где тратят — чаще на оснащение уже работающих магазинов: электронные ценники, кассы самообслуживания, ремонт, склейка касс после сделки. Это не «режем ИТ под ноль», но и не гонка за новыми точками — с расходами аккуратничают. Исключения, где стройка всё же видна: склад «Семишагофф», корпус и склад «Любятово». Крупные федералы (X5, Лента) — другой слой: продажи за 2026 ещё растут, но новые магазины и у них открывают медленнее, чем год назад.</t>
         </is>
       </c>
     </row>
@@ -7339,7 +7351,7 @@
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>По большинству сетей из регионов и заводов своего плана «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год плюс 9–11%; крупные производители еды почти без роста), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку продаж это не ставили — это не продажи компании. Сети поменьше и то, режут ли они ИТ, — на листе «Регионы».</t>
+          <t>По большинству сетей из регионов и заводов своего плана «в 2026 продадим на столько-то» не было ни в конце 2025, ни в начале 2026. Что находилось: общий фон рынка (десять крупнейших сетей за год плюс 9–11%; у крупных заводов за полгода 2026 рост уже слабый), вся доставка продуктов в стране 1,83–1,84 триллиона (это не Ozon и не Лавка), и фразы вроде «новые заводы начнут себя окупать» у ЭФКО. В ячейку продаж это не ставили — это не продажи компании. Сети поменьше и то, режут ли они ИТ, — на листе «Регионы».</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
@@ -7360,7 +7372,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>У сетей на 30–200 точек своего отчёта за период 2026 почти нет. На листе «Регионы» те же десять колонок, что у крупных. В деньгах за 2026 чаще «нет данных». В комментарии — закрытый 2025 и что видно на 2026–27: открывают, склеивают сети, режут расходы или закрывают магазин. Это не «бюджет ИТ в рублях», такого никто не публикует.</t>
+          <t>У сетей на 30–200 точек плана «активно открываемся в 2026» в открытом виде нет. По 2025 кто-то чуть вырос в продажах или в прибыли с рубля, кто-то почти ноль или минус. Где тратят — чаще оснащение уже работающих точек (ценники, кассы, ремонт), не новая сетка магазинов. С расходами аккуратничают. Бюджет ИТ в рублях никто не публикует.</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">

</xml_diff>